<commit_message>
Incorpora pesquisa editorial ao Radar e sincroniza planilha
</commit_message>
<xml_diff>
--- a/Radar_Brasil_2027.xlsx
+++ b/Radar_Brasil_2027.xlsx
@@ -1351,7 +1351,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="NoticiasTable" displayName="NoticiasTable" ref="A1:I91" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="NoticiasTable" displayName="NoticiasTable" ref="A1:I92" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="A1:I58"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Data"/>
@@ -30066,11 +30066,11 @@
     </row>
     <row r="2" ht="150.75" customHeight="1" s="1">
       <c r="A2" s="31" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="B2" s="9" t="inlineStr">
         <is>
-          <t>A 9 meses da Copa do Mundo, TVs já apostam em programas de futebol feminino</t>
+          <t>Câmara aprova férias escolares facultativas durante Copa do Mundo Feminina de 2027 - O GLOBO</t>
         </is>
       </c>
       <c r="C2" s="9" t="inlineStr">
@@ -30085,12 +30085,12 @@
       </c>
       <c r="E2" s="9" t="inlineStr">
         <is>
-          <t>noticiasdatv.uol.com.br</t>
+          <t>oglobo.globo.com</t>
         </is>
       </c>
       <c r="F2" s="9" t="inlineStr">
         <is>
-          <t>https://noticiasdatv.uol.com.br/noticia/televisao/a-9-meses-da-copa-do-mundo-tvs-ja-apostam-em-programas-de-futebol-feminino-156477</t>
+          <t>https://oglobo.globo.com/brasil/noticia/2026/09/01/camara-aprova-ferias-escolares-facultativas-durante-copa-do-mundo-feminina-de-2027.ghtml</t>
         </is>
       </c>
       <c r="G2" s="9" t="inlineStr">
@@ -30103,20 +30103,24 @@
           <t>Médio</t>
         </is>
       </c>
-      <c r="I2" s="9" t="inlineStr"/>
+      <c r="I2" s="9" t="inlineStr">
+        <is>
+          <t>Câmara aprova férias escolares facultativas durante Copa do Mundo Feminina de 2027 Carregando... Acesse sua conta ou cadastre-se grátis sair Últimas Notícias Newsletter O GLOBO por dentro 101 Brasileiros -- Política Voltar Política Página Principal"&gt; Página Principal Sonar - A escuta das redes"&gt; Sonar - A escuta das redes Pulso"&gt; Pulso Rali"&gt; Rali Eleições 2026"&gt; Eleições 2026 Brasil Voltar Brasil Página Principal"&gt; Página Principal Educação"&gt; Educação Voltar Educação Educação &gt; Página Principal"&gt; Página Principal Educação &gt; Enem 2025"&gt; Enem 2025 Voltar Enem 2025 Educação &gt; Enem 2025 &gt; Página Principal"&gt; Página Principal Educação &gt; Prêmio Jovem Cientista"&gt; Prêmio Jovem Cientista Clima Extremo"&gt; Clima Extremo Meio Ambiente"&gt; Meio Ambiente Segurança Pública"&gt; Segurança Pública Direitos Humanos"&gt; Direitos Humanos São Paulo"&gt; São Paulo Minas Gerais"&gt; Minas Gerais Rio Voltar Rio Página Princi</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="114" customHeight="1" s="1">
       <c r="A3" s="31" t="n">
-        <v>46252</v>
+        <v>46277</v>
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>CNE orienta ajustes no calendário escolar durante a Copa Feminina 2027</t>
+          <t>A 9 meses da Copa do Mundo, TVs já apostam em programas de futebol feminino</t>
         </is>
       </c>
       <c r="C3" s="9" t="inlineStr">
         <is>
-          <t>Educação / calendário escolar / cidades-sede / operação da Copa 2027</t>
+          <t>Copa Feminina 2027</t>
         </is>
       </c>
       <c r="D3" s="9" t="inlineStr">
@@ -30126,12 +30130,12 @@
       </c>
       <c r="E3" s="9" t="inlineStr">
         <is>
-          <t>MEC / CNE</t>
+          <t>noticiasdatv.uol.com.br</t>
         </is>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/assuntos/noticias/2026/agosto/cne-orienta-redes-de-ensino-sobre-organizacao-do-calendario-escolar-durante-a-copa-do-mundo-feminina-de-2027</t>
+          <t>https://noticiasdatv.uol.com.br/noticia/televisao/a-9-meses-da-copa-do-mundo-tvs-ja-apostam-em-programas-de-futebol-feminino-156477</t>
         </is>
       </c>
       <c r="G3" s="9" t="inlineStr">
@@ -30141,42 +30145,38 @@
       </c>
       <c r="H3" s="9" t="inlineStr">
         <is>
-          <t>Alto</t>
-        </is>
-      </c>
-      <c r="I3" s="9" t="inlineStr">
-        <is>
-          <t>O Conselho Nacional de Educação aprovou o Parecer CNE/CEB nº 7/2026 orientando os sistemas de ensino sobre a organização dos calendários escolares de 2027 em razão da Copa do Mundo Feminina. Cidades-sede, regiões metropolitanas e áreas diretamente impactadas deverão promover os ajustes necessários conforme a realidade local e o calendário oficial da competição.</t>
-        </is>
-      </c>
+          <t>Médio</t>
+        </is>
+      </c>
+      <c r="I3" s="9" t="inlineStr"/>
     </row>
     <row r="4" ht="99.75" customHeight="1" s="1">
       <c r="A4" s="31" t="n">
-        <v>46276</v>
+        <v>46252</v>
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>Maracanã trocará gramado em 2027 antes da Copa do Mundo Feminina</t>
+          <t>CNE orienta ajustes no calendário escolar durante a Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
-          <t>Rio de Janeiro / Maracanã / gramado / infraestrutura / Copa Feminina 2027</t>
+          <t>Educação / calendário escolar / cidades-sede / operação da Copa 2027</t>
         </is>
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t>Rio de Janeiro/RJ</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
         <is>
-          <t>UOL</t>
+          <t>MEC / CNE</t>
         </is>
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
-          <t>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/09/11/maracana-aponta-fatores-para-campo-ruim-e-informa-que-trocara-tipo-de-grama.ghtm</t>
+          <t>https://www.gov.br/mec/pt-br/assuntos/noticias/2026/agosto/cne-orienta-redes-de-ensino-sobre-organizacao-do-calendario-escolar-durante-a-copa-do-mundo-feminina-de-2027</t>
         </is>
       </c>
       <c r="G4" s="9" t="inlineStr">
@@ -30191,27 +30191,27 @@
       </c>
       <c r="I4" s="9" t="inlineStr">
         <is>
-          <t>A administração do Maracanã informou que substituirá o gramado atual por Celebration Hybrid em 2027. A mudança ocorre em um ano de calendário intenso no estádio, que receberá partidas da Copa do Mundo Feminina, incluindo a abertura e a final do torneio, e busca melhorar a qualidade do campo após críticas recorrentes.</t>
+          <t>O Conselho Nacional de Educação aprovou o Parecer CNE/CEB nº 7/2026 orientando os sistemas de ensino sobre a organização dos calendários escolares de 2027 em razão da Copa do Mundo Feminina. Cidades-sede, regiões metropolitanas e áreas diretamente impactadas deverão promover os ajustes necessários conforme a realidade local e o calendário oficial da competição.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="128.25" customHeight="1" s="1">
       <c r="A5" s="31" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>Debate cobra legado duradouro da Copa Feminina 2027 para mulheres no esporte</t>
+          <t>Maracanã trocará gramado em 2027 antes da Copa do Mundo Feminina</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
         <is>
-          <t>Legado social / futebol feminino / políticas públicas / Copa Feminina 2027</t>
+          <t>Rio de Janeiro / Maracanã / gramado / infraestrutura / Copa Feminina 2027</t>
         </is>
       </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Rio de Janeiro/RJ</t>
         </is>
       </c>
       <c r="E5" s="9" t="inlineStr">
@@ -30221,7 +30221,7 @@
       </c>
       <c r="F5" s="9" t="inlineStr">
         <is>
-          <t>https://noticias.uol.com.br/colunas/joildo-santos/2026/09/10/a-copa-das-mulheres-vai-deixar-um-legado-ou-apenas-uma-fotografia.ghtm</t>
+          <t>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/09/11/maracana-aponta-fatores-para-campo-ruim-e-informa-que-trocara-tipo-de-grama.ghtm</t>
         </is>
       </c>
       <c r="G5" s="9" t="inlineStr">
@@ -30231,12 +30231,12 @@
       </c>
       <c r="H5" s="9" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I5" s="9" t="inlineStr">
         <is>
-          <t>Artigo publicado em 10/09/2026 discute se a Copa do Mundo Feminina de 2027 deixará legado estrutural para mulheres no esporte, defendendo investimentos permanentes em infraestrutura, formação, acesso à modalidade e políticas de proteção e equidade, para que o impacto do torneio ultrapasse a realização dos jogos.</t>
+          <t>A administração do Maracanã informou que substituirá o gramado atual por Celebration Hybrid em 2027. A mudança ocorre em um ano de calendário intenso no estádio, que receberá partidas da Copa do Mundo Feminina, incluindo a abertura e a final do torneio, e busca melhorar a qualidade do campo após críticas recorrentes.</t>
         </is>
       </c>
     </row>
@@ -30246,12 +30246,12 @@
       </c>
       <c r="B6" s="23" t="inlineStr">
         <is>
-          <t>CBF prevê pausa no futebol masculino durante a Copa Feminina 2027</t>
+          <t>Debate cobra legado duradouro da Copa Feminina 2027 para mulheres no esporte</t>
         </is>
       </c>
       <c r="C6" s="23" t="inlineStr">
         <is>
-          <t>Calendário CBF / operação dos estádios / Copa Feminina 2027</t>
+          <t>Legado social / futebol feminino / políticas públicas / Copa Feminina 2027</t>
         </is>
       </c>
       <c r="D6" s="23" t="inlineStr">
@@ -30266,7 +30266,7 @@
       </c>
       <c r="F6" s="23" t="inlineStr">
         <is>
-          <t>https://www.uol.com.br/esporte/futebol/colunas/rodrigo-mattos/2026/09/10/o-que-se-sabe-sobre-o-calendario-do-futebol-para-2027.ghtm</t>
+          <t>https://noticias.uol.com.br/colunas/joildo-santos/2026/09/10/a-copa-das-mulheres-vai-deixar-um-legado-ou-apenas-uma-fotografia.ghtm</t>
         </is>
       </c>
       <c r="G6" s="23" t="inlineStr">
@@ -30276,87 +30276,87 @@
       </c>
       <c r="H6" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I6" s="23" t="inlineStr">
         <is>
-          <t>A CBF prepara o calendário de 2027 prevendo paralisação do futebol masculino durante a Copa do Mundo Feminina e ajustes cerca de 15 dias antes do início do torneio para liberar os estádios cedidos à FIFA. A medida afeta diretamente a operação de arenas como Maracanã, Arena Itaquera, Beira-Rio, Mineirão e Arena Salvador durante o Mundial.</t>
+          <t>Artigo publicado em 10/09/2026 discute se a Copa do Mundo Feminina de 2027 deixará legado estrutural para mulheres no esporte, defendendo investimentos permanentes em infraestrutura, formação, acesso à modalidade e políticas de proteção e equidade, para que o impacto do torneio ultrapasse a realização dos jogos.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="32" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="B7" s="23" t="inlineStr">
         <is>
-          <t>Estádio Presidente Vargas recebe visita técnica da FIFA e avança nos preparativos para 2027</t>
+          <t>CBF prevê pausa no futebol masculino durante a Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C7" s="23" t="inlineStr">
         <is>
-          <t>Fortaleza / estádio de apoio / inspeção FIFA / operação da Copa 2027</t>
+          <t>Calendário CBF / operação dos estádios / Copa Feminina 2027</t>
         </is>
       </c>
       <c r="D7" s="23" t="inlineStr">
         <is>
-          <t>Fortaleza/CE</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E7" s="23" t="inlineStr">
         <is>
-          <t>Portal IN</t>
+          <t>UOL</t>
         </is>
       </c>
       <c r="F7" s="23" t="inlineStr">
         <is>
-          <t>https://www.portalin.com.br/in-loco/estadio-presidente-vargas-recebe-visita-tecnica-da-fifa-e-avanca-os-preparativos/</t>
+          <t>https://www.uol.com.br/esporte/futebol/colunas/rodrigo-mattos/2026/09/10/o-que-se-sabe-sobre-o-calendario-do-futebol-para-2027.ghtm</t>
         </is>
       </c>
       <c r="G7" s="23" t="inlineStr">
         <is>
-          <t>Positivo</t>
+          <t>Neutro</t>
         </is>
       </c>
       <c r="H7" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I7" s="23" t="inlineStr">
         <is>
-          <t>O Estádio Presidente Vargas, em Fortaleza, recebeu visita técnica da FIFA para avaliação de estrutura, logística e operação ligadas à Copa do Mundo Feminina 2027. O equipamento deve integrar a estrutura de apoio da cidade-sede, ao lado da Arena Castelão, atendendo delegações e operações do torneio.</t>
+          <t>A CBF prepara o calendário de 2027 prevendo paralisação do futebol masculino durante a Copa do Mundo Feminina e ajustes cerca de 15 dias antes do início do torneio para liberar os estádios cedidos à FIFA. A medida afeta diretamente a operação de arenas como Maracanã, Arena Itaquera, Beira-Rio, Mineirão e Arena Salvador durante o Mundial.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="32" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B8" s="23" t="inlineStr">
         <is>
-          <t>CBF vê Copa Feminina 2027 como teste para Mundial de Clubes de 2029 no Brasil</t>
+          <t>Estádio Presidente Vargas recebe visita técnica da FIFA e avança nos preparativos para 2027</t>
         </is>
       </c>
       <c r="C8" s="23" t="inlineStr">
         <is>
-          <t>CBF / estratégia internacional / Copa Feminina 2027 / Mundial de Clubes 2029</t>
+          <t>Fortaleza / estádio de apoio / inspeção FIFA / operação da Copa 2027</t>
         </is>
       </c>
       <c r="D8" s="23" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Fortaleza/CE</t>
         </is>
       </c>
       <c r="E8" s="23" t="inlineStr">
         <is>
-          <t>Lance!</t>
+          <t>Portal IN</t>
         </is>
       </c>
       <c r="F8" s="23" t="inlineStr">
         <is>
-          <t>https://www.lance.com.br/futebol-feminino/cbf-ve-copa-do-mundo-feminina-como-teste-para-mundial-de-clubes-de-2029-no-brasil.html</t>
+          <t>https://www.portalin.com.br/in-loco/estadio-presidente-vargas-recebe-visita-tecnica-da-fifa-e-avanca-os-preparativos/</t>
         </is>
       </c>
       <c r="G8" s="23" t="inlineStr">
@@ -30371,37 +30371,37 @@
       </c>
       <c r="I8" s="23" t="inlineStr">
         <is>
-          <t>A CBF trata a organização da Copa do Mundo Feminina de 2027 no Brasil como referência e teste para projetos internacionais futuros, incluindo a possibilidade de receber um Mundial de Clubes em 2029. A pauta destaca iniciativas em discussão e a construção de uma estratégia de longo prazo ligada à realização do torneio feminino no país.</t>
+          <t>O Estádio Presidente Vargas, em Fortaleza, recebeu visita técnica da FIFA para avaliação de estrutura, logística e operação ligadas à Copa do Mundo Feminina 2027. O equipamento deve integrar a estrutura de apoio da cidade-sede, ao lado da Arena Castelão, atendendo delegações e operações do torneio.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="32" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="B9" s="23" t="inlineStr">
         <is>
-          <t>FIFA faz visita técnica ao Estádio Presidente Vargas nos preparativos para a Copa Feminina 2027</t>
+          <t>CBF vê Copa Feminina 2027 como teste para Mundial de Clubes de 2029 no Brasil</t>
         </is>
       </c>
       <c r="C9" s="23" t="inlineStr">
         <is>
-          <t>Fortaleza / centro de treinamento / infraestrutura / preparação da Copa 2027</t>
+          <t>CBF / estratégia internacional / Copa Feminina 2027 / Mundial de Clubes 2029</t>
         </is>
       </c>
       <c r="D9" s="23" t="inlineStr">
         <is>
-          <t>Fortaleza/CE</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E9" s="23" t="inlineStr">
         <is>
-          <t>Prefeitura de Fortaleza</t>
+          <t>Lance!</t>
         </is>
       </c>
       <c r="F9" s="23" t="inlineStr">
         <is>
-          <t>https://fortaleza.ce.gov.br/noticias/nos-preparativos-para-a-copa-do-mundo-feminina-da-fifa-brasil-2027-estadio-presidente-vargas-recebe-visita-tecnica-da-entidade</t>
+          <t>https://www.lance.com.br/futebol-feminino/cbf-ve-copa-do-mundo-feminina-como-teste-para-mundial-de-clubes-de-2029-no-brasil.html</t>
         </is>
       </c>
       <c r="G9" s="23" t="inlineStr">
@@ -30416,67 +30416,67 @@
       </c>
       <c r="I9" s="23" t="inlineStr">
         <is>
-          <t>O Estádio Presidente Vargas, em Fortaleza, recebeu em 04/09/2026 uma visita técnica da FIFA. A equipe avaliou instalações e a organização de espaços que poderão atender delegações e imprensa durante a Copa do Mundo Feminina FIFA 2027, reforçando a preparação da cidade-sede.</t>
+          <t>A CBF trata a organização da Copa do Mundo Feminina de 2027 no Brasil como referência e teste para projetos internacionais futuros, incluindo a possibilidade de receber um Mundial de Clubes em 2029. A pauta destaca iniciativas em discussão e a construção de uma estratégia de longo prazo ligada à realização do torneio feminino no país.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="32" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B10" s="23" t="inlineStr">
         <is>
-          <t>CBF prepara calendário de 2027 com pausa e adaptação de estádios para a Copa Feminina</t>
+          <t>FIFA faz visita técnica ao Estádio Presidente Vargas nos preparativos para a Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C10" s="23" t="inlineStr">
         <is>
-          <t>Calendário CBF / clubes / estádios / operação da Copa 2027</t>
+          <t>Fortaleza / centro de treinamento / infraestrutura / preparação da Copa 2027</t>
         </is>
       </c>
       <c r="D10" s="23" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Fortaleza/CE</t>
         </is>
       </c>
       <c r="E10" s="23" t="inlineStr">
         <is>
-          <t>UOL</t>
+          <t>Prefeitura de Fortaleza</t>
         </is>
       </c>
       <c r="F10" s="23" t="inlineStr">
         <is>
-          <t>https://www.uol.com.br/esporte/futebol/colunas/rodrigo-mattos/2026/09/10/o-que-se-sabe-sobre-o-calendario-do-futebol-para-2027.htm</t>
+          <t>https://fortaleza.ce.gov.br/noticias/nos-preparativos-para-a-copa-do-mundo-feminina-da-fifa-brasil-2027-estadio-presidente-vargas-recebe-visita-tecnica-da-entidade</t>
         </is>
       </c>
       <c r="G10" s="23" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Positivo</t>
         </is>
       </c>
       <c r="H10" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I10" s="23" t="inlineStr">
         <is>
-          <t>A CBF prepara o calendário do futebol brasileiro de 2027 considerando a paralisação do futebol masculino durante a Copa do Mundo Feminina e ajustes cerca de 15 dias antes do torneio para evitar jogos nos estádios cedidos à FIFA. A medida afeta arenas como Maracanã, Neo Química Arena, Beira-Rio e Mineirão.</t>
+          <t>O Estádio Presidente Vargas, em Fortaleza, recebeu em 04/09/2026 uma visita técnica da FIFA. A equipe avaliou instalações e a organização de espaços que poderão atender delegações e imprensa durante a Copa do Mundo Feminina FIFA 2027, reforçando a preparação da cidade-sede.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="32" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="B11" s="23" t="inlineStr">
         <is>
-          <t>Governo negocia ingressos populares para a Copa do Mundo Feminina 2027</t>
+          <t>CBF prepara calendário de 2027 com pausa e adaptação de estádios para a Copa Feminina</t>
         </is>
       </c>
       <c r="C11" s="23" t="inlineStr">
         <is>
-          <t>Ingressos / acesso / organização da Copa 2027</t>
+          <t>Calendário CBF / clubes / estádios / operação da Copa 2027</t>
         </is>
       </c>
       <c r="D11" s="23" t="inlineStr">
@@ -30486,17 +30486,17 @@
       </c>
       <c r="E11" s="23" t="inlineStr">
         <is>
-          <t>ge</t>
+          <t>UOL</t>
         </is>
       </c>
       <c r="F11" s="23" t="inlineStr">
         <is>
-          <t>https://ge.globo.com/futebol/copa-do-mundo/noticia/2026/09/09/copa-feminina-governo-negocia-ingressos-populares-e-cre-em-torneio-blindado-da-crise-na-fifa.ghtml</t>
+          <t>https://www.uol.com.br/esporte/futebol/colunas/rodrigo-mattos/2026/09/10/o-que-se-sabe-sobre-o-calendario-do-futebol-para-2027.htm</t>
         </is>
       </c>
       <c r="G11" s="23" t="inlineStr">
         <is>
-          <t>Positivo</t>
+          <t>Neutro</t>
         </is>
       </c>
       <c r="H11" s="23" t="inlineStr">
@@ -30506,37 +30506,37 @@
       </c>
       <c r="I11" s="23" t="inlineStr">
         <is>
-          <t>O Governo Federal negocia com a FIFA uma cota de ingressos a preços populares para a Copa do Mundo Feminina de 2027 no Brasil. A pauta também envolve transporte, segurança, legado, calendário e medidas para ampliar o acesso do público aos estádios durante o torneio.</t>
+          <t>A CBF prepara o calendário do futebol brasileiro de 2027 considerando a paralisação do futebol masculino durante a Copa do Mundo Feminina e ajustes cerca de 15 dias antes do torneio para evitar jogos nos estádios cedidos à FIFA. A medida afeta arenas como Maracanã, Neo Química Arena, Beira-Rio e Mineirão.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="32" t="n">
-        <v>46267</v>
+        <v>46274</v>
       </c>
       <c r="B12" s="23" t="inlineStr">
         <is>
-          <t>Pernambuco sanciona lei estadual para operação da Copa Feminina 2027</t>
+          <t>Governo negocia ingressos populares para a Copa do Mundo Feminina 2027</t>
         </is>
       </c>
       <c r="C12" s="23" t="inlineStr">
         <is>
-          <t>Recife / legislação estadual / mobilidade / segurança / operação da Copa 2027</t>
+          <t>Ingressos / acesso / organização da Copa 2027</t>
         </is>
       </c>
       <c r="D12" s="23" t="inlineStr">
         <is>
-          <t>Recife/PE</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E12" s="23" t="inlineStr">
         <is>
-          <t>Alepe Legis</t>
+          <t>ge</t>
         </is>
       </c>
       <c r="F12" s="23" t="inlineStr">
         <is>
-          <t>https://legis.alepe.pe.gov.br/texto.aspx?id=89825&amp;tipo=</t>
+          <t>https://ge.globo.com/futebol/copa-do-mundo/noticia/2026/09/09/copa-feminina-governo-negocia-ingressos-populares-e-cre-em-torneio-blindado-da-crise-na-fifa.ghtml</t>
         </is>
       </c>
       <c r="G12" s="23" t="inlineStr">
@@ -30551,37 +30551,37 @@
       </c>
       <c r="I12" s="23" t="inlineStr">
         <is>
-          <t>Sancionada em 1º/09 e publicada no Diário Oficial em 2/09, a Lei nº 19.341/2026 estabelece as medidas estaduais para viabilizar a Copa Feminina 2027 em Pernambuco. A norma disciplina cooperação institucional, proteção comercial, controle de acesso, segurança, mobilidade, tramitação prioritária de licenças, hidratação do público e ações de turismo, futebol feminino e legado social.</t>
+          <t>O Governo Federal negocia com a FIFA uma cota de ingressos a preços populares para a Copa do Mundo Feminina de 2027 no Brasil. A pauta também envolve transporte, segurança, legado, calendário e medidas para ampliar o acesso do público aos estádios durante o torneio.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="32" t="n">
-        <v>46273</v>
+        <v>46267</v>
       </c>
       <c r="B13" s="23" t="inlineStr">
         <is>
-          <t>Lorena é indicada ao prêmio de melhor goleira da Bola de Ouro 2026</t>
+          <t>Pernambuco sanciona lei estadual para operação da Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C13" s="23" t="inlineStr">
         <is>
-          <t>Seleção Brasileira / Lorena / Bola de Ouro 2026 / ciclo da Copa Feminina 2027</t>
+          <t>Recife / legislação estadual / mobilidade / segurança / operação da Copa 2027</t>
         </is>
       </c>
       <c r="D13" s="23" t="inlineStr">
         <is>
-          <t>Internacional</t>
+          <t>Recife/PE</t>
         </is>
       </c>
       <c r="E13" s="23" t="inlineStr">
         <is>
-          <t>CNN Brasil</t>
+          <t>Alepe Legis</t>
         </is>
       </c>
       <c r="F13" s="23" t="inlineStr">
         <is>
-          <t>https://www.cnnbrasil.com.br/esportes/futebol/futebol-internacional/bola-de-ouro-lorena-e-indicada-a-melhor-goleira-do-futebol-feminino/</t>
+          <t>https://legis.alepe.pe.gov.br/texto.aspx?id=89825&amp;tipo=</t>
         </is>
       </c>
       <c r="G13" s="23" t="inlineStr">
@@ -30591,42 +30591,42 @@
       </c>
       <c r="H13" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I13" s="23" t="inlineStr">
         <is>
-          <t>Lorena, goleira titular da Seleção Brasileira principal e atleta do Kansas City, foi indicada em 08/09/2026 ao prêmio de melhor goleira do futebol feminino da Bola de Ouro 2026. O reconhecimento internacional integra o acompanhamento das principais atletas brasileiras no ciclo de preparação para a Copa do Mundo Feminina FIFA 2027 no Brasil.</t>
+          <t>Sancionada em 1º/09 e publicada no Diário Oficial em 2/09, a Lei nº 19.341/2026 estabelece as medidas estaduais para viabilizar a Copa Feminina 2027 em Pernambuco. A norma disciplina cooperação institucional, proteção comercial, controle de acesso, segurança, mobilidade, tramitação prioritária de licenças, hidratação do público e ações de turismo, futebol feminino e legado social.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="32" t="n">
-        <v>46254</v>
+        <v>46273</v>
       </c>
       <c r="B14" s="23" t="inlineStr">
         <is>
-          <t>São Paulo terá 10 jogos da Copa Feminina 2027 e prepara mobilidade, turismo e legado</t>
+          <t>Lorena é indicada ao prêmio de melhor goleira da Bola de Ouro 2026</t>
         </is>
       </c>
       <c r="C14" s="23" t="inlineStr">
         <is>
-          <t>São Paulo / calendário / Arena Itaquera / mobilidade / turismo / legado / Copa 2027</t>
+          <t>Seleção Brasileira / Lorena / Bola de Ouro 2026 / ciclo da Copa Feminina 2027</t>
         </is>
       </c>
       <c r="D14" s="23" t="inlineStr">
         <is>
-          <t>São Paulo/SP</t>
+          <t>Internacional</t>
         </is>
       </c>
       <c r="E14" s="23" t="inlineStr">
         <is>
-          <t>Prefeitura de São Paulo</t>
+          <t>CNN Brasil</t>
         </is>
       </c>
       <c r="F14" s="23" t="inlineStr">
         <is>
-          <t>https://www2.prefeitura.sp.gov.br/web/prefeitura-de-sao-paulo/w/cidade-com-mais-jogos-s%C3%A3o-paulo-receber%C3%A1-10-partidas-da-copa-do-mundo-feminina-2027</t>
+          <t>https://www.cnnbrasil.com.br/esportes/futebol/futebol-internacional/bola-de-ouro-lorena-e-indicada-a-melhor-goleira-do-futebol-feminino/</t>
         </is>
       </c>
       <c r="G14" s="23" t="inlineStr">
@@ -30636,42 +30636,42 @@
       </c>
       <c r="H14" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I14" s="23" t="inlineStr">
         <is>
-          <t>A Prefeitura de São Paulo detalhou em 20/08/2026 o calendário da cidade para a Copa do Mundo Feminina 2027. A capital receberá 10 das 64 partidas, o maior número entre as oito sedes, incluindo seis jogos de fase de grupos, a partida da Seleção Brasileira em 29/06/2027, uma oitava de final, uma quarta de final, uma semifinal e a disputa do terceiro lugar na Arena Itaquera. O município informa que mantém planejamento com a FIFA em mobilidade urbana, segurança, turismo, empreendedorismo e legado esportivo, além de ampliar atividades gratuitas de futebol feminino nos centros esportivos municipais.</t>
+          <t>Lorena, goleira titular da Seleção Brasileira principal e atleta do Kansas City, foi indicada em 08/09/2026 ao prêmio de melhor goleira do futebol feminino da Bola de Ouro 2026. O reconhecimento internacional integra o acompanhamento das principais atletas brasileiras no ciclo de preparação para a Copa do Mundo Feminina FIFA 2027 no Brasil.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="32" t="n">
-        <v>46268</v>
+        <v>46254</v>
       </c>
       <c r="B15" s="23" t="inlineStr">
         <is>
-          <t>Porto Alegre articula participação de pioneiras do Gre-Nal na programação da Copa Feminina 2027</t>
+          <t>São Paulo terá 10 jogos da Copa Feminina 2027 e prepara mobilidade, turismo e legado</t>
         </is>
       </c>
       <c r="C15" s="23" t="inlineStr">
         <is>
-          <t>Porto Alegre / legado / memória do futebol feminino / programação paralela / Copa 2027</t>
+          <t>São Paulo / calendário / Arena Itaquera / mobilidade / turismo / legado / Copa 2027</t>
         </is>
       </c>
       <c r="D15" s="23" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>São Paulo/SP</t>
         </is>
       </c>
       <c r="E15" s="23" t="inlineStr">
         <is>
-          <t>Prefeitura de Porto Alegre / Secopa 2027</t>
+          <t>Prefeitura de São Paulo</t>
         </is>
       </c>
       <c r="F15" s="23" t="inlineStr">
         <is>
-          <t>https://prefeitura.poa.br/secopa2027/noticias/pioneiras-da-dupla-gre-nal-se-reunem-com-secopa-para-alinhar-acoes-para-copa-do</t>
+          <t>https://www2.prefeitura.sp.gov.br/web/prefeitura-de-sao-paulo/w/cidade-com-mais-jogos-s%C3%A3o-paulo-receber%C3%A1-10-partidas-da-copa-do-mundo-feminina-2027</t>
         </is>
       </c>
       <c r="G15" s="23" t="inlineStr">
@@ -30681,42 +30681,42 @@
       </c>
       <c r="H15" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I15" s="23" t="inlineStr">
         <is>
-          <t>A Secretaria Extraordinária da Copa do Mundo Feminina 2027 de Porto Alegre recebeu, em 03/09/2026, cinco pioneiras do futebol feminino de Grêmio e Internacional para discutir sua integração à programação do Mundial na cidade. Entre as propostas apresentadas estão reconhecimento oficial às atletas, homenagem no Beira-Rio, participação em seminários e eventos paralelos e acesso a partidas. A Secopa informou que avaliará, com as áreas municipais e parceiros do torneio, a viabilidade de incorporar as ações à programação oficial, conectando memória, legado e engajamento local em uma das cidades-sede.</t>
+          <t>A Prefeitura de São Paulo detalhou em 20/08/2026 o calendário da cidade para a Copa do Mundo Feminina 2027. A capital receberá 10 das 64 partidas, o maior número entre as oito sedes, incluindo seis jogos de fase de grupos, a partida da Seleção Brasileira em 29/06/2027, uma oitava de final, uma quarta de final, uma semifinal e a disputa do terceiro lugar na Arena Itaquera. O município informa que mantém planejamento com a FIFA em mobilidade urbana, segurança, turismo, empreendedorismo e legado esportivo, além de ampliar atividades gratuitas de futebol feminino nos centros esportivos municipais.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="32" t="n">
-        <v>46267</v>
+        <v>46268</v>
       </c>
       <c r="B16" s="23" t="inlineStr">
         <is>
-          <t>Fortaleza avança em miniterminais no entorno do Castelão para mobilidade da Copa 2027</t>
+          <t>Porto Alegre articula participação de pioneiras do Gre-Nal na programação da Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C16" s="23" t="inlineStr">
         <is>
-          <t>Fortaleza / mobilidade / infraestrutura / Arena Castelão / Copa 2027</t>
+          <t>Porto Alegre / legado / memória do futebol feminino / programação paralela / Copa 2027</t>
         </is>
       </c>
       <c r="D16" s="23" t="inlineStr">
         <is>
-          <t>Fortaleza/CE</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="E16" s="23" t="inlineStr">
         <is>
-          <t>Prefeitura de Fortaleza</t>
+          <t>Prefeitura de Porto Alegre / Secopa 2027</t>
         </is>
       </c>
       <c r="F16" s="23" t="inlineStr">
         <is>
-          <t>https://fortaleza.ce.gov.br/noticias/prefeito-evandro-leitao-visita-obras-dos-miniterminais-da-arena-castelao</t>
+          <t>https://prefeitura.poa.br/secopa2027/noticias/pioneiras-da-dupla-gre-nal-se-reunem-com-secopa-para-alinhar-acoes-para-copa-do</t>
         </is>
       </c>
       <c r="G16" s="23" t="inlineStr">
@@ -30726,42 +30726,42 @@
       </c>
       <c r="H16" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I16" s="23" t="inlineStr">
         <is>
-          <t>A Prefeitura de Fortaleza informou em 02/09/2026 que dois miniterminais de transporte coletivo estão em construção no entorno da Arena Castelão, com investimento aproximado de R$ 2,5 milhões, 30% de execução e conclusão prevista para dezembro de 2026. Os equipamentos terão capacidade para atender até mil pessoas simultaneamente e contarão com painéis de previsão de ônibus, bilhetagem eletrônica, acessibilidade, videomonitoramento e integração com linhas especiais em dias de jogos. O prefeito Evandro Leitão vinculou diretamente a obra à preparação para grandes eventos e para a Copa do Mundo Feminina de 2027, reforçando sua relevância para a mobilidade e a experiência de torcedores na cidade-sede.</t>
+          <t>A Secretaria Extraordinária da Copa do Mundo Feminina 2027 de Porto Alegre recebeu, em 03/09/2026, cinco pioneiras do futebol feminino de Grêmio e Internacional para discutir sua integração à programação do Mundial na cidade. Entre as propostas apresentadas estão reconhecimento oficial às atletas, homenagem no Beira-Rio, participação em seminários e eventos paralelos e acesso a partidas. A Secopa informou que avaliará, com as áreas municipais e parceiros do torneio, a viabilidade de incorporar as ações à programação oficial, conectando memória, legado e engajamento local em uma das cidades-sede.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="32" t="n">
-        <v>46268</v>
+        <v>46267</v>
       </c>
       <c r="B17" s="23" t="inlineStr">
         <is>
-          <t>Turn On The Light inicia agenda de conexões sociais rumo à Copa Feminina 2027</t>
+          <t>Fortaleza avança em miniterminais no entorno do Castelão para mobilidade da Copa 2027</t>
         </is>
       </c>
       <c r="C17" s="23" t="inlineStr">
         <is>
-          <t>Ativação / futebol feminino / maternidade / impacto social / Copa 2027</t>
+          <t>Fortaleza / mobilidade / infraestrutura / Arena Castelão / Copa 2027</t>
         </is>
       </c>
       <c r="D17" s="23" t="inlineStr">
         <is>
-          <t>São Paulo/SP</t>
+          <t>Fortaleza/CE</t>
         </is>
       </c>
       <c r="E17" s="23" t="inlineStr">
         <is>
-          <t>BRA1 / Agência VIVA</t>
+          <t>Prefeitura de Fortaleza</t>
         </is>
       </c>
       <c r="F17" s="23" t="inlineStr">
         <is>
-          <t>https://www.bra1.com.br/geral/id-688491/turn_on_the_light_inaugura_agenda_de_conexoes_entre_futebol_feminino__maternidade_e_causas_sociais_rumo_a_copa_do_mundo_de_2027</t>
+          <t>https://fortaleza.ce.gov.br/noticias/prefeito-evandro-leitao-visita-obras-dos-miniterminais-da-arena-castelao</t>
         </is>
       </c>
       <c r="G17" s="23" t="inlineStr">
@@ -30771,42 +30771,42 @@
       </c>
       <c r="H17" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I17" s="23" t="inlineStr">
         <is>
-          <t>A agência Turn On The Light iniciou uma agenda de encontros e narrativas que conectará futebol feminino, maternidade, carreira e causas sociais até a Copa do Mundo Feminina de 2027. A primeira ação ocorreu na Casa Mãe Paulistana, em São Paulo, com participação da jogadora Tamires, da ex-jogadora Milene Domingues, do comunicador Marco Aurélio e da cantora Gabi Fernandes. A iniciativa pretende usar a preparação para o Mundial como plataforma contínua de engajamento e protagonismo feminino fora dos estádios.</t>
+          <t>A Prefeitura de Fortaleza informou em 02/09/2026 que dois miniterminais de transporte coletivo estão em construção no entorno da Arena Castelão, com investimento aproximado de R$ 2,5 milhões, 30% de execução e conclusão prevista para dezembro de 2026. Os equipamentos terão capacidade para atender até mil pessoas simultaneamente e contarão com painéis de previsão de ônibus, bilhetagem eletrônica, acessibilidade, videomonitoramento e integração com linhas especiais em dias de jogos. O prefeito Evandro Leitão vinculou diretamente a obra à preparação para grandes eventos e para a Copa do Mundo Feminina de 2027, reforçando sua relevância para a mobilidade e a experiência de torcedores na cidade-sede.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="32" t="n">
-        <v>46266</v>
+        <v>46268</v>
       </c>
       <c r="B18" s="23" t="inlineStr">
         <is>
-          <t>Bahia prepara Sala Lilás e ações de proteção e legado feminino para a Copa 2027</t>
+          <t>Turn On The Light inicia agenda de conexões sociais rumo à Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C18" s="23" t="inlineStr">
         <is>
-          <t>Salvador / segurança das mulheres / turismo / legado / futebol feminino / Copa 2027</t>
+          <t>Ativação / futebol feminino / maternidade / impacto social / Copa 2027</t>
         </is>
       </c>
       <c r="D18" s="23" t="inlineStr">
         <is>
-          <t>Salvador/BA</t>
+          <t>São Paulo/SP</t>
         </is>
       </c>
       <c r="E18" s="23" t="inlineStr">
         <is>
-          <t>Bahia Notícias</t>
+          <t>BRA1 / Agência VIVA</t>
         </is>
       </c>
       <c r="F18" s="23" t="inlineStr">
         <is>
-          <t>https://www.bahianoticias.com.br/amp/esportes/noticia/80073-bahia-prepara-sala-lilas-acoes-de-seguranca-e-rdollar-2-mi-para-o-futebol-feminino-na-copa-de-2027-confira-novidades</t>
+          <t>https://www.bra1.com.br/geral/id-688491/turn_on_the_light_inaugura_agenda_de_conexoes_entre_futebol_feminino__maternidade_e_causas_sociais_rumo_a_copa_do_mundo_de_2027</t>
         </is>
       </c>
       <c r="G18" s="23" t="inlineStr">
@@ -30816,42 +30816,42 @@
       </c>
       <c r="H18" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I18" s="23" t="inlineStr">
         <is>
-          <t>A Secretaria de Políticas para as Mulheres da Bahia detalhou medidas de preparação para a Copa do Mundo Feminina 2027 em Salvador, incluindo a implantação de uma Sala Lilás na Arena Fonte Nova para acolhimento de mulheres, certificação da rede turística pelo selo Mulheres Seguras, capacitações e ações de autonomia econômica. O planejamento também inclui edital de R$ 2 milhões com a Sudesb para incentivar torneios femininos no interior e formação voltada à arbitragem feminina, conectando segurança, turismo e legado esportivo do Mundial.</t>
+          <t>A agência Turn On The Light iniciou uma agenda de encontros e narrativas que conectará futebol feminino, maternidade, carreira e causas sociais até a Copa do Mundo Feminina de 2027. A primeira ação ocorreu na Casa Mãe Paulistana, em São Paulo, com participação da jogadora Tamires, da ex-jogadora Milene Domingues, do comunicador Marco Aurélio e da cantora Gabi Fernandes. A iniciativa pretende usar a preparação para o Mundial como plataforma contínua de engajamento e protagonismo feminino fora dos estádios.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="32" t="n">
-        <v>46269</v>
+        <v>46266</v>
       </c>
       <c r="B19" s="23" t="inlineStr">
         <is>
-          <t>Piracicaba reconstrói futebol feminino com foco em ampliar estrutura antes da Copa 2027</t>
+          <t>Bahia prepara Sala Lilás e ações de proteção e legado feminino para a Copa 2027</t>
         </is>
       </c>
       <c r="C19" s="23" t="inlineStr">
         <is>
-          <t>Legado / desenvolvimento local / futebol feminino / formação / Copa 2027</t>
+          <t>Salvador / segurança das mulheres / turismo / legado / futebol feminino / Copa 2027</t>
         </is>
       </c>
       <c r="D19" s="23" t="inlineStr">
         <is>
-          <t>Piracicaba/SP</t>
+          <t>Salvador/BA</t>
         </is>
       </c>
       <c r="E19" s="23" t="inlineStr">
         <is>
-          <t>Jornal de Piracicaba / Sampi</t>
+          <t>Bahia Notícias</t>
         </is>
       </c>
       <c r="F19" s="23" t="inlineStr">
         <is>
-          <t>https://sampi.net.br/campinas/noticias/3002816/cidade/2026/09/piracicaba-busca-reconstruir-futebol-feminino-as-vesperas-da-copa</t>
+          <t>https://www.bahianoticias.com.br/amp/esportes/noticia/80073-bahia-prepara-sala-lilas-acoes-de-seguranca-e-rdollar-2-mi-para-o-futebol-feminino-na-copa-de-2027-confira-novidades</t>
         </is>
       </c>
       <c r="G19" s="23" t="inlineStr">
@@ -30861,42 +30861,42 @@
       </c>
       <c r="H19" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I19" s="23" t="inlineStr">
         <is>
-          <t>Piracicaba mantém em 2026 um projeto municipal de reconstrução do futebol feminino em parceria com o Caldeirão Futebol Clube, com cerca de 50 atletas a partir de 15 anos, treinamentos gratuitos e investimento de R$ 108 mil. A equipe adulta foi vice-campeã dos Jogos Regionais e garantiu vaga nos Jogos Abertos do Interior, enquanto o planejamento prevê ampliar a estrutura e buscar o retorno às competições estaduais de maior nível em 2027. Gestores locais relacionam a realização da Copa do Mundo Feminina no Brasil à expectativa de maior procura e fortalecimento da modalidade na cidade.</t>
+          <t>A Secretaria de Políticas para as Mulheres da Bahia detalhou medidas de preparação para a Copa do Mundo Feminina 2027 em Salvador, incluindo a implantação de uma Sala Lilás na Arena Fonte Nova para acolhimento de mulheres, certificação da rede turística pelo selo Mulheres Seguras, capacitações e ações de autonomia econômica. O planejamento também inclui edital de R$ 2 milhões com a Sudesb para incentivar torneios femininos no interior e formação voltada à arbitragem feminina, conectando segurança, turismo e legado esportivo do Mundial.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="32" t="n">
-        <v>46251</v>
+        <v>46269</v>
       </c>
       <c r="B20" s="23" t="inlineStr">
         <is>
-          <t>Distrito Federal cria grupo de trabalho da Justiça e Cidadania para ações da Copa Feminina 2027</t>
+          <t>Piracicaba reconstrói futebol feminino com foco em ampliar estrutura antes da Copa 2027</t>
         </is>
       </c>
       <c r="C20" s="23" t="inlineStr">
         <is>
-          <t>Brasília / governança / direitos / operação da cidade-sede / Copa 2027</t>
+          <t>Legado / desenvolvimento local / futebol feminino / formação / Copa 2027</t>
         </is>
       </c>
       <c r="D20" s="23" t="inlineStr">
         <is>
-          <t>Brasília/DF</t>
+          <t>Piracicaba/SP</t>
         </is>
       </c>
       <c r="E20" s="23" t="inlineStr">
         <is>
-          <t>Diário Oficial do Distrito Federal</t>
+          <t>Jornal de Piracicaba / Sampi</t>
         </is>
       </c>
       <c r="F20" s="23" t="inlineStr">
         <is>
-          <t>https://www.sinj.df.gov.br/sinj/TextoArquivoDiario.aspx?id_file=afb86271-9977-31e0-ae59-86b99234ddbb</t>
+          <t>https://sampi.net.br/campinas/noticias/3002816/cidade/2026/09/piracicaba-busca-reconstruir-futebol-feminino-as-vesperas-da-copa</t>
         </is>
       </c>
       <c r="G20" s="23" t="inlineStr">
@@ -30911,42 +30911,42 @@
       </c>
       <c r="I20" s="23" t="inlineStr">
         <is>
-          <t>A Secretaria de Estado de Justiça e Cidadania do Distrito Federal instituiu grupo de trabalho para planejar, coordenar, articular, executar, acompanhar e avaliar ações relacionadas à Copa do Mundo Feminina da FIFA Brasil 2027. O grupo deverá elaborar planejamento operacional, articular unidades e instituições, acompanhar cronogramas e resultados e manter integração permanente com a Comissão de Monitoramento e Governança da Copa, reforçando a preparação institucional de Brasília como cidade-sede.</t>
+          <t>Piracicaba mantém em 2026 um projeto municipal de reconstrução do futebol feminino em parceria com o Caldeirão Futebol Clube, com cerca de 50 atletas a partir de 15 anos, treinamentos gratuitos e investimento de R$ 108 mil. A equipe adulta foi vice-campeã dos Jogos Regionais e garantiu vaga nos Jogos Abertos do Interior, enquanto o planejamento prevê ampliar a estrutura e buscar o retorno às competições estaduais de maior nível em 2027. Gestores locais relacionam a realização da Copa do Mundo Feminina no Brasil à expectativa de maior procura e fortalecimento da modalidade na cidade.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="32" t="n">
-        <v>46267</v>
+        <v>46251</v>
       </c>
       <c r="B21" s="23" t="inlineStr">
         <is>
-          <t>Congresso torna facultativo ajuste das férias escolares durante a Copa Feminina 2027</t>
+          <t>Distrito Federal cria grupo de trabalho da Justiça e Cidadania para ações da Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C21" s="23" t="inlineStr">
         <is>
-          <t>Legislação / calendário escolar / impacto social / Copa 2027</t>
+          <t>Brasília / governança / direitos / operação da cidade-sede / Copa 2027</t>
         </is>
       </c>
       <c r="D21" s="23" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Brasília/DF</t>
         </is>
       </c>
       <c r="E21" s="23" t="inlineStr">
         <is>
-          <t>Agência Senado / Câmara dos Deputados</t>
+          <t>Diário Oficial do Distrito Federal</t>
         </is>
       </c>
       <c r="F21" s="23" t="inlineStr">
         <is>
-          <t>https://www12.senado.leg.br/noticias/senado-agora/2026/09/02/copa-feminina-de-futebol</t>
+          <t>https://www.sinj.df.gov.br/sinj/TextoArquivoDiario.aspx?id_file=afb86271-9977-31e0-ae59-86b99234ddbb</t>
         </is>
       </c>
       <c r="G21" s="23" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Positivo</t>
         </is>
       </c>
       <c r="H21" s="23" t="inlineStr">
@@ -30956,87 +30956,87 @@
       </c>
       <c r="I21" s="23" t="inlineStr">
         <is>
-          <t>O Senado aprovou em 02/09/2026 o PL 3.481/2026, que torna facultativo o ajuste dos calendários escolares para coincidir com a Copa do Mundo Feminina de 2027. A Câmara havia aprovado o texto em 31/08/2026. A proposta altera a regra da Lei Geral da Copa que previa ajuste obrigatório e segue para sanção presidencial. A mudança afeta a organização social e educacional durante o torneio e pode influenciar a participação de famílias, estudantes e comunidades nas ações ligadas ao Mundial.</t>
+          <t>A Secretaria de Estado de Justiça e Cidadania do Distrito Federal instituiu grupo de trabalho para planejar, coordenar, articular, executar, acompanhar e avaliar ações relacionadas à Copa do Mundo Feminina da FIFA Brasil 2027. O grupo deverá elaborar planejamento operacional, articular unidades e instituições, acompanhar cronogramas e resultados e manter integração permanente com a Comissão de Monitoramento e Governança da Copa, reforçando a preparação institucional de Brasília como cidade-sede.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="32" t="n">
-        <v>46268</v>
+        <v>46267</v>
       </c>
       <c r="B22" s="23" t="inlineStr">
         <is>
-          <t>Maracanã prepara reforma de R$ 2,5 milhões para adequações da Copa Feminina 2027</t>
+          <t>Congresso torna facultativo ajuste das férias escolares durante a Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C22" s="23" t="inlineStr">
         <is>
-          <t>Infraestrutura / estádio-sede / acessibilidade / hospitalidade / Copa 2027</t>
+          <t>Legislação / calendário escolar / impacto social / Copa 2027</t>
         </is>
       </c>
       <c r="D22" s="23" t="inlineStr">
         <is>
-          <t>Rio de Janeiro/RJ</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E22" s="23" t="inlineStr">
         <is>
-          <t>ge</t>
+          <t>Agência Senado / Câmara dos Deputados</t>
         </is>
       </c>
       <c r="F22" s="23" t="inlineStr">
         <is>
-          <t>https://ge.globo.com/futebol/copa-do-mundo-feminina/noticia/2026/09/03/governo-e-consorcio-fla-flu-preparam-reforma-de-r-25-milhoes-em-tribuna-do-maracana-para-a-copa-de-2027.ghtml</t>
+          <t>https://www12.senado.leg.br/noticias/senado-agora/2026/09/02/copa-feminina-de-futebol</t>
         </is>
       </c>
       <c r="G22" s="23" t="inlineStr">
         <is>
-          <t>Positivo</t>
+          <t>Neutro</t>
         </is>
       </c>
       <c r="H22" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I22" s="23" t="inlineStr">
         <is>
-          <t>O Governo do Estado do Rio de Janeiro e o Consórcio Fla-Flu preparam uma reforma estimada em R$ 2,5 milhões na Tribuna de Honra do Maracanã, como parte das adequações para a Copa do Mundo Feminina de 2027. O aditivo contratual prevê melhorias em acessibilidade, hospitalidade, segurança, conforto e funcionalidade, com prazo de execução estimado em 45 dias para a proposta escolhida. O estádio receberá nove partidas do Mundial, incluindo abertura e final.</t>
+          <t>O Senado aprovou em 02/09/2026 o PL 3.481/2026, que torna facultativo o ajuste dos calendários escolares para coincidir com a Copa do Mundo Feminina de 2027. A Câmara havia aprovado o texto em 31/08/2026. A proposta altera a regra da Lei Geral da Copa que previa ajuste obrigatório e segue para sanção presidencial. A mudança afeta a organização social e educacional durante o torneio e pode influenciar a participação de famílias, estudantes e comunidades nas ações ligadas ao Mundial.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="32" t="n">
-        <v>46265</v>
+        <v>46268</v>
       </c>
       <c r="B23" s="23" t="inlineStr">
         <is>
-          <t>Porto Alegre protocola regras especiais para a Copa Feminina 2027</t>
+          <t>Maracanã prepara reforma de R$ 2,5 milhões para adequações da Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C23" s="23" t="inlineStr">
         <is>
-          <t>Cidade-sede / legislação municipal / mobilidade / ingressos / operação da Copa 2027</t>
+          <t>Infraestrutura / estádio-sede / acessibilidade / hospitalidade / Copa 2027</t>
         </is>
       </c>
       <c r="D23" s="23" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Rio de Janeiro/RJ</t>
         </is>
       </c>
       <c r="E23" s="23" t="inlineStr">
         <is>
-          <t>Prefeitura de Porto Alegre</t>
+          <t>ge</t>
         </is>
       </c>
       <c r="F23" s="23" t="inlineStr">
         <is>
-          <t>https://prefeitura.poa.br/secopa2027/noticias/prefeitura-protocola-projeto-de-lei-com-regras-especiais-para-copa-feminina</t>
+          <t>https://ge.globo.com/futebol/copa-do-mundo-feminina/noticia/2026/09/03/governo-e-consorcio-fla-flu-preparam-reforma-de-r-25-milhoes-em-tribuna-do-maracana-para-a-copa-de-2027.ghtml</t>
         </is>
       </c>
       <c r="G23" s="23" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Positivo</t>
         </is>
       </c>
       <c r="H23" s="23" t="inlineStr">
@@ -31046,52 +31046,52 @@
       </c>
       <c r="I23" s="23" t="inlineStr">
         <is>
-          <t>A Prefeitura de Porto Alegre protocolou o Projeto de Lei nº 028/26 com regras específicas para a realização da Copa do Mundo Feminina FIFA 2027 e seus eventos oficiais. A proposta prevê perímetro temporário de proteção comercial de 1 km no entorno do Beira-Rio, regras exclusivas de ingressos, prioridade de licenciamento, gratuidade no transporte municipal para voluntários e credenciados e coordenação pública da segurança em áreas oficiais. O texto ainda depende de análise e votação pela Câmara Municipal.</t>
+          <t>O Governo do Estado do Rio de Janeiro e o Consórcio Fla-Flu preparam uma reforma estimada em R$ 2,5 milhões na Tribuna de Honra do Maracanã, como parte das adequações para a Copa do Mundo Feminina de 2027. O aditivo contratual prevê melhorias em acessibilidade, hospitalidade, segurança, conforto e funcionalidade, com prazo de execução estimado em 45 dias para a proposta escolhida. O estádio receberá nove partidas do Mundial, incluindo abertura e final.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="32" t="n">
-        <v>46269</v>
+        <v>46265</v>
       </c>
       <c r="B24" s="23" t="inlineStr">
         <is>
-          <t>Painel em Salvador conecta proteção no esporte e legado da Copa Feminina 2027</t>
+          <t>Porto Alegre protocola regras especiais para a Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C24" s="23" t="inlineStr">
         <is>
-          <t>Salvador / safeguarding / legado / formação profissional / Copa 2027</t>
+          <t>Cidade-sede / legislação municipal / mobilidade / ingressos / operação da Copa 2027</t>
         </is>
       </c>
       <c r="D24" s="23" t="inlineStr">
         <is>
-          <t>Salvador/BA</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="E24" s="23" t="inlineStr">
         <is>
-          <t>Jornal Grande Bahia / GovBA</t>
+          <t>Prefeitura de Porto Alegre</t>
         </is>
       </c>
       <c r="F24" s="23" t="inlineStr">
         <is>
-          <t>https://jornalgrandebahia.com.br/2026/09/futebol-feminino-e-copa-do-mundo-2027-painel-em-salvador-debate-seguranca-e-abre-inscricoes-para-voluntarios/</t>
+          <t>https://prefeitura.poa.br/secopa2027/noticias/prefeitura-protocola-projeto-de-lei-com-regras-especiais-para-copa-feminina</t>
         </is>
       </c>
       <c r="G24" s="23" t="inlineStr">
         <is>
-          <t>Positivo</t>
+          <t>Neutro</t>
         </is>
       </c>
       <c r="H24" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I24" s="23" t="inlineStr">
         <is>
-          <t>Painel Futebol &amp; Cidadania, realizado em 03/09/2026 no Colégio Estadual Professor Rômulo Almeida, em Salvador, reuniu Setre, IPIE, UFBA e comunidade escolar para discutir proteção e prevenção de abusos no esporte, formação profissional e legado ligado à Copa Feminina 2027. O encontro também anunciou mapeamento de projetos de futebol feminino em escolas de tempo integral e apresentou propostas de Centro de Referência do Futebol Feminino e plano estadual de formação para árbitras, treinadoras e gestoras.</t>
+          <t>A Prefeitura de Porto Alegre protocolou o Projeto de Lei nº 028/26 com regras específicas para a realização da Copa do Mundo Feminina FIFA 2027 e seus eventos oficiais. A proposta prevê perímetro temporário de proteção comercial de 1 km no entorno do Beira-Rio, regras exclusivas de ingressos, prioridade de licenciamento, gratuidade no transporte municipal para voluntários e credenciados e coordenação pública da segurança em áreas oficiais. O texto ainda depende de análise e votação pela Câmara Municipal.</t>
         </is>
       </c>
     </row>
@@ -31101,27 +31101,27 @@
       </c>
       <c r="B25" s="23" t="inlineStr">
         <is>
-          <t>Formiga destaca potencial da Copa Feminina 2027 para transformar oportunidades de meninas e jogadoras</t>
+          <t>Painel em Salvador conecta proteção no esporte e legado da Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C25" s="23" t="inlineStr">
         <is>
-          <t>Legado / futebol feminino / inspiração / Copa 2027</t>
+          <t>Salvador / safeguarding / legado / formação profissional / Copa 2027</t>
         </is>
       </c>
       <c r="D25" s="23" t="inlineStr">
         <is>
-          <t>São Paulo/SP</t>
+          <t>Salvador/BA</t>
         </is>
       </c>
       <c r="E25" s="23" t="inlineStr">
         <is>
-          <t>AFP/BOL</t>
+          <t>Jornal Grande Bahia / GovBA</t>
         </is>
       </c>
       <c r="F25" s="23" t="inlineStr">
         <is>
-          <t>https://www.bol.uol.com.br/noticias/2026/09/04/copa-do-mundo-feminina-no-brasil-pode-mudar-vidas-de-muitas-jogadoras-diz-formiga.htm</t>
+          <t>https://jornalgrandebahia.com.br/2026/09/futebol-feminino-e-copa-do-mundo-2027-painel-em-salvador-debate-seguranca-e-abre-inscricoes-para-voluntarios/</t>
         </is>
       </c>
       <c r="G25" s="23" t="inlineStr">
@@ -31136,37 +31136,37 @@
       </c>
       <c r="I25" s="23" t="inlineStr">
         <is>
-          <t>Em entrevista à AFP publicada em 04/09/2026, durante o evento Esporte Cria em São Paulo, Formiga afirmou que a Copa do Mundo Feminina de 2027 no Brasil pode mudar a realidade de inúmeras meninas e jogadoras na região. A fala da ex-capitã da Seleção reforça o potencial de legado social e esportivo do torneio e conecta a realização do Mundial à ampliação de oportunidades e visibilidade para o futebol feminino.</t>
+          <t>Painel Futebol &amp; Cidadania, realizado em 03/09/2026 no Colégio Estadual Professor Rômulo Almeida, em Salvador, reuniu Setre, IPIE, UFBA e comunidade escolar para discutir proteção e prevenção de abusos no esporte, formação profissional e legado ligado à Copa Feminina 2027. O encontro também anunciou mapeamento de projetos de futebol feminino em escolas de tempo integral e apresentou propostas de Centro de Referência do Futebol Feminino e plano estadual de formação para árbitras, treinadoras e gestoras.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="32" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="B26" s="23" t="inlineStr">
         <is>
-          <t>Futebol feminino bate recordes de transferências internacionais em 2026</t>
+          <t>Formiga destaca potencial da Copa Feminina 2027 para transformar oportunidades de meninas e jogadoras</t>
         </is>
       </c>
       <c r="C26" s="23" t="inlineStr">
         <is>
-          <t>Mercado / crescimento / futebol feminino</t>
+          <t>Legado / futebol feminino / inspiração / Copa 2027</t>
         </is>
       </c>
       <c r="D26" s="23" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>São Paulo/SP</t>
         </is>
       </c>
       <c r="E26" s="23" t="inlineStr">
         <is>
-          <t>FIFA</t>
+          <t>AFP/BOL</t>
         </is>
       </c>
       <c r="F26" s="23" t="inlineStr">
         <is>
-          <t>https://inside.fifa.com/media-releases/world-cup-2026-impact-mid-year-transfer-window</t>
+          <t>https://www.bol.uol.com.br/noticias/2026/09/04/copa-do-mundo-feminina-no-brasil-pode-mudar-vidas-de-muitas-jogadoras-diz-formiga.htm</t>
         </is>
       </c>
       <c r="G26" s="23" t="inlineStr">
@@ -31176,12 +31176,12 @@
       </c>
       <c r="H26" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I26" s="23" t="inlineStr">
         <is>
-          <t>A FIFA registrou 1.406 transferências internacionais no futebol profissional feminino entre 1º de junho e 2 de setembro de 2026, alta de 19,2% sobre o recorde anterior. Os clubes movimentaram US$ 28,6 milhões em taxas, mais que o dobro da janela equivalente de 2025, confirmando expansão histórica do mercado da modalidade.</t>
+          <t>Em entrevista à AFP publicada em 04/09/2026, durante o evento Esporte Cria em São Paulo, Formiga afirmou que a Copa do Mundo Feminina de 2027 no Brasil pode mudar a realidade de inúmeras meninas e jogadoras na região. A fala da ex-capitã da Seleção reforça o potencial de legado social e esportivo do torneio e conecta a realização do Mundial à ampliação de oportunidades e visibilidade para o futebol feminino.</t>
         </is>
       </c>
     </row>
@@ -31191,27 +31191,27 @@
       </c>
       <c r="B27" s="23" t="inlineStr">
         <is>
-          <t>Bahia planeja usar a Copa Feminina 2027 para ampliar turismo além de Salvador</t>
+          <t>Futebol feminino bate recordes de transferências internacionais em 2026</t>
         </is>
       </c>
       <c r="C27" s="23" t="inlineStr">
         <is>
-          <t>Turismo / cidade-sede / legado econômico / infraestrutura aeroportuária</t>
+          <t>Mercado / crescimento / futebol feminino</t>
         </is>
       </c>
       <c r="D27" s="23" t="inlineStr">
         <is>
-          <t>Salvador/BA</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="E27" s="23" t="inlineStr">
         <is>
-          <t>Let's Go Bahia</t>
+          <t>FIFA</t>
         </is>
       </c>
       <c r="F27" s="23" t="inlineStr">
         <is>
-          <t>https://letsgobahia.com.br/index.php/noticia/radar-por-matheus-pastori/exclusivo-com-mais-de-r-400-milhoes-investidos-bahia-planeja-aproveitar-copa-do-mundo-feminina-para-impulsionar-o-turismo-no-interior</t>
+          <t>https://inside.fifa.com/media-releases/world-cup-2026-impact-mid-year-transfer-window</t>
         </is>
       </c>
       <c r="G27" s="23" t="inlineStr">
@@ -31221,12 +31221,12 @@
       </c>
       <c r="H27" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I27" s="23" t="inlineStr">
         <is>
-          <t>Em entrevista publicada em 03/09/2026, o secretário de Turismo da Bahia, Maurício Bacelar, detalhou a estratégia de aproveitar o fluxo gerado pelos sete jogos da Copa Feminina 2027 na Fonte Nova para prolongar a permanência dos visitantes e estimular roteiros no interior. O estado relaciona a preparação a mais de R$ 400 milhões em intervenções aeroportuárias, reforçando o legado turístico e econômico do torneio para além de Salvador.</t>
+          <t>A FIFA registrou 1.406 transferências internacionais no futebol profissional feminino entre 1º de junho e 2 de setembro de 2026, alta de 19,2% sobre o recorde anterior. Os clubes movimentaram US$ 28,6 milhões em taxas, mais que o dobro da janela equivalente de 2025, confirmando expansão histórica do mercado da modalidade.</t>
         </is>
       </c>
     </row>
@@ -31236,27 +31236,27 @@
       </c>
       <c r="B28" s="23" t="inlineStr">
         <is>
-          <t>Fortaleza supera 7,3 mil interessados locais no voluntariado da Copa Feminina 2027</t>
+          <t>Bahia planeja usar a Copa Feminina 2027 para ampliar turismo além de Salvador</t>
         </is>
       </c>
       <c r="C28" s="23" t="inlineStr">
         <is>
-          <t>Voluntariado / engajamento local / cidade-sede</t>
+          <t>Turismo / cidade-sede / legado econômico / infraestrutura aeroportuária</t>
         </is>
       </c>
       <c r="D28" s="23" t="inlineStr">
         <is>
-          <t>Fortaleza/CE</t>
+          <t>Salvador/BA</t>
         </is>
       </c>
       <c r="E28" s="23" t="inlineStr">
         <is>
-          <t>Prefeitura de Fortaleza</t>
+          <t>Let's Go Bahia</t>
         </is>
       </c>
       <c r="F28" s="23" t="inlineStr">
         <is>
-          <t>https://www.fortaleza.ce.gov.br/noticias/fortaleza-mobiliza-voluntarios-para-a-copa-do-mundo-feminina-da-fifa-brasil-2027-e-celebra-abertura-oficial-das-inscricoes</t>
+          <t>https://letsgobahia.com.br/index.php/noticia/radar-por-matheus-pastori/exclusivo-com-mais-de-r-400-milhoes-investidos-bahia-planeja-aproveitar-copa-do-mundo-feminina-para-impulsionar-o-turismo-no-interior</t>
         </is>
       </c>
       <c r="G28" s="23" t="inlineStr">
@@ -31271,7 +31271,7 @@
       </c>
       <c r="I28" s="23" t="inlineStr">
         <is>
-          <t>A Prefeitura de Fortaleza informou em 03/09/2026 que mais de 7,3 mil pessoas já haviam indicado a capital cearense como cidade-sede de preferência durante a fase de registro de interesse do Programa de Voluntários da Copa do Mundo Feminina 2027. O dado local, divulgado junto à abertura das inscrições oficiais, evidencia forte mobilização e engajamento da população da cidade-sede antes do torneio.</t>
+          <t>Em entrevista publicada em 03/09/2026, o secretário de Turismo da Bahia, Maurício Bacelar, detalhou a estratégia de aproveitar o fluxo gerado pelos sete jogos da Copa Feminina 2027 na Fonte Nova para prolongar a permanência dos visitantes e estimular roteiros no interior. O estado relaciona a preparação a mais de R$ 400 milhões em intervenções aeroportuárias, reforçando o legado turístico e econômico do torneio para além de Salvador.</t>
         </is>
       </c>
     </row>
@@ -31281,27 +31281,27 @@
       </c>
       <c r="B29" s="23" t="inlineStr">
         <is>
-          <t>FIFA abre inscrições oficiais para mais de 6 mil voluntários da Copa Feminina 2027</t>
+          <t>Fortaleza supera 7,3 mil interessados locais no voluntariado da Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C29" s="23" t="inlineStr">
         <is>
-          <t>Voluntariado / engajamento / operação do torneio</t>
+          <t>Voluntariado / engajamento local / cidade-sede</t>
         </is>
       </c>
       <c r="D29" s="23" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Fortaleza/CE</t>
         </is>
       </c>
       <c r="E29" s="23" t="inlineStr">
         <is>
-          <t>FIFA</t>
+          <t>Prefeitura de Fortaleza</t>
         </is>
       </c>
       <c r="F29" s="23" t="inlineStr">
         <is>
-          <t>https://inside.fifa.com/tournament-organisation/volunteers/media-releases/volunteer-applications-open-womens-world-cup-brazil-2027</t>
+          <t>https://www.fortaleza.ce.gov.br/noticias/fortaleza-mobiliza-voluntarios-para-a-copa-do-mundo-feminina-da-fifa-brasil-2027-e-celebra-abertura-oficial-das-inscricoes</t>
         </is>
       </c>
       <c r="G29" s="23" t="inlineStr">
@@ -31311,27 +31311,27 @@
       </c>
       <c r="H29" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I29" s="23" t="inlineStr">
         <is>
-          <t>A FIFA abriu oficialmente em 03/09/2026 as inscrições para o programa de voluntariado da Copa do Mundo Feminina de 2027 no Brasil. Mais de 6 mil voluntários serão recrutados nas oito cidades-sede, após mais de 100 mil manifestações de interesse registradas desde julho. A abertura efetiva das candidaturas é um novo marco operacional e de engajamento, distinto da divulgação anterior das funções disponíveis aos voluntários.</t>
+          <t>A Prefeitura de Fortaleza informou em 03/09/2026 que mais de 7,3 mil pessoas já haviam indicado a capital cearense como cidade-sede de preferência durante a fase de registro de interesse do Programa de Voluntários da Copa do Mundo Feminina 2027. O dado local, divulgado junto à abertura das inscrições oficiais, evidencia forte mobilização e engajamento da população da cidade-sede antes do torneio.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="32" t="n">
-        <v>46267</v>
+        <v>46268</v>
       </c>
       <c r="B30" s="23" t="inlineStr">
         <is>
-          <t>Senado aprova prioridade ao futebol feminino e prevê plano de legado da Copa 2027</t>
+          <t>FIFA abre inscrições oficiais para mais de 6 mil voluntários da Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C30" s="23" t="inlineStr">
         <is>
-          <t>Legislação federal / futebol feminino / legado da Copa 2027</t>
+          <t>Voluntariado / engajamento / operação do torneio</t>
         </is>
       </c>
       <c r="D30" s="23" t="inlineStr">
@@ -31341,12 +31341,12 @@
       </c>
       <c r="E30" s="23" t="inlineStr">
         <is>
-          <t>Agência Senado</t>
+          <t>FIFA</t>
         </is>
       </c>
       <c r="F30" s="23" t="inlineStr">
         <is>
-          <t>https://www12.senado.leg.br/noticias/materias/2026/09/02/senado-aprova-prioridade-para-futebol-feminino-na-politica-de-esporte</t>
+          <t>https://inside.fifa.com/tournament-organisation/volunteers/media-releases/volunteer-applications-open-womens-world-cup-brazil-2027</t>
         </is>
       </c>
       <c r="G30" s="23" t="inlineStr">
@@ -31361,7 +31361,7 @@
       </c>
       <c r="I30" s="23" t="inlineStr">
         <is>
-          <t>O Senado aprovou projeto que torna o futebol feminino prioridade na política pública esportiva nacional e determina a elaboração de um plano de legado social, esportivo e financeiro da Copa do Mundo Feminina FIFA 2027 no Brasil. O texto também prevê ações para profissionalização, igualdade salarial, participação de mulheres na gestão e arbitragem e combate à discriminação e à violência no esporte.</t>
+          <t>A FIFA abriu oficialmente em 03/09/2026 as inscrições para o programa de voluntariado da Copa do Mundo Feminina de 2027 no Brasil. Mais de 6 mil voluntários serão recrutados nas oito cidades-sede, após mais de 100 mil manifestações de interesse registradas desde julho. A abertura efetiva das candidaturas é um novo marco operacional e de engajamento, distinto da divulgação anterior das funções disponíveis aos voluntários.</t>
         </is>
       </c>
     </row>
@@ -31371,12 +31371,12 @@
       </c>
       <c r="B31" s="23" t="inlineStr">
         <is>
-          <t>SporTV estreia Aquecimento Delas com bancada feminina dedicada ao futebol feminino</t>
+          <t>Senado aprova prioridade ao futebol feminino e prevê plano de legado da Copa 2027</t>
         </is>
       </c>
       <c r="C31" s="23" t="inlineStr">
         <is>
-          <t>Mídia / futebol feminino / cobertura esportiva</t>
+          <t>Legislação federal / futebol feminino / legado da Copa 2027</t>
         </is>
       </c>
       <c r="D31" s="23" t="inlineStr">
@@ -31386,12 +31386,12 @@
       </c>
       <c r="E31" s="23" t="inlineStr">
         <is>
-          <t>O Globo</t>
+          <t>Agência Senado</t>
         </is>
       </c>
       <c r="F31" s="23" t="inlineStr">
         <is>
-          <t>https://oglobo.globo.com/play/noticia/2026/09/02/nota-10-a-estreia-do-aquecimento-delas-no-sportv.ghtml</t>
+          <t>https://www12.senado.leg.br/noticias/materias/2026/09/02/senado-aprova-prioridade-para-futebol-feminino-na-politica-de-esporte</t>
         </is>
       </c>
       <c r="G31" s="23" t="inlineStr">
@@ -31401,12 +31401,12 @@
       </c>
       <c r="H31" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I31" s="23" t="inlineStr">
         <is>
-          <t>O SporTV lançou o programa Aquecimento Delas, dedicado ao futebol feminino e apresentado por uma bancada formada por Ana Thais Matos, Renata Mendonça, Mariana Spinelli e Luana Maluf. A iniciativa amplia o espaço permanente de análise e cobertura da modalidade na televisão esportiva em um período de crescente atenção ao futebol feminino antes da Copa do Mundo de 2027 no Brasil.</t>
+          <t>O Senado aprovou projeto que torna o futebol feminino prioridade na política pública esportiva nacional e determina a elaboração de um plano de legado social, esportivo e financeiro da Copa do Mundo Feminina FIFA 2027 no Brasil. O texto também prevê ações para profissionalização, igualdade salarial, participação de mulheres na gestão e arbitragem e combate à discriminação e à violência no esporte.</t>
         </is>
       </c>
     </row>
@@ -31416,12 +31416,12 @@
       </c>
       <c r="B32" s="23" t="inlineStr">
         <is>
-          <t>FIFA detalha mais de 30 funções de voluntariado para a Copa do Mundo Feminina 2027</t>
+          <t>SporTV estreia Aquecimento Delas com bancada feminina dedicada ao futebol feminino</t>
         </is>
       </c>
       <c r="C32" s="23" t="inlineStr">
         <is>
-          <t>Voluntariado / operação do torneio / engajamento</t>
+          <t>Mídia / futebol feminino / cobertura esportiva</t>
         </is>
       </c>
       <c r="D32" s="23" t="inlineStr">
@@ -31431,12 +31431,12 @@
       </c>
       <c r="E32" s="23" t="inlineStr">
         <is>
-          <t>FIFA</t>
+          <t>O Globo</t>
         </is>
       </c>
       <c r="F32" s="23" t="inlineStr">
         <is>
-          <t>https://www.fifa.com/pt/tournaments/womens/womensworldcup/brazil-2027/articles/funcoes-voluntarios-copa-do-mundo-feminina-brasil-2027</t>
+          <t>https://oglobo.globo.com/play/noticia/2026/09/02/nota-10-a-estreia-do-aquecimento-delas-no-sportv.ghtml</t>
         </is>
       </c>
       <c r="G32" s="23" t="inlineStr">
@@ -31446,27 +31446,27 @@
       </c>
       <c r="H32" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I32" s="23" t="inlineStr">
         <is>
-          <t>A FIFA detalhou mais de 30 funções previstas para voluntários da Copa do Mundo Feminina de 2027, com atuação em locais oficiais como estádios, hotéis, centros de treinamento e aeroportos. As áreas incluem gestão de acessos, hospedagem, credenciamento, competição, entretenimento, transportes, serviços ao espectador, tecnologia, mídia, hospitalidade, segurança, sustentabilidade, ingressos e operações de estádio.</t>
+          <t>O SporTV lançou o programa Aquecimento Delas, dedicado ao futebol feminino e apresentado por uma bancada formada por Ana Thais Matos, Renata Mendonça, Mariana Spinelli e Luana Maluf. A iniciativa amplia o espaço permanente de análise e cobertura da modalidade na televisão esportiva em um período de crescente atenção ao futebol feminino antes da Copa do Mundo de 2027 no Brasil.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="32" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="B33" s="23" t="inlineStr">
         <is>
-          <t>Câmara torna facultativo o ajuste das férias escolares durante a Copa Feminina 2027</t>
+          <t>FIFA detalha mais de 30 funções de voluntariado para a Copa do Mundo Feminina 2027</t>
         </is>
       </c>
       <c r="C33" s="23" t="inlineStr">
         <is>
-          <t>Legislação federal / educação / calendário escolar / Copa Feminina 2027</t>
+          <t>Voluntariado / operação do torneio / engajamento</t>
         </is>
       </c>
       <c r="D33" s="23" t="inlineStr">
@@ -31476,17 +31476,17 @@
       </c>
       <c r="E33" s="23" t="inlineStr">
         <is>
-          <t>Agência Câmara</t>
+          <t>FIFA</t>
         </is>
       </c>
       <c r="F33" s="23" t="inlineStr">
         <is>
-          <t>https://www.camara.leg.br/noticias/1301485-camara-aprova-autonomia-de-escolas-para-ajustar-calendario-na-copa-do-mundo-feminina</t>
+          <t>https://www.fifa.com/pt/tournaments/womens/womensworldcup/brazil-2027/articles/funcoes-voluntarios-copa-do-mundo-feminina-brasil-2027</t>
         </is>
       </c>
       <c r="G33" s="23" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Positivo</t>
         </is>
       </c>
       <c r="H33" s="23" t="inlineStr">
@@ -31496,52 +31496,52 @@
       </c>
       <c r="I33" s="23" t="inlineStr">
         <is>
-          <t>A Câmara dos Deputados aprovou o PL 3.481/2026, que torna facultativo aos sistemas de ensino ajustar as férias escolares ao período da Copa do Mundo Feminina 2027. O texto preserva a autonomia das redes, exige o cumprimento da carga horária e dos 200 dias letivos previstos na LDB e foi remetido ao Senado em 1º de setembro de 2026.</t>
+          <t>A FIFA detalhou mais de 30 funções previstas para voluntários da Copa do Mundo Feminina de 2027, com atuação em locais oficiais como estádios, hotéis, centros de treinamento e aeroportos. As áreas incluem gestão de acessos, hospedagem, credenciamento, competição, entretenimento, transportes, serviços ao espectador, tecnologia, mídia, hospitalidade, segurança, sustentabilidade, ingressos e operações de estádio.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="32" t="n">
-        <v>46264</v>
+        <v>46265</v>
       </c>
       <c r="B34" s="23" t="inlineStr">
         <is>
-          <t>Seleção Feminina Sub-20 chega a Bielsko-Biała para a reta final antes do Mundial</t>
+          <t>Câmara torna facultativo o ajuste das férias escolares durante a Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C34" s="23" t="inlineStr">
         <is>
-          <t>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</t>
+          <t>Legislação federal / educação / calendário escolar / Copa Feminina 2027</t>
         </is>
       </c>
       <c r="D34" s="23" t="inlineStr">
         <is>
-          <t>Bielsko-Biała/POL</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E34" s="23" t="inlineStr">
         <is>
-          <t>CBF</t>
+          <t>Agência Câmara</t>
         </is>
       </c>
       <c r="F34" s="23" t="inlineStr">
         <is>
-          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-base-feminina/selecao-feminina-sub-20/selecao-feminina-sub-20-chega-a-bielsko-biala-para-reta-final-antes-da-estreia-no-mundial</t>
+          <t>https://www.camara.leg.br/noticias/1301485-camara-aprova-autonomia-de-escolas-para-ajustar-calendario-na-copa-do-mundo-feminina</t>
         </is>
       </c>
       <c r="G34" s="23" t="inlineStr">
         <is>
-          <t>Positivo</t>
+          <t>Neutro</t>
         </is>
       </c>
       <c r="H34" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I34" s="23" t="inlineStr">
         <is>
-          <t>A Seleção Brasileira Feminina Sub-20 chegou a Bielsko-Biała, na Polônia, para concluir a preparação antes da estreia na Copa do Mundo da categoria. A delegação entra na etapa final de adaptação e treinamentos para o torneio, que começa em 5 de setembro.</t>
+          <t>A Câmara dos Deputados aprovou o PL 3.481/2026, que torna facultativo aos sistemas de ensino ajustar as férias escolares ao período da Copa do Mundo Feminina 2027. O texto preserva a autonomia das redes, exige o cumprimento da carga horária e dos 200 dias letivos previstos na LDB e foi remetido ao Senado em 1º de setembro de 2026.</t>
         </is>
       </c>
     </row>
@@ -31551,17 +31551,17 @@
       </c>
       <c r="B35" s="23" t="inlineStr">
         <is>
-          <t>Thaís Lima destaca integração entre base e Seleção principal antes do Mundial Sub-20</t>
+          <t>Seleção Feminina Sub-20 chega a Bielsko-Biała para a reta final antes do Mundial</t>
         </is>
       </c>
       <c r="C35" s="23" t="inlineStr">
         <is>
-          <t>Seleções de Base / Sub-20 Feminina / integração com a Seleção principal</t>
+          <t>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</t>
         </is>
       </c>
       <c r="D35" s="23" t="inlineStr">
         <is>
-          <t>Polônia</t>
+          <t>Bielsko-Biała/POL</t>
         </is>
       </c>
       <c r="E35" s="23" t="inlineStr">
@@ -31571,7 +31571,7 @@
       </c>
       <c r="F35" s="23" t="inlineStr">
         <is>
-          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/thais-lima-comenta-integracao-entre-as-selecoes-de-base-e-a-principal</t>
+          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-base-feminina/selecao-feminina-sub-20/selecao-feminina-sub-20-chega-a-bielsko-biala-para-reta-final-antes-da-estreia-no-mundial</t>
         </is>
       </c>
       <c r="G35" s="23" t="inlineStr">
@@ -31586,22 +31586,22 @@
       </c>
       <c r="I35" s="23" t="inlineStr">
         <is>
-          <t>Às vésperas da Copa do Mundo Feminina Sub-20, a atacante Thaís Lima destacou a integração entre as Seleções de base e a equipe principal. A jogadora, que acumula convocações em diferentes categorias, exemplifica a continuidade do processo de formação da CBF durante a preparação do Brasil na Polônia.</t>
+          <t>A Seleção Brasileira Feminina Sub-20 chegou a Bielsko-Biała, na Polônia, para concluir a preparação antes da estreia na Copa do Mundo da categoria. A delegação entra na etapa final de adaptação e treinamentos para o torneio, que começa em 5 de setembro.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="32" t="n">
-        <v>46263</v>
+        <v>46264</v>
       </c>
       <c r="B36" s="23" t="inlineStr">
         <is>
-          <t>Bianca destaca entrosamento da Seleção Sub-20 antes do Mundial</t>
+          <t>Thaís Lima destaca integração entre base e Seleção principal antes do Mundial Sub-20</t>
         </is>
       </c>
       <c r="C36" s="23" t="inlineStr">
         <is>
-          <t>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</t>
+          <t>Seleções de Base / Sub-20 Feminina / integração com a Seleção principal</t>
         </is>
       </c>
       <c r="D36" s="23" t="inlineStr">
@@ -31616,7 +31616,7 @@
       </c>
       <c r="F36" s="23" t="inlineStr">
         <is>
-          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/bianca-relembra-conquista-do-sul-americano-e-valoriza-entrosamento-na-selecao-sub-20</t>
+          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/thais-lima-comenta-integracao-entre-as-selecoes-de-base-e-a-principal</t>
         </is>
       </c>
       <c r="G36" s="23" t="inlineStr">
@@ -31631,37 +31631,37 @@
       </c>
       <c r="I36" s="23" t="inlineStr">
         <is>
-          <t>A zagueira Bianca relembrou a conquista do Sul-Americano Sub-20 e destacou o entrosamento da Seleção Brasileira durante a preparação na Polônia para a Copa do Mundo Feminina Sub-20 de 2026. A fala reforça a confiança do grupo antes da estreia no Mundial.</t>
+          <t>Às vésperas da Copa do Mundo Feminina Sub-20, a atacante Thaís Lima destacou a integração entre as Seleções de base e a equipe principal. A jogadora, que acumula convocações em diferentes categorias, exemplifica a continuidade do processo de formação da CBF durante a preparação do Brasil na Polônia.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="32" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="B37" s="23" t="inlineStr">
         <is>
-          <t>Fortaleza avança na Lei da Copa e prepara inspeção da FIFA no Castelão</t>
+          <t>Bianca destaca entrosamento da Seleção Sub-20 antes do Mundial</t>
         </is>
       </c>
       <c r="C37" s="23" t="inlineStr">
         <is>
-          <t>Preparação de cidade-sede / legislação estadual / mobilidade / Arena Castelão</t>
+          <t>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</t>
         </is>
       </c>
       <c r="D37" s="23" t="inlineStr">
         <is>
-          <t>Fortaleza/CE</t>
+          <t>Polônia</t>
         </is>
       </c>
       <c r="E37" s="23" t="inlineStr">
         <is>
-          <t>Diário do Nordeste</t>
+          <t>CBF</t>
         </is>
       </c>
       <c r="F37" s="23" t="inlineStr">
         <is>
-          <t>https://diariodonordeste.verdesmares.com.br/jogada/fortaleza-avanca-na-lei-da-copa-e-prepara-castelao-para-inspecao-da-fifa-a-300-dias-do-mundial-1.3787756</t>
+          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/bianca-relembra-conquista-do-sul-americano-e-valoriza-entrosamento-na-selecao-sub-20</t>
         </is>
       </c>
       <c r="G37" s="23" t="inlineStr">
@@ -31671,12 +31671,12 @@
       </c>
       <c r="H37" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I37" s="23" t="inlineStr">
         <is>
-          <t>A 300 dias da Copa do Mundo Feminina 2027, Fortaleza informou que prepara a promulgação da Lei Estadual da Copa, conclui o plano de mobilidade e discute gratuidade no transporte público em dias de jogos. A Arena Castelão, que receberá nove partidas, terá nova inspeção técnica da FIFA em setembro, enquanto Estado, município e federação avançam em infraestrutura, responsabilidade social e legado.</t>
+          <t>A zagueira Bianca relembrou a conquista do Sul-Americano Sub-20 e destacou o entrosamento da Seleção Brasileira durante a preparação na Polônia para a Copa do Mundo Feminina Sub-20 de 2026. A fala reforça a confiança do grupo antes da estreia no Mundial.</t>
         </is>
       </c>
     </row>
@@ -31686,27 +31686,27 @@
       </c>
       <c r="B38" s="23" t="inlineStr">
         <is>
-          <t>Dulce transforma experiência no Mundial Sub-17 em preparação para a Seleção Sub-20</t>
+          <t>Fortaleza avança na Lei da Copa e prepara inspeção da FIFA no Castelão</t>
         </is>
       </c>
       <c r="C38" s="23" t="inlineStr">
         <is>
-          <t>Seleções de Base / Sub-20 Feminina / transição de categoria</t>
+          <t>Preparação de cidade-sede / legislação estadual / mobilidade / Arena Castelão</t>
         </is>
       </c>
       <c r="D38" s="23" t="inlineStr">
         <is>
-          <t>Cracóvia/POL</t>
+          <t>Fortaleza/CE</t>
         </is>
       </c>
       <c r="E38" s="23" t="inlineStr">
         <is>
-          <t>CBF</t>
+          <t>Diário do Nordeste</t>
         </is>
       </c>
       <c r="F38" s="23" t="inlineStr">
         <is>
-          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/de-um-mundial-ao-outro-dulce-vive-novo-desafio-com-a-selecao-brasileira</t>
+          <t>https://diariodonordeste.verdesmares.com.br/jogada/fortaleza-avanca-na-lei-da-copa-e-prepara-castelao-para-inspecao-da-fifa-a-300-dias-do-mundial-1.3787756</t>
         </is>
       </c>
       <c r="G38" s="23" t="inlineStr">
@@ -31716,12 +31716,12 @@
       </c>
       <c r="H38" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I38" s="23" t="inlineStr">
         <is>
-          <t>A CBF destacou a trajetória da meio-campista Dulce, que integrou a campanha brasileira de quarto lugar no Mundial Sub-17 de 2025 e agora se prepara na Polônia para disputar sua primeira Copa do Mundo Feminina Sub-20. A atleta do Corinthians chega ao torneio após marcar 12 gols em 15 jogos na temporada e representa a transição da formação para uma categoria mais próxima da Seleção principal.</t>
+          <t>A 300 dias da Copa do Mundo Feminina 2027, Fortaleza informou que prepara a promulgação da Lei Estadual da Copa, conclui o plano de mobilidade e discute gratuidade no transporte público em dias de jogos. A Arena Castelão, que receberá nove partidas, terá nova inspeção técnica da FIFA em setembro, enquanto Estado, município e federação avançam em infraestrutura, responsabilidade social e legado.</t>
         </is>
       </c>
     </row>
@@ -31731,27 +31731,27 @@
       </c>
       <c r="B39" s="23" t="inlineStr">
         <is>
-          <t>Empetur abre licitação para infraestrutura temporária da Copa 2027 na Arena Pernambuco</t>
+          <t>Dulce transforma experiência no Mundial Sub-17 em preparação para a Seleção Sub-20</t>
         </is>
       </c>
       <c r="C39" s="23" t="inlineStr">
         <is>
-          <t>Infraestrutura / Arena Pernambuco / contratação pública</t>
+          <t>Seleções de Base / Sub-20 Feminina / transição de categoria</t>
         </is>
       </c>
       <c r="D39" s="23" t="inlineStr">
         <is>
-          <t>Recife/PE</t>
+          <t>Cracóvia/POL</t>
         </is>
       </c>
       <c r="E39" s="23" t="inlineStr">
         <is>
-          <t>Empetur</t>
+          <t>CBF</t>
         </is>
       </c>
       <c r="F39" s="23" t="inlineStr">
         <is>
-          <t>https://www.empetur.pe.gov.br/h-licitacoes/2556-empetur-aviso-de-abertura-processo-n-1687-2026-cel-iii-pe-0008-empetur</t>
+          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/de-um-mundial-ao-outro-dulce-vive-novo-desafio-com-a-selecao-brasileira</t>
         </is>
       </c>
       <c r="G39" s="23" t="inlineStr">
@@ -31766,7 +31766,7 @@
       </c>
       <c r="I39" s="23" t="inlineStr">
         <is>
-          <t>A Empetur abriu disputa para o fornecimento de cadeiras empilháveis destinadas à infraestrutura temporária da Copa do Mundo Feminina FIFA 2027 na Arena Pernambuco. A contratação tem valor máximo estimado de R$ 155.176, com posterior incorporação dos bens ao patrimônio do estádio.</t>
+          <t>A CBF destacou a trajetória da meio-campista Dulce, que integrou a campanha brasileira de quarto lugar no Mundial Sub-17 de 2025 e agora se prepara na Polônia para disputar sua primeira Copa do Mundo Feminina Sub-20. A atleta do Corinthians chega ao torneio após marcar 12 gols em 15 jogos na temporada e representa a transição da formação para uma categoria mais próxima da Seleção principal.</t>
         </is>
       </c>
     </row>
@@ -31776,27 +31776,27 @@
       </c>
       <c r="B40" s="23" t="inlineStr">
         <is>
-          <t>Lei Complementar destrava benefícios tributários federais para a Copa Feminina 2027</t>
+          <t>Empetur abre licitação para infraestrutura temporária da Copa 2027 na Arena Pernambuco</t>
         </is>
       </c>
       <c r="C40" s="23" t="inlineStr">
         <is>
-          <t>Tributação / legislação federal / organização</t>
+          <t>Infraestrutura / Arena Pernambuco / contratação pública</t>
         </is>
       </c>
       <c r="D40" s="23" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Recife/PE</t>
         </is>
       </c>
       <c r="E40" s="23" t="inlineStr">
         <is>
-          <t>Presidência da República</t>
+          <t>Empetur</t>
         </is>
       </c>
       <c r="F40" s="23" t="inlineStr">
         <is>
-          <t>https://www.planalto.gov.br/ccivil_03/leis/lcp/lcp235.htm</t>
+          <t>https://www.empetur.pe.gov.br/h-licitacoes/2556-empetur-aviso-de-abertura-processo-n-1687-2026-cel-iii-pe-0008-empetur</t>
         </is>
       </c>
       <c r="G40" s="23" t="inlineStr">
@@ -31806,12 +31806,12 @@
       </c>
       <c r="H40" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I40" s="23" t="inlineStr">
         <is>
-          <t>Sancionada em 27/08 e publicada em 28/08, a Lei Complementar nº 235/2026 excepciona regras fiscais para viabilizar benefícios tributários federais destinados à realização da Copa do Mundo Feminina FIFA 2027 no Brasil. A medida remove restrições legais à concessão dos incentivos previstos para a organização do torneio.</t>
+          <t>A Empetur abriu disputa para o fornecimento de cadeiras empilháveis destinadas à infraestrutura temporária da Copa do Mundo Feminina FIFA 2027 na Arena Pernambuco. A contratação tem valor máximo estimado de R$ 155.176, com posterior incorporação dos bens ao patrimônio do estádio.</t>
         </is>
       </c>
     </row>
@@ -31821,27 +31821,27 @@
       </c>
       <c r="B41" s="23" t="inlineStr">
         <is>
-          <t>Porto Alegre detalha Fan Fest e Caminho das Gurias a 300 dias da Copa 2027</t>
+          <t>Lei Complementar destrava benefícios tributários federais para a Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C41" s="23" t="inlineStr">
         <is>
-          <t>Contagem regressiva / Porto Alegre / Fan Fest / legado</t>
+          <t>Tributação / legislação federal / organização</t>
         </is>
       </c>
       <c r="D41" s="23" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E41" s="23" t="inlineStr">
         <is>
-          <t>Correio do Povo</t>
+          <t>Presidência da República</t>
         </is>
       </c>
       <c r="F41" s="23" t="inlineStr">
         <is>
-          <t>https://www.correiodopovo.com.br/esportes/300-dias-para-a-copa-feminina-veja-o-que-ja-se-sabe-sobre-o-mundial-1.1743064</t>
+          <t>https://www.planalto.gov.br/ccivil_03/leis/lcp/lcp235.htm</t>
         </is>
       </c>
       <c r="G41" s="23" t="inlineStr">
@@ -31851,12 +31851,12 @@
       </c>
       <c r="H41" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I41" s="23" t="inlineStr">
         <is>
-          <t>A 300 dias da Copa do Mundo Feminina 2027, Porto Alegre informou que prepara Fan Fest, ativações e o Caminho das Gurias, experiência inspirada no Caminho do Gol de 2014. A matéria também consolida os sete jogos no Beira-Rio, o programa de voluntários e a estratégia de levar o legado do torneio a escolas, projetos sociais e comunidades.</t>
+          <t>Sancionada em 27/08 e publicada em 28/08, a Lei Complementar nº 235/2026 excepciona regras fiscais para viabilizar benefícios tributários federais destinados à realização da Copa do Mundo Feminina FIFA 2027 no Brasil. A medida remove restrições legais à concessão dos incentivos previstos para a organização do torneio.</t>
         </is>
       </c>
     </row>
@@ -31866,77 +31866,77 @@
       </c>
       <c r="B42" s="23" t="inlineStr">
         <is>
-          <t>Vaquejada e reforma podem tirar fase final da repescagem da Arena Pernambuco</t>
+          <t>Porto Alegre detalha Fan Fest e Caminho das Gurias a 300 dias da Copa 2027</t>
         </is>
       </c>
       <c r="C42" s="23" t="inlineStr">
         <is>
-          <t>Repescagem / infraestrutura / cidade-sede</t>
+          <t>Contagem regressiva / Porto Alegre / Fan Fest / legado</t>
         </is>
       </c>
       <c r="D42" s="23" t="inlineStr">
         <is>
-          <t>Recife/PE</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="E42" s="23" t="inlineStr">
         <is>
-          <t>Diário de Pernambuco</t>
+          <t>Correio do Povo</t>
         </is>
       </c>
       <c r="F42" s="23" t="inlineStr">
         <is>
-          <t>https://www.diariodepernambuco.com.br/esportes-dp/internacional/2026/08/11722675-vaquejada-pode-tirar-repescagem-da-copa-do-mundo-feminina-da-arena-de-pernambuco.html</t>
+          <t>https://www.correiodopovo.com.br/esportes/300-dias-para-a-copa-feminina-veja-o-que-ja-se-sabe-sobre-o-mundial-1.1743064</t>
         </is>
       </c>
       <c r="G42" s="23" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Positivo</t>
         </is>
       </c>
       <c r="H42" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I42" s="23" t="inlineStr">
         <is>
-          <t>A FIFA solicitou a Arena Pernambuco para a fase final do Torneio Classificatório da Copa Feminina 2027, prevista entre 23 de fevereiro e 6 de março de 2027. Uma vaquejada marcada para novembro de 2026, a substituição do gramado e o cronograma de reformas podem inviabilizar o estádio; as tratativas continuam e outras sedes são avaliadas.</t>
+          <t>A 300 dias da Copa do Mundo Feminina 2027, Porto Alegre informou que prepara Fan Fest, ativações e o Caminho das Gurias, experiência inspirada no Caminho do Gol de 2014. A matéria também consolida os sete jogos no Beira-Rio, o programa de voluntários e a estratégia de levar o legado do torneio a escolas, projetos sociais e comunidades.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="32" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="B43" s="23" t="inlineStr">
         <is>
-          <t>Bahia propõe proteção às mulheres e fórum permanente das cidades-sede para a Copa 2027</t>
+          <t>Vaquejada e reforma podem tirar fase final da repescagem da Arena Pernambuco</t>
         </is>
       </c>
       <c r="C43" s="23" t="inlineStr">
         <is>
-          <t>Workshop das Cidades-Sede / segurança das mulheres / legado / Salvador</t>
+          <t>Repescagem / infraestrutura / cidade-sede</t>
         </is>
       </c>
       <c r="D43" s="23" t="inlineStr">
         <is>
-          <t>Salvador/BA</t>
+          <t>Recife/PE</t>
         </is>
       </c>
       <c r="E43" s="23" t="inlineStr">
         <is>
-          <t>Bahia Notícias</t>
+          <t>Diário de Pernambuco</t>
         </is>
       </c>
       <c r="F43" s="23" t="inlineStr">
         <is>
-          <t>https://www.bahianoticias.com.br/esportes/noticia/80028-protecao-as-mulheres-entra-no-planejamento-da-bahia-para-a-copa-feminina-de-2027</t>
+          <t>https://www.diariodepernambuco.com.br/esportes-dp/internacional/2026/08/11722675-vaquejada-pode-tirar-repescagem-da-copa-do-mundo-feminina-da-arena-de-pernambuco.html</t>
         </is>
       </c>
       <c r="G43" s="23" t="inlineStr">
         <is>
-          <t>Positivo</t>
+          <t>Neutro</t>
         </is>
       </c>
       <c r="H43" s="23" t="inlineStr">
@@ -31946,7 +31946,7 @@
       </c>
       <c r="I43" s="23" t="inlineStr">
         <is>
-          <t>No Workshop das Cidades-Sede da Copa Feminina 2027, a delegação baiana propôs tornar permanente a ação de vagão exclusivo para mulheres no metrô de Salvador, ampliar as Salas Elas à Frente e criar um fórum contínuo entre as oito sedes para articular mobilidade, segurança e operação do torneio.</t>
+          <t>A FIFA solicitou a Arena Pernambuco para a fase final do Torneio Classificatório da Copa Feminina 2027, prevista entre 23 de fevereiro e 6 de março de 2027. Uma vaquejada marcada para novembro de 2026, a substituição do gramado e o cronograma de reformas podem inviabilizar o estádio; as tratativas continuam e outras sedes são avaliadas.</t>
         </is>
       </c>
     </row>
@@ -31956,27 +31956,27 @@
       </c>
       <c r="B44" s="23" t="inlineStr">
         <is>
-          <t>Buscas pela Copa Feminina 2027 impulsionam interesse digital e oportunidades para marcas</t>
+          <t>Bahia propõe proteção às mulheres e fórum permanente das cidades-sede para a Copa 2027</t>
         </is>
       </c>
       <c r="C44" s="23" t="inlineStr">
         <is>
-          <t>Marketing / audiência digital / patrocínios / Copa Feminina 2027</t>
+          <t>Workshop das Cidades-Sede / segurança das mulheres / legado / Salvador</t>
         </is>
       </c>
       <c r="D44" s="23" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Salvador/BA</t>
         </is>
       </c>
       <c r="E44" s="23" t="inlineStr">
         <is>
-          <t>Meio &amp; Mensagem</t>
+          <t>Bahia Notícias</t>
         </is>
       </c>
       <c r="F44" s="23" t="inlineStr">
         <is>
-          <t>https://www.meioemensagem.com.br/womentowatch/interesse-pelo-futebol-feminino-dispara-no-digital</t>
+          <t>https://www.bahianoticias.com.br/esportes/noticia/80028-protecao-as-mulheres-entra-no-planejamento-da-bahia-para-a-copa-feminina-de-2027</t>
         </is>
       </c>
       <c r="G44" s="23" t="inlineStr">
@@ -31986,12 +31986,12 @@
       </c>
       <c r="H44" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I44" s="23" t="inlineStr">
         <is>
-          <t>Estudo divulgado no evento FF.Co mostrou alta de 200% nas buscas brasileiras por futebol feminino no YouTube e de 130% no Google em cinco anos. As dúvidas mais pesquisadas em 2026 incluem sedes, voluntariado, ingressos e transmissão da Copa do Mundo Feminina 2027, reforçando o potencial comercial do torneio para patrocinadores.</t>
+          <t>No Workshop das Cidades-Sede da Copa Feminina 2027, a delegação baiana propôs tornar permanente a ação de vagão exclusivo para mulheres no metrô de Salvador, ampliar as Salas Elas à Frente e criar um fórum contínuo entre as oito sedes para articular mobilidade, segurança e operação do torneio.</t>
         </is>
       </c>
     </row>
@@ -32001,27 +32001,27 @@
       </c>
       <c r="B45" s="23" t="inlineStr">
         <is>
-          <t>Camilla Orlando avalia ajustes finais da Seleção Sub-20 após primeiro treino na Polônia</t>
+          <t>Buscas pela Copa Feminina 2027 impulsionam interesse digital e oportunidades para marcas</t>
         </is>
       </c>
       <c r="C45" s="23" t="inlineStr">
         <is>
-          <t>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</t>
+          <t>Marketing / audiência digital / patrocínios / Copa Feminina 2027</t>
         </is>
       </c>
       <c r="D45" s="23" t="inlineStr">
         <is>
-          <t>Cracóvia/POL</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E45" s="23" t="inlineStr">
         <is>
-          <t>CBF</t>
+          <t>Meio &amp; Mensagem</t>
         </is>
       </c>
       <c r="F45" s="23" t="inlineStr">
         <is>
-          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/camilla-orlando-analisa-preparacao-do-brasil-apos-primeiro-treino-para-o-mundial-sub-20-e-o-momento-dos-ajustes-finais</t>
+          <t>https://www.meioemensagem.com.br/womentowatch/interesse-pelo-futebol-feminino-dispara-no-digital</t>
         </is>
       </c>
       <c r="G45" s="23" t="inlineStr">
@@ -32036,7 +32036,7 @@
       </c>
       <c r="I45" s="23" t="inlineStr">
         <is>
-          <t>Após o primeiro treino em campo na Polônia, a técnica Camilla Orlando avaliou a preparação da Seleção Brasileira Feminina Sub-20 para a Copa do Mundo e destacou que a etapa é dedicada aos ajustes finais antes da estreia no torneio.</t>
+          <t>Estudo divulgado no evento FF.Co mostrou alta de 200% nas buscas brasileiras por futebol feminino no YouTube e de 130% no Google em cinco anos. As dúvidas mais pesquisadas em 2026 incluem sedes, voluntariado, ingressos e transmissão da Copa do Mundo Feminina 2027, reforçando o potencial comercial do torneio para patrocinadores.</t>
         </is>
       </c>
     </row>
@@ -32046,27 +32046,27 @@
       </c>
       <c r="B46" s="23" t="inlineStr">
         <is>
-          <t>Rio propõe benefícios fiscais e metas de legado para a Copa Feminina 2027</t>
+          <t>Camilla Orlando avalia ajustes finais da Seleção Sub-20 após primeiro treino na Polônia</t>
         </is>
       </c>
       <c r="C46" s="23" t="inlineStr">
         <is>
-          <t>Políticas públicas / benefícios fiscais / legado / Rio de Janeiro</t>
+          <t>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</t>
         </is>
       </c>
       <c r="D46" s="23" t="inlineStr">
         <is>
-          <t>Rio de Janeiro/RJ</t>
+          <t>Cracóvia/POL</t>
         </is>
       </c>
       <c r="E46" s="23" t="inlineStr">
         <is>
-          <t>Alerj</t>
+          <t>CBF</t>
         </is>
       </c>
       <c r="F46" s="23" t="inlineStr">
         <is>
-          <t>https://www.alerj.rj.gov.br/Visualizar/Noticia/87696</t>
+          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/camilla-orlando-analisa-preparacao-do-brasil-apos-primeiro-treino-para-o-mundial-sub-20-e-o-momento-dos-ajustes-finais</t>
         </is>
       </c>
       <c r="G46" s="23" t="inlineStr">
@@ -32076,12 +32076,12 @@
       </c>
       <c r="H46" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I46" s="23" t="inlineStr">
         <is>
-          <t>A Alerj recebeu o Projeto de Lei 8.223/26, que incorpora benefícios de ICMS vinculados à organização da Copa do Mundo Feminina 2027. A proposta estabelece metas de mais de 7.500 empregos diretos no estado, público acumulado superior a 150 mil pessoas nos jogos e compromissos ambientais, com avaliação após o torneio.</t>
+          <t>Após o primeiro treino em campo na Polônia, a técnica Camilla Orlando avaliou a preparação da Seleção Brasileira Feminina Sub-20 para a Copa do Mundo e destacou que a etapa é dedicada aos ajustes finais antes da estreia no torneio.</t>
         </is>
       </c>
     </row>
@@ -32091,27 +32091,27 @@
       </c>
       <c r="B47" s="23" t="inlineStr">
         <is>
-          <t>Vitorinha destaca força de vontade e companheirismo da Seleção Sub-20 para o Mundial</t>
+          <t>Rio propõe benefícios fiscais e metas de legado para a Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C47" s="23" t="inlineStr">
         <is>
-          <t>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</t>
+          <t>Políticas públicas / benefícios fiscais / legado / Rio de Janeiro</t>
         </is>
       </c>
       <c r="D47" s="23" t="inlineStr">
         <is>
-          <t>Cracóvia/POL</t>
+          <t>Rio de Janeiro/RJ</t>
         </is>
       </c>
       <c r="E47" s="23" t="inlineStr">
         <is>
-          <t>CBF</t>
+          <t>Alerj</t>
         </is>
       </c>
       <c r="F47" s="23" t="inlineStr">
         <is>
-          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/vitorinha-celebra-oportunidade-no-mundial-e-destaca-pontos-fortes-do-brasil-para-a-competicao</t>
+          <t>https://www.alerj.rj.gov.br/Visualizar/Noticia/87696</t>
         </is>
       </c>
       <c r="G47" s="23" t="inlineStr">
@@ -32121,42 +32121,42 @@
       </c>
       <c r="H47" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I47" s="23" t="inlineStr">
         <is>
-          <t>Em preparação na Polônia para a Copa do Mundo Feminina Sub-20, a meio-campista Vitorinha celebrou a oportunidade de disputar o Mundial e apontou força de vontade e companheirismo como pontos fortes da Seleção Brasileira. A atleta também relembrou sua trajetória até a convocação.</t>
+          <t>A Alerj recebeu o Projeto de Lei 8.223/26, que incorpora benefícios de ICMS vinculados à organização da Copa do Mundo Feminina 2027. A proposta estabelece metas de mais de 7.500 empregos diretos no estado, público acumulado superior a 150 mil pessoas nos jogos e compromissos ambientais, com avaliação após o torneio.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="32" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="B48" s="23" t="inlineStr">
         <is>
-          <t>FIFA anuncia Tour da Taça por todas as cidades-sede antes da Copa 2027</t>
+          <t>Vitorinha destaca força de vontade e companheirismo da Seleção Sub-20 para o Mundial</t>
         </is>
       </c>
       <c r="C48" s="23" t="inlineStr">
         <is>
-          <t>Tour da Taça / ativações / EVT-0090</t>
+          <t>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</t>
         </is>
       </c>
       <c r="D48" s="23" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Cracóvia/POL</t>
         </is>
       </c>
       <c r="E48" s="23" t="inlineStr">
         <is>
-          <t>Correio do Povo</t>
+          <t>CBF</t>
         </is>
       </c>
       <c r="F48" s="23" t="inlineStr">
         <is>
-          <t>https://www.correiodopovo.com.br/esportes/taca-da-copa-feminina-fara-tour-pelo-brasil-entre-abril-e-maio-de-2027-1.1742125</t>
+          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/vitorinha-celebra-oportunidade-no-mundial-e-destaca-pontos-fortes-do-brasil-para-a-competicao</t>
         </is>
       </c>
       <c r="G48" s="23" t="inlineStr">
@@ -32166,12 +32166,12 @@
       </c>
       <c r="H48" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I48" s="23" t="inlineStr">
         <is>
-          <t>Durante o II Workshop de Cidades-Sede e Estádios, a FIFA anunciou o Tour da Taça (EVT-0090) para abril e maio de 2027. O troféu deverá passar pelas oito cidades-sede; datas e locais ainda serão definidos, enquanto Porto Alegre negocia uma permanência de pelo menos cinco dias e exposição no Beira-Rio.</t>
+          <t>Em preparação na Polônia para a Copa do Mundo Feminina Sub-20, a meio-campista Vitorinha celebrou a oportunidade de disputar o Mundial e apontou força de vontade e companheirismo como pontos fortes da Seleção Brasileira. A atleta também relembrou sua trajetória até a convocação.</t>
         </is>
       </c>
     </row>
@@ -32181,27 +32181,27 @@
       </c>
       <c r="B49" s="23" t="inlineStr">
         <is>
-          <t>Porto Alegre mapeia ajustes de infraestrutura no workshop da Copa 2027</t>
+          <t>FIFA anuncia Tour da Taça por todas as cidades-sede antes da Copa 2027</t>
         </is>
       </c>
       <c r="C49" s="23" t="inlineStr">
         <is>
-          <t>II Workshop de Cidades-Sede e Estádios / Porto Alegre</t>
+          <t>Tour da Taça / ativações / EVT-0090</t>
         </is>
       </c>
       <c r="D49" s="23" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E49" s="23" t="inlineStr">
         <is>
-          <t>Federação Gaúcha de Futebol</t>
+          <t>Correio do Povo</t>
         </is>
       </c>
       <c r="F49" s="23" t="inlineStr">
         <is>
-          <t>https://www.fgf.com.br/noticia/fgf-participa-do-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-2027</t>
+          <t>https://www.correiodopovo.com.br/esportes/taca-da-copa-feminina-fara-tour-pelo-brasil-entre-abril-e-maio-de-2027-1.1742125</t>
         </is>
       </c>
       <c r="G49" s="23" t="inlineStr">
@@ -32211,12 +32211,12 @@
       </c>
       <c r="H49" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I49" s="23" t="inlineStr">
         <is>
-          <t>A delegação gaúcha detalhou sua participação no II Workshop de Cidades-Sede e Estádios da Copa 2027. FIFA e CBF realizaram sessões individuais com as sedes para avaliar o planejamento, mapear iniciativas já executadas e indicar ajustes de infraestrutura; Porto Alegre apresentou seu avanço ao lado do Governo do RS, da FGF e do Internacional, responsável pelo Beira-Rio.</t>
+          <t>Durante o II Workshop de Cidades-Sede e Estádios, a FIFA anunciou o Tour da Taça (EVT-0090) para abril e maio de 2027. O troféu deverá passar pelas oito cidades-sede; datas e locais ainda serão definidos, enquanto Porto Alegre negocia uma permanência de pelo menos cinco dias e exposição no Beira-Rio.</t>
         </is>
       </c>
     </row>
@@ -32226,27 +32226,27 @@
       </c>
       <c r="B50" s="23" t="inlineStr">
         <is>
-          <t>Recife integrará programa de voluntários da Copa Feminina 2027</t>
+          <t>Porto Alegre mapeia ajustes de infraestrutura no workshop da Copa 2027</t>
         </is>
       </c>
       <c r="C50" s="23" t="inlineStr">
         <is>
-          <t>Voluntariado / preparação das cidades-sede / Recife</t>
+          <t>II Workshop de Cidades-Sede e Estádios / Porto Alegre</t>
         </is>
       </c>
       <c r="D50" s="23" t="inlineStr">
         <is>
-          <t>Recife/PE</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="E50" s="23" t="inlineStr">
         <is>
-          <t>Folha de Pernambuco</t>
+          <t>Federação Gaúcha de Futebol</t>
         </is>
       </c>
       <c r="F50" s="23" t="inlineStr">
         <is>
-          <t>https://www.folhape.com.br/esportes/copa-feminina-2027-recife-integrara-programa-de-voluntarios/508924/</t>
+          <t>https://www.fgf.com.br/noticia/fgf-participa-do-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-2027</t>
         </is>
       </c>
       <c r="G50" s="23" t="inlineStr">
@@ -32261,7 +32261,7 @@
       </c>
       <c r="I50" s="23" t="inlineStr">
         <is>
-          <t>Recife confirmou participação no programa de voluntários da Copa do Mundo Feminina 2027. A seleção oficial para atuar no Mundial está prevista para começar em setembro, ampliando a preparação operacional e o envolvimento da cidade-sede pernambucana.</t>
+          <t>A delegação gaúcha detalhou sua participação no II Workshop de Cidades-Sede e Estádios da Copa 2027. FIFA e CBF realizaram sessões individuais com as sedes para avaliar o planejamento, mapear iniciativas já executadas e indicar ajustes de infraestrutura; Porto Alegre apresentou seu avanço ao lado do Governo do RS, da FGF e do Internacional, responsável pelo Beira-Rio.</t>
         </is>
       </c>
     </row>
@@ -32271,27 +32271,27 @@
       </c>
       <c r="B51" s="23" t="inlineStr">
         <is>
-          <t>Seleção Brasileira Sub-20 desembarca na Polônia para o Mundial</t>
+          <t>Recife integrará programa de voluntários da Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C51" s="23" t="inlineStr">
         <is>
-          <t>Seleções de Base / Sub-20 Feminina</t>
+          <t>Voluntariado / preparação das cidades-sede / Recife</t>
         </is>
       </c>
       <c r="D51" s="23" t="inlineStr">
         <is>
-          <t>Bielsko-Biała/POL</t>
+          <t>Recife/PE</t>
         </is>
       </c>
       <c r="E51" s="23" t="inlineStr">
         <is>
-          <t>CBF</t>
+          <t>Folha de Pernambuco</t>
         </is>
       </c>
       <c r="F51" s="23" t="inlineStr">
         <is>
-          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/selecao-feminina-sub-20-desembarca-na-polonia-para-disputar-a-copa-do-mundo</t>
+          <t>https://www.folhape.com.br/esportes/copa-feminina-2027-recife-integrara-programa-de-voluntarios/508924/</t>
         </is>
       </c>
       <c r="G51" s="23" t="inlineStr">
@@ -32306,7 +32306,7 @@
       </c>
       <c r="I51" s="23" t="inlineStr">
         <is>
-          <t>A Seleção Brasileira Feminina Sub-20 chegou à Polônia e iniciou a preparação local para a Copa do Mundo da categoria, que começa em 5 de setembro. O Brasil enfrentará Tanzânia, Canadá e Inglaterra na fase de grupos.</t>
+          <t>Recife confirmou participação no programa de voluntários da Copa do Mundo Feminina 2027. A seleção oficial para atuar no Mundial está prevista para começar em setembro, ampliando a preparação operacional e o envolvimento da cidade-sede pernambucana.</t>
         </is>
       </c>
     </row>
@@ -32316,12 +32316,12 @@
       </c>
       <c r="B52" s="23" t="inlineStr">
         <is>
-          <t>Seleção Feminina Sub-20 inicia adaptação na Polônia após viagem</t>
+          <t>Seleção Brasileira Sub-20 desembarca na Polônia para o Mundial</t>
         </is>
       </c>
       <c r="C52" s="23" t="inlineStr">
         <is>
-          <t>Seleções de Base / Sub-20 Feminina / preparação</t>
+          <t>Seleções de Base / Sub-20 Feminina</t>
         </is>
       </c>
       <c r="D52" s="23" t="inlineStr">
@@ -32336,7 +32336,7 @@
       </c>
       <c r="F52" s="23" t="inlineStr">
         <is>
-          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/com-atividades-no-hotel-selecao-feminina-sub-20-comeca-adaptacao-na-polonia</t>
+          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/selecao-feminina-sub-20-desembarca-na-polonia-para-disputar-a-copa-do-mundo</t>
         </is>
       </c>
       <c r="G52" s="23" t="inlineStr">
@@ -32351,7 +32351,7 @@
       </c>
       <c r="I52" s="23" t="inlineStr">
         <is>
-          <t>Em novo capítulo da preparação para a Copa do Mundo Feminina Sub-20, a Seleção Brasileira iniciou em Bielsko-Biała atividades leves de adaptação após a viagem à Polônia, com caminhada, mobilidade e recuperação orientadas pela comissão técnica antes dos treinamentos de campo.</t>
+          <t>A Seleção Brasileira Feminina Sub-20 chegou à Polônia e iniciou a preparação local para a Copa do Mundo da categoria, que começa em 5 de setembro. O Brasil enfrentará Tanzânia, Canadá e Inglaterra na fase de grupos.</t>
         </is>
       </c>
     </row>
@@ -32361,27 +32361,27 @@
       </c>
       <c r="B53" s="23" t="inlineStr">
         <is>
-          <t>Sportv lança campanha e debate cobertura da Copa 2027 no Festival Feitas de Esporte</t>
+          <t>Seleção Feminina Sub-20 inicia adaptação na Polônia após viagem</t>
         </is>
       </c>
       <c r="C53" s="23" t="inlineStr">
         <is>
-          <t>Festival Feitas de Esporte / mídia / ativação / Copa Feminina 2027</t>
+          <t>Seleções de Base / Sub-20 Feminina / preparação</t>
         </is>
       </c>
       <c r="D53" s="23" t="inlineStr">
         <is>
-          <t>São Paulo/SP</t>
+          <t>Bielsko-Biała/POL</t>
         </is>
       </c>
       <c r="E53" s="23" t="inlineStr">
         <is>
-          <t>Meio &amp; Mensagem</t>
+          <t>CBF</t>
         </is>
       </c>
       <c r="F53" s="23" t="inlineStr">
         <is>
-          <t>https://www.meioemensagem.com.br/midia/sportv-faz-evento-para-celebrar-protagonismo-feminino</t>
+          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/com-atividades-no-hotel-selecao-feminina-sub-20-comeca-adaptacao-na-polonia</t>
         </is>
       </c>
       <c r="G53" s="23" t="inlineStr">
@@ -32396,7 +32396,7 @@
       </c>
       <c r="I53" s="23" t="inlineStr">
         <is>
-          <t>O Sportv anunciou o Festival Feitas de Esporte para 30/08 na Nossa Arena, em São Paulo, com atividades esportivas, lançamento de campanha sobre futebol feminino e debate específico sobre a cobertura do canal para a Copa do Mundo Feminina 2027. O evento relacionado reúne Alline Calandrini, Júlia Vergueiro e convidados e também marca a entrega de novos vestiários.</t>
+          <t>Em novo capítulo da preparação para a Copa do Mundo Feminina Sub-20, a Seleção Brasileira iniciou em Bielsko-Biała atividades leves de adaptação após a viagem à Polônia, com caminhada, mobilidade e recuperação orientadas pela comissão técnica antes dos treinamentos de campo.</t>
         </is>
       </c>
     </row>
@@ -32406,87 +32406,87 @@
       </c>
       <c r="B54" s="23" t="inlineStr">
         <is>
-          <t>UEFA deve retirar ameaça de boicote antes do Mundial Feminino Sub-20</t>
+          <t>Sportv lança campanha e debate cobertura da Copa 2027 no Festival Feitas de Esporte</t>
         </is>
       </c>
       <c r="C54" s="23" t="inlineStr">
         <is>
-          <t>Seleções de Base / Sub-20 Feminina / governança FIFA</t>
+          <t>Festival Feitas de Esporte / mídia / ativação / Copa Feminina 2027</t>
         </is>
       </c>
       <c r="D54" s="23" t="inlineStr">
         <is>
-          <t>Internacional</t>
+          <t>São Paulo/SP</t>
         </is>
       </c>
       <c r="E54" s="23" t="inlineStr">
         <is>
-          <t>Folha de S.Paulo / AFP</t>
+          <t>Meio &amp; Mensagem</t>
         </is>
       </c>
       <c r="F54" s="23" t="inlineStr">
         <is>
-          <t>https://www1.folha.uol.com.br/esporte/2026/08/uefa-deve-retirar-ameaca-de-boicote-a-torneios-da-fifa.shtml</t>
+          <t>https://www.meioemensagem.com.br/midia/sportv-faz-evento-para-celebrar-protagonismo-feminino</t>
         </is>
       </c>
       <c r="G54" s="23" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Positivo</t>
         </is>
       </c>
       <c r="H54" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I54" s="23" t="inlineStr">
         <is>
-          <t>A UEFA deve retirar a ameaça de boicote às competições da FIFA antes da Copa do Mundo Feminina Sub-20 de 2026 na Polônia, torneio que contará com a Seleção Brasileira. O desdobramento reduz a incerteza institucional às vésperas da estreia do Brasil em 5 de setembro.</t>
+          <t>O Sportv anunciou o Festival Feitas de Esporte para 30/08 na Nossa Arena, em São Paulo, com atividades esportivas, lançamento de campanha sobre futebol feminino e debate específico sobre a cobertura do canal para a Copa do Mundo Feminina 2027. O evento relacionado reúne Alline Calandrini, Júlia Vergueiro e convidados e também marca a entrega de novos vestiários.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="32" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="B55" s="23" t="inlineStr">
         <is>
-          <t>Acarajé é autorizado dentro da Arena Fonte Nova durante a Copa Feminina 2027</t>
+          <t>UEFA deve retirar ameaça de boicote antes do Mundial Feminino Sub-20</t>
         </is>
       </c>
       <c r="C55" s="23" t="inlineStr">
         <is>
-          <t>Cultura / turismo / alimentação / Salvador</t>
+          <t>Seleções de Base / Sub-20 Feminina / governança FIFA</t>
         </is>
       </c>
       <c r="D55" s="23" t="inlineStr">
         <is>
-          <t>Salvador/BA</t>
+          <t>Internacional</t>
         </is>
       </c>
       <c r="E55" s="23" t="inlineStr">
         <is>
-          <t>A TARDE</t>
+          <t>Folha de S.Paulo / AFP</t>
         </is>
       </c>
       <c r="F55" s="23" t="inlineStr">
         <is>
-          <t>https://atarde.com.br/bahia/copa-feminina-2027-tera-acaraje-dentro-da-arena-fonte-nova-1399762</t>
+          <t>https://www1.folha.uol.com.br/esporte/2026/08/uefa-deve-retirar-ameaca-de-boicote-a-torneios-da-fifa.shtml</t>
         </is>
       </c>
       <c r="G55" s="23" t="inlineStr">
         <is>
-          <t>Positivo</t>
+          <t>Neutro</t>
         </is>
       </c>
       <c r="H55" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I55" s="23" t="inlineStr">
         <is>
-          <t>Após articulação do Governo da Bahia, GECOPA, Prefeitura de Salvador e Arena Fonte Nova, as baianas de acarajé foram autorizadas a vender o produto dentro do estádio durante os jogos da Copa Feminina 2027. A decisão integra a estratégia de legado cultural e promoção turística da sede baiana.</t>
+          <t>A UEFA deve retirar a ameaça de boicote às competições da FIFA antes da Copa do Mundo Feminina Sub-20 de 2026 na Polônia, torneio que contará com a Seleção Brasileira. O desdobramento reduz a incerteza institucional às vésperas da estreia do Brasil em 5 de setembro.</t>
         </is>
       </c>
     </row>
@@ -32496,42 +32496,42 @@
       </c>
       <c r="B56" s="23" t="inlineStr">
         <is>
-          <t>Boicote europeu e meta de premiação pressionam o sorteio da Copa Feminina 2027</t>
+          <t>Acarajé é autorizado dentro da Arena Fonte Nova durante a Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C56" s="23" t="inlineStr">
         <is>
-          <t>Sorteio / governança / premiação / EVT-0010</t>
+          <t>Cultura / turismo / alimentação / Salvador</t>
         </is>
       </c>
       <c r="D56" s="23" t="inlineStr">
         <is>
-          <t>Rio de Janeiro/RJ</t>
+          <t>Salvador/BA</t>
         </is>
       </c>
       <c r="E56" s="23" t="inlineStr">
         <is>
-          <t>Máquina do Esporte</t>
+          <t>A TARDE</t>
         </is>
       </c>
       <c r="F56" s="23" t="inlineStr">
         <is>
-          <t>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/boicote-da-uefa-e-premios-em-dinheiro-marcam-sorteio-da-copa-do-mundo-feminina-2027-no-rio/</t>
+          <t>https://atarde.com.br/bahia/copa-feminina-2027-tera-acaraje-dentro-da-arena-fonte-nova-1399762</t>
         </is>
       </c>
       <c r="G56" s="23" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Positivo</t>
         </is>
       </c>
       <c r="H56" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I56" s="23" t="inlineStr">
         <is>
-          <t>Em novo desdobramento do sorteio dos grupos (EVT-0010), a FIFA enfrenta ameaça de boicote de países da Uefa e projeta US$ 1 bilhão em receita para a Copa Feminina 2027. Gianni Infantino também prometeu equiparar a premiação do torneio no Brasil à da Copa Masculina de 2026, embora o valor ainda não tenha sido anunciado.</t>
+          <t>Após articulação do Governo da Bahia, GECOPA, Prefeitura de Salvador e Arena Fonte Nova, as baianas de acarajé foram autorizadas a vender o produto dentro do estádio durante os jogos da Copa Feminina 2027. A decisão integra a estratégia de legado cultural e promoção turística da sede baiana.</t>
         </is>
       </c>
     </row>
@@ -32541,27 +32541,27 @@
       </c>
       <c r="B57" s="23" t="inlineStr">
         <is>
-          <t>Conmebol ajusta calendário continental de 2027 para a pausa da Copa Feminina</t>
+          <t>Boicote europeu e meta de premiação pressionam o sorteio da Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C57" s="23" t="inlineStr">
         <is>
-          <t>Calendário continental / clubes / organização</t>
+          <t>Sorteio / governança / premiação / EVT-0010</t>
         </is>
       </c>
       <c r="D57" s="23" t="inlineStr">
         <is>
-          <t>América do Sul / Brasil</t>
+          <t>Rio de Janeiro/RJ</t>
         </is>
       </c>
       <c r="E57" s="23" t="inlineStr">
         <is>
-          <t>ge</t>
+          <t>Máquina do Esporte</t>
         </is>
       </c>
       <c r="F57" s="23" t="inlineStr">
         <is>
-          <t>https://ge.globo.com/rs/futebol/noticia/2026/08/25/conmebol-divulga-calendario-de-2027-com-paralisacao-para-copa-do-mundo-feminina.ghtml</t>
+          <t>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/boicote-da-uefa-e-premios-em-dinheiro-marcam-sorteio-da-copa-do-mundo-feminina-2027-no-rio/</t>
         </is>
       </c>
       <c r="G57" s="23" t="inlineStr">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="I57" s="23" t="inlineStr">
         <is>
-          <t>A Conmebol divulgou o calendário de Libertadores, Sul-Americana e Recopa de 2027 já considerando a paralisação durante a Copa do Mundo Feminina no Brasil. A decisão amplia para as competições continentais o ajuste de calendário que afeta os clubes brasileiros e reduz conflitos durante o Mundial.</t>
+          <t>Em novo desdobramento do sorteio dos grupos (EVT-0010), a FIFA enfrenta ameaça de boicote de países da Uefa e projeta US$ 1 bilhão em receita para a Copa Feminina 2027. Gianni Infantino também prometeu equiparar a premiação do torneio no Brasil à da Copa Masculina de 2026, embora o valor ainda não tenha sido anunciado.</t>
         </is>
       </c>
     </row>
@@ -32586,32 +32586,32 @@
       </c>
       <c r="B58" s="23" t="inlineStr">
         <is>
-          <t>FIFA projeta Copa Feminina 2027 como primeira edição lucrativa da história</t>
+          <t>Conmebol ajusta calendário continental de 2027 para a pausa da Copa Feminina</t>
         </is>
       </c>
       <c r="C58" s="23" t="inlineStr">
         <is>
-          <t>Negócios / audiência / patrocínios</t>
+          <t>Calendário continental / clubes / organização</t>
         </is>
       </c>
       <c r="D58" s="23" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>América do Sul / Brasil</t>
         </is>
       </c>
       <c r="E58" s="23" t="inlineStr">
         <is>
-          <t>MKT Esportivo</t>
+          <t>ge</t>
         </is>
       </c>
       <c r="F58" s="23" t="inlineStr">
         <is>
-          <t>https://www.mktesportivo.com/2026/08/copa-do-mundo-2027-chega-ao-brasil-com-meta-de-lucro-e-maior-interesse-comercial/</t>
+          <t>https://ge.globo.com/rs/futebol/noticia/2026/08/25/conmebol-divulga-calendario-de-2027-com-paralisacao-para-copa-do-mundo-feminina.ghtml</t>
         </is>
       </c>
       <c r="G58" s="23" t="inlineStr">
         <is>
-          <t>Positivo</t>
+          <t>Neutro</t>
         </is>
       </c>
       <c r="H58" s="23" t="inlineStr">
@@ -32621,7 +32621,7 @@
       </c>
       <c r="I58" s="23" t="inlineStr">
         <is>
-          <t>Em entrevista, Gal Barradas, executiva da FIFA para receitas, marketing e inteligência de negócios da Copa Feminina 2027, afirmou que a entidade projeta a primeira edição lucrativa da história do torneio. O mercado brasileiro, o fuso favorável à audiência internacional e o interesse de marcas sustentam a expectativa comercial.</t>
+          <t>A Conmebol divulgou o calendário de Libertadores, Sul-Americana e Recopa de 2027 já considerando a paralisação durante a Copa do Mundo Feminina no Brasil. A decisão amplia para as competições continentais o ajuste de calendário que afeta os clubes brasileiros e reduz conflitos durante o Mundial.</t>
         </is>
       </c>
     </row>
@@ -32631,87 +32631,87 @@
       </c>
       <c r="B59" s="23" t="inlineStr">
         <is>
-          <t>Porto Alegre busca amistoso da Seleção antes da Copa Feminina 2027</t>
+          <t>FIFA projeta Copa Feminina 2027 como primeira edição lucrativa da história</t>
         </is>
       </c>
       <c r="C59" s="23" t="inlineStr">
         <is>
-          <t>Seleção Brasileira / preparação / Porto Alegre</t>
+          <t>Negócios / audiência / patrocínios</t>
         </is>
       </c>
       <c r="D59" s="23" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E59" s="23" t="inlineStr">
         <is>
-          <t>GZH</t>
+          <t>MKT Esportivo</t>
         </is>
       </c>
       <c r="F59" s="23" t="inlineStr">
         <is>
-          <t>https://gauchazh.clicrbs.com.br/esportes/futebol-feminino/noticia/2026/08/uma-das-sedes-da-copa-do-mundo-feminina-de-2027-porto-alegre-ainda-sonha-com-primeiro-jogo-da-selecao-brasileira-cmt7r6ipv00br015gysntaz4r.html</t>
+          <t>https://www.mktesportivo.com/2026/08/copa-do-mundo-2027-chega-ao-brasil-com-meta-de-lucro-e-maior-interesse-comercial/</t>
         </is>
       </c>
       <c r="G59" s="23" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Positivo</t>
         </is>
       </c>
       <c r="H59" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I59" s="23" t="inlineStr">
         <is>
-          <t>Sem jogos do Brasil previstos no Beira-Rio durante a Copa Feminina 2027, Porto Alegre tenta receber pela primeira vez a Seleção Feminina em um amistoso preparatório. A CBF confirmou que a capital nunca sediou partida da equipe, e ainda há cinco janelas internacionais antes do Mundial.</t>
+          <t>Em entrevista, Gal Barradas, executiva da FIFA para receitas, marketing e inteligência de negócios da Copa Feminina 2027, afirmou que a entidade projeta a primeira edição lucrativa da história do torneio. O mercado brasileiro, o fuso favorável à audiência internacional e o interesse de marcas sustentam a expectativa comercial.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="33" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="B60" s="23" t="inlineStr">
         <is>
-          <t>CBF ajusta calendário para preservar mandos dos clubes durante a Copa 2027</t>
+          <t>Porto Alegre busca amistoso da Seleção antes da Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C60" s="23" t="inlineStr">
         <is>
-          <t>Calendário / estádios / EVT-0077</t>
+          <t>Seleção Brasileira / preparação / Porto Alegre</t>
         </is>
       </c>
       <c r="D60" s="23" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="E60" s="23" t="inlineStr">
         <is>
-          <t>UOL</t>
+          <t>GZH</t>
         </is>
       </c>
       <c r="F60" s="23" t="inlineStr">
         <is>
-          <t>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/cbf-garante-solucao-para-clubes-nao-perderem-mandos-na-copa-feminina.ghtm</t>
+          <t>https://gauchazh.clicrbs.com.br/esportes/futebol-feminino/noticia/2026/08/uma-das-sedes-da-copa-do-mundo-feminina-de-2027-porto-alegre-ainda-sonha-com-primeiro-jogo-da-selecao-brasileira-cmt7r6ipv00br015gysntaz4r.html</t>
         </is>
       </c>
       <c r="G60" s="23" t="inlineStr">
         <is>
-          <t>Positivo</t>
+          <t>Neutro</t>
         </is>
       </c>
       <c r="H60" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I60" s="23" t="inlineStr">
         <is>
-          <t>Em desdobramento do período de uso exclusivo dos estádios — incluindo o início da entrega do Maracanã em 10/06/2027, registrado no EVT-0077 — a CBF trabalha para acomodar no calendário os 14 dias anteriores à Copa Feminina 2027 e evitar que clubes percam mandos, receitas ou precisem atuar longe de casa.</t>
+          <t>Sem jogos do Brasil previstos no Beira-Rio durante a Copa Feminina 2027, Porto Alegre tenta receber pela primeira vez a Seleção Feminina em um amistoso preparatório. A CBF confirmou que a capital nunca sediou partida da equipe, e ainda há cinco janelas internacionais antes do Mundial.</t>
         </is>
       </c>
     </row>
@@ -32721,27 +32721,27 @@
       </c>
       <c r="B61" s="23" t="inlineStr">
         <is>
-          <t>CBF reúne cidades-sede para alinhar operação da Copa Feminina 2027</t>
+          <t>CBF ajusta calendário para preservar mandos dos clubes durante a Copa 2027</t>
         </is>
       </c>
       <c r="C61" s="23" t="inlineStr">
         <is>
-          <t>II Workshop de Cidades-Sede / planejamento / EVT-0023</t>
+          <t>Calendário / estádios / EVT-0077</t>
         </is>
       </c>
       <c r="D61" s="23" t="inlineStr">
         <is>
-          <t>Rio de Janeiro/RJ</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E61" s="23" t="inlineStr">
         <is>
-          <t>CBF</t>
+          <t>UOL</t>
         </is>
       </c>
       <c r="F61" s="23" t="inlineStr">
         <is>
-          <t>https://www.cbf.com.br/a-cbf/noticias/por-dentro-cbf-noticias/a/rio-sedia-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-da-fifa-2027</t>
+          <t>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/cbf-garante-solucao-para-clubes-nao-perderem-mandos-na-copa-feminina.ghtm</t>
         </is>
       </c>
       <c r="G61" s="23" t="inlineStr">
@@ -32751,12 +32751,12 @@
       </c>
       <c r="H61" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I61" s="23" t="inlineStr">
         <is>
-          <t>A CBF confirmou a realização do II Workshop de Cidades-Sede e Estádios (EVT-0023), de 24 a 26 de agosto no Rio, reunindo FIFA, CBF, governos e representantes das oito sedes para alinhar temas operacionais, infraestrutura e preparação do Mundial.</t>
+          <t>Em desdobramento do período de uso exclusivo dos estádios — incluindo o início da entrega do Maracanã em 10/06/2027, registrado no EVT-0077 — a CBF trabalha para acomodar no calendário os 14 dias anteriores à Copa Feminina 2027 e evitar que clubes percam mandos, receitas ou precisem atuar longe de casa.</t>
         </is>
       </c>
     </row>
@@ -32766,27 +32766,27 @@
       </c>
       <c r="B62" s="23" t="inlineStr">
         <is>
-          <t>Elas Jogam Summit defende legado social, turístico e econômico para a Copa 2027</t>
+          <t>CBF reúne cidades-sede para alinhar operação da Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C62" s="23" t="inlineStr">
         <is>
-          <t>Elas Jogam Summit / legado / EVT-0021</t>
+          <t>II Workshop de Cidades-Sede / planejamento / EVT-0023</t>
         </is>
       </c>
       <c r="D62" s="23" t="inlineStr">
         <is>
-          <t>São Paulo/SP</t>
+          <t>Rio de Janeiro/RJ</t>
         </is>
       </c>
       <c r="E62" s="23" t="inlineStr">
         <is>
-          <t>TV Brasil</t>
+          <t>CBF</t>
         </is>
       </c>
       <c r="F62" s="23" t="inlineStr">
         <is>
-          <t>https://tvbrasil.ebc.com.br/reporter-brasil-tarde/2026/08/museu-do-futebol-sedia-evento-sobre-legado-da-copa-feminina-de-futebol</t>
+          <t>https://www.cbf.com.br/a-cbf/noticias/por-dentro-cbf-noticias/a/rio-sedia-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-da-fifa-2027</t>
         </is>
       </c>
       <c r="G62" s="23" t="inlineStr">
@@ -32801,7 +32801,7 @@
       </c>
       <c r="I62" s="23" t="inlineStr">
         <is>
-          <t>A cobertura pós-evento do Elas Jogam Summit (EVT-0021) destacou a defesa de um legado social, turístico e econômico duradouro para a Copa Feminina 2027, com estruturação da base e fortalecimento do futebol feminino profissional.</t>
+          <t>A CBF confirmou a realização do II Workshop de Cidades-Sede e Estádios (EVT-0023), de 24 a 26 de agosto no Rio, reunindo FIFA, CBF, governos e representantes das oito sedes para alinhar temas operacionais, infraestrutura e preparação do Mundial.</t>
         </is>
       </c>
     </row>
@@ -32811,27 +32811,27 @@
       </c>
       <c r="B63" s="23" t="inlineStr">
         <is>
-          <t>Fortaleza projeta aumento do turismo e da demanda por serviços com a Copa 2027</t>
+          <t>Elas Jogam Summit defende legado social, turístico e econômico para a Copa 2027</t>
         </is>
       </c>
       <c r="C63" s="23" t="inlineStr">
         <is>
-          <t>Turismo / hotelaria / economia local</t>
+          <t>Elas Jogam Summit / legado / EVT-0021</t>
         </is>
       </c>
       <c r="D63" s="23" t="inlineStr">
         <is>
-          <t>Fortaleza/CE</t>
+          <t>São Paulo/SP</t>
         </is>
       </c>
       <c r="E63" s="23" t="inlineStr">
         <is>
-          <t>TurisNews</t>
+          <t>TV Brasil</t>
         </is>
       </c>
       <c r="F63" s="23" t="inlineStr">
         <is>
-          <t>https://turisnews.com.br/fortaleza-projeta-alta-no-turismo-com-a-copa-feminina-2027/</t>
+          <t>https://tvbrasil.ebc.com.br/reporter-brasil-tarde/2026/08/museu-do-futebol-sedia-evento-sobre-legado-da-copa-feminina-de-futebol</t>
         </is>
       </c>
       <c r="G63" s="23" t="inlineStr">
@@ -32846,7 +32846,7 @@
       </c>
       <c r="I63" s="23" t="inlineStr">
         <is>
-          <t>Com nove jogos previstos no Castelão, Fortaleza projeta aumento da demanda por hotelaria, gastronomia, transporte, comércio e serviços durante a Copa Feminina 2027. A cidade recebeu 2,24 milhões de turistas no primeiro semestre de 2026, e o Visite Ceará já mapeou a rede hoteleira segundo os critérios da FIFA.</t>
+          <t>A cobertura pós-evento do Elas Jogam Summit (EVT-0021) destacou a defesa de um legado social, turístico e econômico duradouro para a Copa Feminina 2027, com estruturação da base e fortalecimento do futebol feminino profissional.</t>
         </is>
       </c>
     </row>
@@ -32856,12 +32856,12 @@
       </c>
       <c r="B64" s="23" t="inlineStr">
         <is>
-          <t>Sebrae e Sesporte articulam programa de sustentabilidade para o Castelão na Copa 2027</t>
+          <t>Fortaleza projeta aumento do turismo e da demanda por serviços com a Copa 2027</t>
         </is>
       </c>
       <c r="C64" s="23" t="inlineStr">
         <is>
-          <t>Sustentabilidade / Fortaleza</t>
+          <t>Turismo / hotelaria / economia local</t>
         </is>
       </c>
       <c r="D64" s="23" t="inlineStr">
@@ -32871,12 +32871,12 @@
       </c>
       <c r="E64" s="23" t="inlineStr">
         <is>
-          <t>Agência Sebrae de Notícias</t>
+          <t>TurisNews</t>
         </is>
       </c>
       <c r="F64" s="23" t="inlineStr">
         <is>
-          <t>https://ce.agenciasebrae.com.br/cultura-empreendedora/sebrae-ce-e-sesporte-discutem-acoes-na-area-da-sustentabilidade/</t>
+          <t>https://turisnews.com.br/fortaleza-projeta-alta-no-turismo-com-a-copa-feminina-2027/</t>
         </is>
       </c>
       <c r="G64" s="23" t="inlineStr">
@@ -32891,7 +32891,7 @@
       </c>
       <c r="I64" s="23" t="inlineStr">
         <is>
-          <t>Sebrae/CE e Secretaria do Esporte do Ceará iniciaram diálogo para implementar o programa de sustentabilidade e responsabilidade social exigido pela FIFA na Arena Castelão, sede da Copa Feminina 2027, com participação da comunidade e dos pequenos negócios do entorno.</t>
+          <t>Com nove jogos previstos no Castelão, Fortaleza projeta aumento da demanda por hotelaria, gastronomia, transporte, comércio e serviços durante a Copa Feminina 2027. A cidade recebeu 2,24 milhões de turistas no primeiro semestre de 2026, e o Visite Ceará já mapeou a rede hoteleira segundo os critérios da FIFA.</t>
         </is>
       </c>
     </row>
@@ -32901,27 +32901,27 @@
       </c>
       <c r="B65" s="23" t="inlineStr">
         <is>
-          <t>Sorteio da Copa Feminina 2027 será em 11 de dezembro no MAM Rio</t>
+          <t>Sebrae e Sesporte articulam programa de sustentabilidade para o Castelão na Copa 2027</t>
         </is>
       </c>
       <c r="C65" s="23" t="inlineStr">
         <is>
-          <t>Sorteio / calendário / EVT-0010</t>
+          <t>Sustentabilidade / Fortaleza</t>
         </is>
       </c>
       <c r="D65" s="23" t="inlineStr">
         <is>
-          <t>Rio de Janeiro/RJ</t>
+          <t>Fortaleza/CE</t>
         </is>
       </c>
       <c r="E65" s="23" t="inlineStr">
         <is>
-          <t>UOL</t>
+          <t>Agência Sebrae de Notícias</t>
         </is>
       </c>
       <c r="F65" s="23" t="inlineStr">
         <is>
-          <t>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/sorteio-da-copa-do-mundo-feminina-2027-sera-em-11-de-dezembro-no-mam-rio.ghtm</t>
+          <t>https://ce.agenciasebrae.com.br/cultura-empreendedora/sebrae-ce-e-sesporte-discutem-acoes-na-area-da-sustentabilidade/</t>
         </is>
       </c>
       <c r="G65" s="23" t="inlineStr">
@@ -32931,42 +32931,42 @@
       </c>
       <c r="H65" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I65" s="23" t="inlineStr">
         <is>
-          <t>A FIFA confirmou que o sorteio final dos grupos da Copa Feminina 2027 será realizado em 11/12/2026 no Museu de Arte Moderna do Rio. O anúncio atualiza o EVT-0010 e antecipa um evento para mais de mil convidados, que definirá os grupos e o caminho das 32 seleções.</t>
+          <t>Sebrae/CE e Secretaria do Esporte do Ceará iniciaram diálogo para implementar o programa de sustentabilidade e responsabilidade social exigido pela FIFA na Arena Castelão, sede da Copa Feminina 2027, com participação da comunidade e dos pequenos negócios do entorno.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="33" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="B66" s="23" t="inlineStr">
         <is>
-          <t>Coca-Cola confirma patrocínio e prepara presença de peso na Copa Feminina 2027</t>
+          <t>Sorteio da Copa Feminina 2027 será em 11 de dezembro no MAM Rio</t>
         </is>
       </c>
       <c r="C66" s="23" t="inlineStr">
         <is>
-          <t>Patrocínio / negócios</t>
+          <t>Sorteio / calendário / EVT-0010</t>
         </is>
       </c>
       <c r="D66" s="23" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Rio de Janeiro/RJ</t>
         </is>
       </c>
       <c r="E66" s="23" t="inlineStr">
         <is>
-          <t>Exame</t>
+          <t>UOL</t>
         </is>
       </c>
       <c r="F66" s="23" t="inlineStr">
         <is>
-          <t>https://exame.com/negocios/vamos-patrocinar-a-copa-do-mundo-feminina-2027-diz-presidente-da-coca-cola-brasil/</t>
+          <t>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/sorteio-da-copa-do-mundo-feminina-2027-sera-em-11-de-dezembro-no-mam-rio.ghtm</t>
         </is>
       </c>
       <c r="G66" s="23" t="inlineStr">
@@ -32981,7 +32981,7 @@
       </c>
       <c r="I66" s="23" t="inlineStr">
         <is>
-          <t>A presidente da Coca-Cola Brasil confirmou que a companhia patrocinará a Copa do Mundo Feminina 2027 no Brasil e pretende ter presença comparável à adotada no Mundial masculino. A empresa prepara ativações para o torneio e ampliou sua atuação no futebol nacional por meio de novos acordos com a CBF.</t>
+          <t>A FIFA confirmou que o sorteio final dos grupos da Copa Feminina 2027 será realizado em 11/12/2026 no Museu de Arte Moderna do Rio. O anúncio atualiza o EVT-0010 e antecipa um evento para mais de mil convidados, que definirá os grupos e o caminho das 32 seleções.</t>
         </is>
       </c>
     </row>
@@ -32991,27 +32991,27 @@
       </c>
       <c r="B67" s="23" t="inlineStr">
         <is>
-          <t>Rio envia à Alerj projeto de isenção de ICMS para a Copa Feminina 2027</t>
+          <t>Coca-Cola confirma patrocínio e prepara presença de peso na Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C67" s="23" t="inlineStr">
         <is>
-          <t>Tributação / organização / políticas públicas</t>
+          <t>Patrocínio / negócios</t>
         </is>
       </c>
       <c r="D67" s="23" t="inlineStr">
         <is>
-          <t>Rio de Janeiro/RJ</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E67" s="23" t="inlineStr">
         <is>
-          <t>Governo do Estado do Rio de Janeiro</t>
+          <t>Exame</t>
         </is>
       </c>
       <c r="F67" s="23" t="inlineStr">
         <is>
-          <t>https://www.rj.gov.br/radioroquettepinto/node/20221</t>
+          <t>https://exame.com/negocios/vamos-patrocinar-a-copa-do-mundo-feminina-2027-diz-presidente-da-coca-cola-brasil/</t>
         </is>
       </c>
       <c r="G67" s="23" t="inlineStr">
@@ -33026,37 +33026,37 @@
       </c>
       <c r="I67" s="23" t="inlineStr">
         <is>
-          <t>O Governo do Rio encaminhou à Alerj projeto para incorporar à legislação estadual a isenção e a suspensão de ICMS previstas pelo Confaz em operações e prestações ligadas à organização da Copa Feminina 2027. A proposta, protocolada em 21/08, busca viabilizar a desoneração tributária das atividades do torneio no estado.</t>
+          <t>A presidente da Coca-Cola Brasil confirmou que a companhia patrocinará a Copa do Mundo Feminina 2027 no Brasil e pretende ter presença comparável à adotada no Mundial masculino. A empresa prepara ativações para o torneio e ampliou sua atuação no futebol nacional por meio de novos acordos com a CBF.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="33" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="B68" s="23" t="inlineStr">
         <is>
-          <t>Copa Salvador Interbairros amplia participação feminina e premia campeãs com R$ 40 mil</t>
+          <t>Rio envia à Alerj projeto de isenção de ICMS para a Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C68" s="23" t="inlineStr">
         <is>
-          <t>Copa Salvador Interbairros / legado / EVT-0064</t>
+          <t>Tributação / organização / políticas públicas</t>
         </is>
       </c>
       <c r="D68" s="23" t="inlineStr">
         <is>
-          <t>Salvador/BA</t>
+          <t>Rio de Janeiro/RJ</t>
         </is>
       </c>
       <c r="E68" s="23" t="inlineStr">
         <is>
-          <t>Correio</t>
+          <t>Governo do Estado do Rio de Janeiro</t>
         </is>
       </c>
       <c r="F68" s="23" t="inlineStr">
         <is>
-          <t>https://www.correio24horas.com.br/salvador/copa-salvador-interbairros-2026-tera-r-40-mil-para-campeoes-e-comeca-dia-30-veja-novidades-0826</t>
+          <t>https://www.rj.gov.br/radioroquettepinto/node/20221</t>
         </is>
       </c>
       <c r="G68" s="23" t="inlineStr">
@@ -33066,42 +33066,42 @@
       </c>
       <c r="H68" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I68" s="23" t="inlineStr">
         <is>
-          <t>A Copa Salvador Interbairros (EVT-0064) reunirá cerca de 1,2 mil atletas, incluindo dez equipes femininas, e distribuirá R$ 40 mil aos campeões das categorias Livre masculina e feminina. A Prefeitura apresenta a competição como legado comunitário para a Copa 2027.</t>
+          <t>O Governo do Rio encaminhou à Alerj projeto para incorporar à legislação estadual a isenção e a suspensão de ICMS previstas pelo Confaz em operações e prestações ligadas à organização da Copa Feminina 2027. A proposta, protocolada em 21/08, busca viabilizar a desoneração tributária das atividades do torneio no estado.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="33" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="B69" s="23" t="inlineStr">
         <is>
-          <t>Elas Jogam Summit reúne atletas e especialistas para discutir o legado da Copa 2027</t>
+          <t>Copa Salvador Interbairros amplia participação feminina e premia campeãs com R$ 40 mil</t>
         </is>
       </c>
       <c r="C69" s="23" t="inlineStr">
         <is>
-          <t>Elas Jogam Summit / legado</t>
+          <t>Copa Salvador Interbairros / legado / EVT-0064</t>
         </is>
       </c>
       <c r="D69" s="23" t="inlineStr">
         <is>
-          <t>São Paulo/SP</t>
+          <t>Salvador/BA</t>
         </is>
       </c>
       <c r="E69" s="23" t="inlineStr">
         <is>
-          <t>Folha de S.Paulo</t>
+          <t>Correio</t>
         </is>
       </c>
       <c r="F69" s="23" t="inlineStr">
         <is>
-          <t>https://www1.folha.uol.com.br/colunas/monicabergamo/2026/08/tamires-fala-sobre-copa-do-mundo-feminina-de-2027-no-museu-do-futebol.shtml</t>
+          <t>https://www.correio24horas.com.br/salvador/copa-salvador-interbairros-2026-tera-r-40-mil-para-campeoes-e-comeca-dia-30-veja-novidades-0826</t>
         </is>
       </c>
       <c r="G69" s="23" t="inlineStr">
@@ -33116,37 +33116,37 @@
       </c>
       <c r="I69" s="23" t="inlineStr">
         <is>
-          <t>A cobertura antecipou o Elas Jogam Summit no Museu do Futebol, destacando debates sobre formação, comunicação, mercado, investimento, memória e transformação social como parte do legado da Copa Feminina 2027, além de uma oficina para meninas da periferia de São Paulo.</t>
+          <t>A Copa Salvador Interbairros (EVT-0064) reunirá cerca de 1,2 mil atletas, incluindo dez equipes femininas, e distribuirá R$ 40 mil aos campeões das categorias Livre masculina e feminina. A Prefeitura apresenta a competição como legado comunitário para a Copa 2027.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="33" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="B70" s="23" t="inlineStr">
         <is>
-          <t>Arthur Elias diz que Seleção está 70% definida e vê vantagem na abertura no Maracanã</t>
+          <t>Elas Jogam Summit reúne atletas e especialistas para discutir o legado da Copa 2027</t>
         </is>
       </c>
       <c r="C70" s="23" t="inlineStr">
         <is>
-          <t>Seleção Brasileira / preparação</t>
+          <t>Elas Jogam Summit / legado</t>
         </is>
       </c>
       <c r="D70" s="23" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>São Paulo/SP</t>
         </is>
       </c>
       <c r="E70" s="23" t="inlineStr">
         <is>
-          <t>ge</t>
+          <t>Folha de S.Paulo</t>
         </is>
       </c>
       <c r="F70" s="23" t="inlineStr">
         <is>
-          <t>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/20/arthur-elias-diz-que-selecao-esta-70percent-fechada-para-a-copa-e-que-marta-tem-ano-desafiador.ghtml</t>
+          <t>https://www1.folha.uol.com.br/colunas/monicabergamo/2026/08/tamires-fala-sobre-copa-do-mundo-feminina-de-2027-no-museu-do-futebol.shtml</t>
         </is>
       </c>
       <c r="G70" s="23" t="inlineStr">
@@ -33161,7 +33161,7 @@
       </c>
       <c r="I70" s="23" t="inlineStr">
         <is>
-          <t>Após a divulgação da tabela da Copa Feminina 2027, o técnico Arthur Elias afirmou que cerca de 70% do grupo da Seleção está definido, manteve Marta nos planos e avaliou que abrir o torneio no Maracanã representa vantagem para o Brasil.</t>
+          <t>A cobertura antecipou o Elas Jogam Summit no Museu do Futebol, destacando debates sobre formação, comunicação, mercado, investimento, memória e transformação social como parte do legado da Copa Feminina 2027, além de uma oficina para meninas da periferia de São Paulo.</t>
         </is>
       </c>
     </row>
@@ -33171,12 +33171,12 @@
       </c>
       <c r="B71" s="23" t="inlineStr">
         <is>
-          <t>FIFA abre cadastro de interesse para ingressos da Copa Feminina 2027</t>
+          <t>Arthur Elias diz que Seleção está 70% definida e vê vantagem na abertura no Maracanã</t>
         </is>
       </c>
       <c r="C71" s="23" t="inlineStr">
         <is>
-          <t>Ingressos / relacionamento</t>
+          <t>Seleção Brasileira / preparação</t>
         </is>
       </c>
       <c r="D71" s="23" t="inlineStr">
@@ -33186,17 +33186,17 @@
       </c>
       <c r="E71" s="23" t="inlineStr">
         <is>
-          <t>UOL</t>
+          <t>ge</t>
         </is>
       </c>
       <c r="F71" s="23" t="inlineStr">
         <is>
-          <t>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/20/copa-2027-venda-de-ingressos-ainda-nao-comecou-como-registrar-interesse.ghtm</t>
+          <t>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/20/arthur-elias-diz-que-selecao-esta-70percent-fechada-para-a-copa-e-que-marta-tem-ano-desafiador.ghtml</t>
         </is>
       </c>
       <c r="G71" s="23" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Positivo</t>
         </is>
       </c>
       <c r="H71" s="23" t="inlineStr">
@@ -33206,7 +33206,7 @@
       </c>
       <c r="I71" s="23" t="inlineStr">
         <is>
-          <t>A venda de ingressos ainda não começou e não há data oficial de abertura; torcedores já podem registrar interesse no portal da FIFA para receber atualizações.</t>
+          <t>Após a divulgação da tabela da Copa Feminina 2027, o técnico Arthur Elias afirmou que cerca de 70% do grupo da Seleção está definido, manteve Marta nos planos e avaliou que abrir o torneio no Maracanã representa vantagem para o Brasil.</t>
         </is>
       </c>
     </row>
@@ -33216,12 +33216,12 @@
       </c>
       <c r="B72" s="23" t="inlineStr">
         <is>
-          <t>FIFA divulga tabela-base da Copa 2027 e confirma Maracanã na abertura e final</t>
+          <t>FIFA abre cadastro de interesse para ingressos da Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C72" s="23" t="inlineStr">
         <is>
-          <t>Calendário / sedes</t>
+          <t>Ingressos / relacionamento</t>
         </is>
       </c>
       <c r="D72" s="23" t="inlineStr">
@@ -33231,27 +33231,27 @@
       </c>
       <c r="E72" s="23" t="inlineStr">
         <is>
-          <t>FIFA</t>
+          <t>UOL</t>
         </is>
       </c>
       <c r="F72" s="23" t="inlineStr">
         <is>
-          <t>https://www.fifa.com/pt/articles/tabela-jogos-copa-feminina-divulgacao-maracana-final-abertura</t>
+          <t>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/20/copa-2027-venda-de-ingressos-ainda-nao-comecou-como-registrar-interesse.ghtm</t>
         </is>
       </c>
       <c r="G72" s="23" t="inlineStr">
         <is>
-          <t>Positivo</t>
+          <t>Neutro</t>
         </is>
       </c>
       <c r="H72" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I72" s="23" t="inlineStr">
         <is>
-          <t>Tabela-base confirma 64 jogos entre 24/06 e 25/07/2027, abertura e final no Maracanã e partidas do Brasil no Rio, em São Paulo e em Brasília.</t>
+          <t>A venda de ingressos ainda não começou e não há data oficial de abertura; torcedores já podem registrar interesse no portal da FIFA para receber atualizações.</t>
         </is>
       </c>
     </row>
@@ -33261,12 +33261,12 @@
       </c>
       <c r="B73" s="23" t="inlineStr">
         <is>
-          <t>Governo prevê aporte mínimo de R$ 1,5 bilhão para organizar a Copa Feminina 2027</t>
+          <t>FIFA divulga tabela-base da Copa 2027 e confirma Maracanã na abertura e final</t>
         </is>
       </c>
       <c r="C73" s="23" t="inlineStr">
         <is>
-          <t>Investimentos públicos / segurança / infraestrutura</t>
+          <t>Calendário / sedes</t>
         </is>
       </c>
       <c r="D73" s="23" t="inlineStr">
@@ -33276,17 +33276,17 @@
       </c>
       <c r="E73" s="23" t="inlineStr">
         <is>
-          <t>Folha de S.Paulo</t>
+          <t>FIFA</t>
         </is>
       </c>
       <c r="F73" s="23" t="inlineStr">
         <is>
-          <t>https://www1.folha.uol.com.br/esporte/2026/08/brasil-joga-na-fase-de-grupos-da-copa-feminina-em-sao-paulo-rio-e-brasilia.shtml</t>
+          <t>https://www.fifa.com/pt/articles/tabela-jogos-copa-feminina-divulgacao-maracana-final-abertura</t>
         </is>
       </c>
       <c r="G73" s="23" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Positivo</t>
         </is>
       </c>
       <c r="H73" s="23" t="inlineStr">
@@ -33296,7 +33296,7 @@
       </c>
       <c r="I73" s="23" t="inlineStr">
         <is>
-          <t>Ao detalhar o calendário e o caminho da Seleção na Copa Feminina 2027, a Folha informou que o governo federal estima aporte mínimo de R$ 1,5 bilhão. Os recursos devem atender segurança pública, telecomunicações, promoção do torneio e construção do legado nas oito cidades-sede.</t>
+          <t>Tabela-base confirma 64 jogos entre 24/06 e 25/07/2027, abertura e final no Maracanã e partidas do Brasil no Rio, em São Paulo e em Brasília.</t>
         </is>
       </c>
     </row>
@@ -33306,12 +33306,12 @@
       </c>
       <c r="B74" s="23" t="inlineStr">
         <is>
-          <t>Sorteio define caminhos da fase preliminar da repescagem mundial</t>
+          <t>Governo prevê aporte mínimo de R$ 1,5 bilhão para organizar a Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C74" s="23" t="inlineStr">
         <is>
-          <t>Repescagem / sorteio</t>
+          <t>Investimentos públicos / segurança / infraestrutura</t>
         </is>
       </c>
       <c r="D74" s="23" t="inlineStr">
@@ -33321,12 +33321,12 @@
       </c>
       <c r="E74" s="23" t="inlineStr">
         <is>
-          <t>FIFA</t>
+          <t>Folha de S.Paulo</t>
         </is>
       </c>
       <c r="F74" s="23" t="inlineStr">
         <is>
-          <t>https://www.fifa.com/pt/tournaments/womens/womensworldcup/brazil-2027/articles/resultados-sorteio-fase-preliminar-torneio-classificatorio-fifa-brasil-2027</t>
+          <t>https://www1.folha.uol.com.br/esporte/2026/08/brasil-joga-na-fase-de-grupos-da-copa-feminina-em-sao-paulo-rio-e-brasilia.shtml</t>
         </is>
       </c>
       <c r="G74" s="23" t="inlineStr">
@@ -33341,27 +33341,27 @@
       </c>
       <c r="I74" s="23" t="inlineStr">
         <is>
-          <t>FIFA definiu a ordem dos confrontos entre Uzbequistão, África do Sul, Papua-Nova Guiné, Taipé Chinês, Gana e Equador; a fase será disputada de 24/11 a 05/12/2026.</t>
+          <t>Ao detalhar o calendário e o caminho da Seleção na Copa Feminina 2027, a Folha informou que o governo federal estima aporte mínimo de R$ 1,5 bilhão. Os recursos devem atender segurança pública, telecomunicações, promoção do torneio e construção do legado nas oito cidades-sede.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="33" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="B75" s="23" t="inlineStr">
         <is>
-          <t>Brasil confirma convocadas para a Copa do Mundo Feminina Sub-20</t>
+          <t>Sorteio define caminhos da fase preliminar da repescagem mundial</t>
         </is>
       </c>
       <c r="C75" s="23" t="inlineStr">
         <is>
-          <t>Seleções de Base / Sub-20 Feminina</t>
+          <t>Repescagem / sorteio</t>
         </is>
       </c>
       <c r="D75" s="23" t="inlineStr">
         <is>
-          <t>Brasil / Polônia</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E75" s="23" t="inlineStr">
@@ -33371,22 +33371,22 @@
       </c>
       <c r="F75" s="23" t="inlineStr">
         <is>
-          <t>https://www.fifa.com/pt/articles/brasil-convocadas-copa-do-mundo-feminina-sub-20-2026</t>
+          <t>https://www.fifa.com/pt/tournaments/womens/womensworldcup/brazil-2027/articles/resultados-sorteio-fase-preliminar-torneio-classificatorio-fifa-brasil-2027</t>
         </is>
       </c>
       <c r="G75" s="23" t="inlineStr">
         <is>
-          <t>Positivo</t>
+          <t>Neutro</t>
         </is>
       </c>
       <c r="H75" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I75" s="23" t="inlineStr">
         <is>
-          <t>A lista brasileira para o Mundial Feminino Sub-20 de 2026 foi confirmada. A equipe de Camilla Orlando se apresenta antes do embarque e estreia contra a Tanzânia em 5 de setembro, seguida por Canadá e Inglaterra.</t>
+          <t>FIFA definiu a ordem dos confrontos entre Uzbequistão, África do Sul, Papua-Nova Guiné, Taipé Chinês, Gana e Equador; a fase será disputada de 24/11 a 05/12/2026.</t>
         </is>
       </c>
     </row>
@@ -33396,42 +33396,42 @@
       </c>
       <c r="B76" s="23" t="inlineStr">
         <is>
-          <t>CNE limita férias escolares da Copa Feminina 2027 às cidades-sede e vizinhas</t>
+          <t>Brasil confirma convocadas para a Copa do Mundo Feminina Sub-20</t>
         </is>
       </c>
       <c r="C76" s="23" t="inlineStr">
         <is>
-          <t>Políticas públicas / educação</t>
+          <t>Seleções de Base / Sub-20 Feminina</t>
         </is>
       </c>
       <c r="D76" s="23" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Brasil / Polônia</t>
         </is>
       </c>
       <c r="E76" s="23" t="inlineStr">
         <is>
-          <t>UOL</t>
+          <t>FIFA</t>
         </is>
       </c>
       <c r="F76" s="23" t="inlineStr">
         <is>
-          <t>https://educacao.uol.com.br/noticias/2026/08/19/conselho-ferias-copa-do-mundo-futebol-feminina.ghtm</t>
+          <t>https://www.fifa.com/pt/articles/brasil-convocadas-copa-do-mundo-feminina-sub-20-2026</t>
         </is>
       </c>
       <c r="G76" s="23" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Positivo</t>
         </is>
       </c>
       <c r="H76" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I76" s="23" t="inlineStr">
         <is>
-          <t>O Conselho Nacional de Educação decidiu que a obrigação de férias durante a Copa Feminina 2027 deve alcançar somente as oito cidades-sede e municípios vizinhos; o parecer ainda depende de homologação do Ministério da Educação e afeta o planejamento do ano letivo.</t>
+          <t>A lista brasileira para o Mundial Feminino Sub-20 de 2026 foi confirmada. A equipe de Camilla Orlando se apresenta antes do embarque e estreia contra a Tanzânia em 5 de setembro, seguida por Canadá e Inglaterra.</t>
         </is>
       </c>
     </row>
@@ -33441,12 +33441,12 @@
       </c>
       <c r="B77" s="23" t="inlineStr">
         <is>
-          <t>Supermercados entram no planejamento comercial para a Copa Feminina 2027</t>
+          <t>CNE limita férias escolares da Copa Feminina 2027 às cidades-sede e vizinhas</t>
         </is>
       </c>
       <c r="C77" s="23" t="inlineStr">
         <is>
-          <t>Varejo / consumo / oportunidades comerciais</t>
+          <t>Políticas públicas / educação</t>
         </is>
       </c>
       <c r="D77" s="23" t="inlineStr">
@@ -33456,57 +33456,57 @@
       </c>
       <c r="E77" s="23" t="inlineStr">
         <is>
-          <t>Revista Super Negócios / ASSERJ</t>
+          <t>UOL</t>
         </is>
       </c>
       <c r="F77" s="23" t="inlineStr">
         <is>
-          <t>https://asserj.com.br/en/w/copa-do-mundo-feminina-entra-no-radar-dos-supermercados</t>
+          <t>https://educacao.uol.com.br/noticias/2026/08/19/conselho-ferias-copa-do-mundo-futebol-feminina.ghtm</t>
         </is>
       </c>
       <c r="G77" s="23" t="inlineStr">
         <is>
-          <t>Positivo</t>
+          <t>Neutro</t>
         </is>
       </c>
       <c r="H77" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I77" s="23" t="inlineStr">
         <is>
-          <t>A Associação de Supermercados do Estado do Rio de Janeiro aponta a Copa Feminina 2027 como oportunidade para o varejo alimentar, com foco no consumo doméstico e familiar, cestas mais diversificadas e ativações comerciais. A análise cita 750 mil interessados em ingressos e a projeção de R$ 8,8 bilhões movimentados pelo torneio.</t>
+          <t>O Conselho Nacional de Educação decidiu que a obrigação de férias durante a Copa Feminina 2027 deve alcançar somente as oito cidades-sede e municípios vizinhos; o parecer ainda depende de homologação do Ministério da Educação e afeta o planejamento do ano letivo.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="33" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="B78" s="23" t="inlineStr">
         <is>
-          <t>Painel em Brasília defende estrutura duradoura como legado da Copa 2027</t>
+          <t>Supermercados entram no planejamento comercial para a Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C78" s="23" t="inlineStr">
         <is>
-          <t>Elas em Ação / legado / EVT-0081</t>
+          <t>Varejo / consumo / oportunidades comerciais</t>
         </is>
       </c>
       <c r="D78" s="23" t="inlineStr">
         <is>
-          <t>Brasília/DF</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E78" s="23" t="inlineStr">
         <is>
-          <t>FSports</t>
+          <t>Revista Super Negócios / ASSERJ</t>
         </is>
       </c>
       <c r="F78" s="23" t="inlineStr">
         <is>
-          <t>https://pt.linkedin.com/posts/fsports-ag_o-legado-come%C3%A7a-antes-do-primeiro-apito-activity-7495445214967484417-5m11</t>
+          <t>https://asserj.com.br/en/w/copa-do-mundo-feminina-entra-no-radar-dos-supermercados</t>
         </is>
       </c>
       <c r="G78" s="23" t="inlineStr">
@@ -33521,37 +33521,37 @@
       </c>
       <c r="I78" s="23" t="inlineStr">
         <is>
-          <t>No painel “Esporte como Arena de Poder” do Elas em Ação (EVT-0081), Juliana Picoli Agatte e Ruskaya Zanini defenderam que a Copa Feminina 2027 deixe estrutura para clubes e atletas, amplie a participação de meninas, mantenha marcas investindo e coloque mais mulheres em posições de decisão.</t>
+          <t>A Associação de Supermercados do Estado do Rio de Janeiro aponta a Copa Feminina 2027 como oportunidade para o varejo alimentar, com foco no consumo doméstico e familiar, cestas mais diversificadas e ativações comerciais. A análise cita 750 mil interessados em ingressos e a projeção de R$ 8,8 bilhões movimentados pelo torneio.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="33" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="B79" s="23" t="inlineStr">
         <is>
-          <t>Brasil convoca Seleção Feminina Sub-15 para a Liga Evolução</t>
+          <t>Painel em Brasília defende estrutura duradoura como legado da Copa 2027</t>
         </is>
       </c>
       <c r="C79" s="23" t="inlineStr">
         <is>
-          <t>Seleções de Base / Sub-15 Feminina</t>
+          <t>Elas em Ação / legado / EVT-0081</t>
         </is>
       </c>
       <c r="D79" s="23" t="inlineStr">
         <is>
-          <t>Assunção/PRY</t>
+          <t>Brasília/DF</t>
         </is>
       </c>
       <c r="E79" s="23" t="inlineStr">
         <is>
-          <t>CBF</t>
+          <t>FSports</t>
         </is>
       </c>
       <c r="F79" s="23" t="inlineStr">
         <is>
-          <t>https://www.cbf.com.br/selecao-brasileira/noticias/convocacoes-selecao-feminina-sub-15/a/beatriz-vaz-convoca-20-atletas-para-liga-evolucao-sub-15-da-conmebol</t>
+          <t>https://pt.linkedin.com/posts/fsports-ag_o-legado-come%C3%A7a-antes-do-primeiro-apito-activity-7495445214967484417-5m11</t>
         </is>
       </c>
       <c r="G79" s="23" t="inlineStr">
@@ -33566,7 +33566,7 @@
       </c>
       <c r="I79" s="23" t="inlineStr">
         <is>
-          <t>Bia Vaz convocou 20 atletas para defender a Seleção Brasileira Feminina Sub-15 na Liga Evolução da CONMEBOL, de 8 a 20 de setembro no Paraguai, em busca do bicampeonato.</t>
+          <t>No painel “Esporte como Arena de Poder” do Elas em Ação (EVT-0081), Juliana Picoli Agatte e Ruskaya Zanini defenderam que a Copa Feminina 2027 deixe estrutura para clubes e atletas, amplie a participação de meninas, mantenha marcas investindo e coloque mais mulheres em posições de decisão.</t>
         </is>
       </c>
     </row>
@@ -33576,27 +33576,27 @@
       </c>
       <c r="B80" s="23" t="inlineStr">
         <is>
-          <t>FIFA e FPF alinham preparativos da Copa do Mundo Feminina</t>
+          <t>Brasil convoca Seleção Feminina Sub-15 para a Liga Evolução</t>
         </is>
       </c>
       <c r="C80" s="23" t="inlineStr">
         <is>
-          <t>Operação / cidade-sede</t>
+          <t>Seleções de Base / Sub-15 Feminina</t>
         </is>
       </c>
       <c r="D80" s="23" t="inlineStr">
         <is>
-          <t>Recife/PE</t>
+          <t>Assunção/PRY</t>
         </is>
       </c>
       <c r="E80" s="23" t="inlineStr">
         <is>
-          <t>Tribuna Online</t>
+          <t>CBF</t>
         </is>
       </c>
       <c r="F80" s="23" t="inlineStr">
         <is>
-          <t>https://tribunaonline.com.br/pernambuco/esporte/fpf-recebe-comitiva-da-fifa-para-alinhar-preparativos-da-copa-do-mundo-feminina-328649</t>
+          <t>https://www.cbf.com.br/selecao-brasileira/noticias/convocacoes-selecao-feminina-sub-15/a/beatriz-vaz-convoca-20-atletas-para-liga-evolucao-sub-15-da-conmebol</t>
         </is>
       </c>
       <c r="G80" s="23" t="inlineStr">
@@ -33606,12 +33606,12 @@
       </c>
       <c r="H80" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I80" s="23" t="inlineStr">
         <is>
-          <t>Reunião institucional reforçou integração da sede pernambucana com as áreas responsáveis pela organização do Mundial.</t>
+          <t>Bia Vaz convocou 20 atletas para defender a Seleção Brasileira Feminina Sub-15 na Liga Evolução da CONMEBOL, de 8 a 20 de setembro no Paraguai, em busca do bicampeonato.</t>
         </is>
       </c>
     </row>
@@ -33621,72 +33621,72 @@
       </c>
       <c r="B81" s="23" t="inlineStr">
         <is>
-          <t>Tamires cobra mobilização das cidades-sede para lotar a Copa Feminina 2027</t>
+          <t>FIFA e FPF alinham preparativos da Copa do Mundo Feminina</t>
         </is>
       </c>
       <c r="C81" s="23" t="inlineStr">
         <is>
-          <t>Elas Jogam Summit / público / legado / EVT-0021</t>
+          <t>Operação / cidade-sede</t>
         </is>
       </c>
       <c r="D81" s="23" t="inlineStr">
         <is>
-          <t>São Paulo/SP</t>
+          <t>Recife/PE</t>
         </is>
       </c>
       <c r="E81" s="23" t="inlineStr">
         <is>
-          <t>UOL</t>
+          <t>Tribuna Online</t>
         </is>
       </c>
       <c r="F81" s="23" t="inlineStr">
         <is>
-          <t>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/17/copa-2027-tamires-pede-engajamento-das-cidades-sede-para-lotar-estadios.ghtm</t>
+          <t>https://tribunaonline.com.br/pernambuco/esporte/fpf-recebe-comitiva-da-fifa-para-alinhar-preparativos-da-copa-do-mundo-feminina-328649</t>
         </is>
       </c>
       <c r="G81" s="23" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Positivo</t>
         </is>
       </c>
       <c r="H81" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I81" s="23" t="inlineStr">
         <is>
-          <t>Em entrevista durante evento em São Paulo ligado ao debate de legado do Elas Jogam Summit (EVT-0021), Tamires defendeu estratégias locais nas oito cidades-sede para encher os 64 jogos da Copa Feminina 2027. A FIFA pretende superar dois milhões de espectadores e acompanha ações de promoção, Fan Fests e centros de treinamento.</t>
+          <t>Reunião institucional reforçou integração da sede pernambucana com as áreas responsáveis pela organização do Mundial.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="33" t="n">
-        <v>46248</v>
+        <v>46251</v>
       </c>
       <c r="B82" s="23" t="inlineStr">
         <is>
-          <t>FIFA confirma evento de 20/08 para revelar calendário e sorteio da repescagem</t>
+          <t>Tamires cobra mobilização das cidades-sede para lotar a Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C82" s="23" t="inlineStr">
         <is>
-          <t>Calendário / sorteio</t>
+          <t>Elas Jogam Summit / público / legado / EVT-0021</t>
         </is>
       </c>
       <c r="D82" s="23" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>São Paulo/SP</t>
         </is>
       </c>
       <c r="E82" s="23" t="inlineStr">
         <is>
-          <t>ge</t>
+          <t>UOL</t>
         </is>
       </c>
       <c r="F82" s="23" t="inlineStr">
         <is>
-          <t>https://ge.globo.com/futebol/copa-do-mundo-feminina/noticia/2026/08/14/copa-do-mundo-2027-calendario-sera-revelado-dia-20-de-agosto.ghtml</t>
+          <t>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/17/copa-2027-tamires-pede-engajamento-das-cidades-sede-para-lotar-estadios.ghtm</t>
         </is>
       </c>
       <c r="G82" s="23" t="inlineStr">
@@ -33696,12 +33696,12 @@
       </c>
       <c r="H82" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I82" s="23" t="inlineStr">
         <is>
-          <t>Em 20/08 serão anunciados distribuição de jogos por sede, locais dos jogos do Brasil e confrontos da fase preliminar da repescagem.</t>
+          <t>Em entrevista durante evento em São Paulo ligado ao debate de legado do Elas Jogam Summit (EVT-0021), Tamires defendeu estratégias locais nas oito cidades-sede para encher os 64 jogos da Copa Feminina 2027. A FIFA pretende superar dois milhões de espectadores e acompanha ações de promoção, Fan Fests e centros de treinamento.</t>
         </is>
       </c>
     </row>
@@ -33711,32 +33711,32 @@
       </c>
       <c r="B83" s="23" t="inlineStr">
         <is>
-          <t>FIFA reúne marcas no SP2B para discutir ativações da Copa 2027</t>
+          <t>FIFA confirma evento de 20/08 para revelar calendário e sorteio da repescagem</t>
         </is>
       </c>
       <c r="C83" s="23" t="inlineStr">
         <is>
-          <t>Patrocínio / ativações</t>
+          <t>Calendário / sorteio</t>
         </is>
       </c>
       <c r="D83" s="23" t="inlineStr">
         <is>
-          <t>São Paulo/SP</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E83" s="23" t="inlineStr">
         <is>
-          <t>UOL</t>
+          <t>ge</t>
         </is>
       </c>
       <c r="F83" s="23" t="inlineStr">
         <is>
-          <t>https://economia.uol.com.br/noticias/redacao/2026/08/14/copa-do-mundo-feminina-alcanca-750-mil-interessados-em-ingressos.ghtm</t>
+          <t>https://ge.globo.com/futebol/copa-do-mundo-feminina/noticia/2026/08/14/copa-do-mundo-2027-calendario-sera-revelado-dia-20-de-agosto.ghtml</t>
         </is>
       </c>
       <c r="G83" s="23" t="inlineStr">
         <is>
-          <t>Positivo</t>
+          <t>Neutro</t>
         </is>
       </c>
       <c r="H83" s="23" t="inlineStr">
@@ -33746,7 +33746,7 @@
       </c>
       <c r="I83" s="23" t="inlineStr">
         <is>
-          <t>Encontro no SP2B discutiu oportunidades comerciais e estratégias de ativação com patrocinadores e executivos.</t>
+          <t>Em 20/08 serão anunciados distribuição de jogos por sede, locais dos jogos do Brasil e confrontos da fase preliminar da repescagem.</t>
         </is>
       </c>
     </row>
@@ -33756,27 +33756,27 @@
       </c>
       <c r="B84" s="23" t="inlineStr">
         <is>
-          <t>Sesc RJ amplia turmas gratuitas de futebol feminino com foco no legado da Copa 2027</t>
+          <t>FIFA reúne marcas no SP2B para discutir ativações da Copa 2027</t>
         </is>
       </c>
       <c r="C84" s="23" t="inlineStr">
         <is>
-          <t>Legado / formação de base / inclusão esportiva</t>
+          <t>Patrocínio / ativações</t>
         </is>
       </c>
       <c r="D84" s="23" t="inlineStr">
         <is>
-          <t>Diversas cidades/RJ</t>
+          <t>São Paulo/SP</t>
         </is>
       </c>
       <c r="E84" s="23" t="inlineStr">
         <is>
-          <t>Sesc RJ</t>
+          <t>UOL</t>
         </is>
       </c>
       <c r="F84" s="23" t="inlineStr">
         <is>
-          <t>https://www.sescrio.org.br/noticias/esporte/em-clima-de-copa-2027-sesc-rj-amplia-turmas-gratuitas-de-futebol-feminino/</t>
+          <t>https://economia.uol.com.br/noticias/redacao/2026/08/14/copa-do-mundo-feminina-alcanca-750-mil-interessados-em-ingressos.ghtm</t>
         </is>
       </c>
       <c r="G84" s="23" t="inlineStr">
@@ -33786,42 +33786,42 @@
       </c>
       <c r="H84" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I84" s="23" t="inlineStr">
         <is>
-          <t>Em iniciativa vinculada ao legado da Copa do Mundo Feminina 2027, o Sesc RJ ampliou as turmas gratuitas de futebol feminino para meninas de 7 a 17 anos. O projeto alcança unidades na capital e em Petrópolis, Nova Iguaçu, São João de Meriti, Niterói e São Gonçalo, com foco em acesso ao esporte, permanência na prática e formação de novas atletas.</t>
+          <t>Encontro no SP2B discutiu oportunidades comerciais e estratégias de ativação com patrocinadores e executivos.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="33" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="B85" s="23" t="inlineStr">
         <is>
-          <t>Base feminina soma 206 atletas convocadas e três desafios internacionais</t>
+          <t>Sesc RJ amplia turmas gratuitas de futebol feminino com foco no legado da Copa 2027</t>
         </is>
       </c>
       <c r="C85" s="23" t="inlineStr">
         <is>
-          <t>Seleções de Base / Sub-15, Sub-17 e Sub-20 Femininas</t>
+          <t>Legado / formação de base / inclusão esportiva</t>
         </is>
       </c>
       <c r="D85" s="23" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Diversas cidades/RJ</t>
         </is>
       </c>
       <c r="E85" s="23" t="inlineStr">
         <is>
-          <t>CBF</t>
+          <t>Sesc RJ</t>
         </is>
       </c>
       <c r="F85" s="23" t="inlineStr">
         <is>
-          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-base-feminina/a/campeas-continentais-e-mais-de-200-atletas-convocadas-conquistas-e-numeros-do-atual-ciclo-da-base-feminina</t>
+          <t>https://www.sescrio.org.br/noticias/esporte/em-clima-de-copa-2027-sesc-rj-amplia-turmas-gratuitas-de-futebol-feminino/</t>
         </is>
       </c>
       <c r="G85" s="23" t="inlineStr">
@@ -33836,22 +33836,22 @@
       </c>
       <c r="I85" s="23" t="inlineStr">
         <is>
-          <t>A CBF apresentou o balanço do ciclo das Seleções Femininas de Base: 206 atletas convocadas, 47 jogos, 32 vitórias e 68% de aproveitamento. Sub-15, Sub-17 e Sub-20 terão competições internacionais no segundo semestre de 2026.</t>
+          <t>Em iniciativa vinculada ao legado da Copa do Mundo Feminina 2027, o Sesc RJ ampliou as turmas gratuitas de futebol feminino para meninas de 7 a 17 anos. O projeto alcança unidades na capital e em Petrópolis, Nova Iguaçu, São João de Meriti, Niterói e São Gonçalo, com foco em acesso ao esporte, permanência na prática e formação de novas atletas.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="33" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="B86" s="23" t="inlineStr">
         <is>
-          <t>Atricon apoia revisão das férias escolares obrigatórias durante a Copa 2027</t>
+          <t>Base feminina soma 206 atletas convocadas e três desafios internacionais</t>
         </is>
       </c>
       <c r="C86" s="23" t="inlineStr">
         <is>
-          <t>Políticas públicas / educação</t>
+          <t>Seleções de Base / Sub-15, Sub-17 e Sub-20 Femininas</t>
         </is>
       </c>
       <c r="D86" s="23" t="inlineStr">
@@ -33861,17 +33861,17 @@
       </c>
       <c r="E86" s="23" t="inlineStr">
         <is>
-          <t>Folha de S.Paulo</t>
+          <t>CBF</t>
         </is>
       </c>
       <c r="F86" s="23" t="inlineStr">
         <is>
-          <t>https://www1.folha.uol.com.br/colunas/painel/2026/08/associacao-de-tribunais-de-contas-se-opoe-a-ferias-escolares-obrigatorias-na-copa-do-mundo-feminina.shtml</t>
+          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-base-feminina/a/campeas-continentais-e-mais-de-200-atletas-convocadas-conquistas-e-numeros-do-atual-ciclo-da-base-feminina</t>
         </is>
       </c>
       <c r="G86" s="23" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Positivo</t>
         </is>
       </c>
       <c r="H86" s="23" t="inlineStr">
@@ -33881,22 +33881,22 @@
       </c>
       <c r="I86" s="23" t="inlineStr">
         <is>
-          <t>A Atricon enviou ofícios à Câmara e ao Senado apoiando projeto que revoga a obrigatoriedade de férias escolares durante a Copa Feminina 2027, argumentando que a regra pode prejudicar calendários pedagógicos, transporte e alimentação escolar em regiões sem jogos.</t>
+          <t>A CBF apresentou o balanço do ciclo das Seleções Femininas de Base: 206 atletas convocadas, 47 jogos, 32 vitórias e 68% de aproveitamento. Sub-15, Sub-17 e Sub-20 terão competições internacionais no segundo semestre de 2026.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="33" t="n">
-        <v>46239</v>
+        <v>46246</v>
       </c>
       <c r="B87" s="23" t="inlineStr">
         <is>
-          <t>CBF determina pausa nacional durante toda a Copa Feminina 2027</t>
+          <t>Atricon apoia revisão das férias escolares obrigatórias durante a Copa 2027</t>
         </is>
       </c>
       <c r="C87" s="23" t="inlineStr">
         <is>
-          <t>Calendário / competições nacionais</t>
+          <t>Políticas públicas / educação</t>
         </is>
       </c>
       <c r="D87" s="23" t="inlineStr">
@@ -33906,12 +33906,12 @@
       </c>
       <c r="E87" s="23" t="inlineStr">
         <is>
-          <t>ge</t>
+          <t>Folha de S.Paulo</t>
         </is>
       </c>
       <c r="F87" s="23" t="inlineStr">
         <is>
-          <t>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/05/cbf-comunica-aos-clubes-parada-obrigatoria-durante-periodo-da-copa-do-mundo-feminina-de-2027.ghtml</t>
+          <t>https://www1.folha.uol.com.br/colunas/painel/2026/08/associacao-de-tribunais-de-contas-se-opoe-a-ferias-escolares-obrigatorias-na-copa-do-mundo-feminina.shtml</t>
         </is>
       </c>
       <c r="G87" s="23" t="inlineStr">
@@ -33921,12 +33921,12 @@
       </c>
       <c r="H87" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I87" s="23" t="inlineStr">
         <is>
-          <t>A CBF comunicou aos clubes que as competições masculinas e femininas terão pausa obrigatória entre 24/06 e 25/07/2027, durante toda a Copa do Mundo Feminina, enquanto a entidade ajusta o calendário nacional e a disponibilidade das oito arenas do torneio.</t>
+          <t>A Atricon enviou ofícios à Câmara e ao Senado apoiando projeto que revoga a obrigatoriedade de férias escolares durante a Copa Feminina 2027, argumentando que a regra pode prejudicar calendários pedagógicos, transporte e alimentação escolar em regiões sem jogos.</t>
         </is>
       </c>
     </row>
@@ -33936,42 +33936,42 @@
       </c>
       <c r="B88" s="23" t="inlineStr">
         <is>
-          <t>Elas Jogam Summit propõe ações para construir o legado da Copa Feminina 2027</t>
+          <t>CBF determina pausa nacional durante toda a Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C88" s="23" t="inlineStr">
         <is>
-          <t>Elas Jogam Summit / legado</t>
+          <t>Calendário / competições nacionais</t>
         </is>
       </c>
       <c r="D88" s="23" t="inlineStr">
         <is>
-          <t>São Paulo/SP</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E88" s="23" t="inlineStr">
         <is>
-          <t>Donas FC</t>
+          <t>ge</t>
         </is>
       </c>
       <c r="F88" s="23" t="inlineStr">
         <is>
-          <t>https://donasfc.com.br/2026/08/05/elas-jogam-summit-discutira-o-legado-da-copa-do-mundo-feminina-2027-em-evento-no-pacaembu/</t>
+          <t>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/05/cbf-comunica-aos-clubes-parada-obrigatoria-durante-periodo-da-copa-do-mundo-feminina-de-2027.ghtml</t>
         </is>
       </c>
       <c r="G88" s="23" t="inlineStr">
         <is>
-          <t>Positivo</t>
+          <t>Neutro</t>
         </is>
       </c>
       <c r="H88" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I88" s="23" t="inlineStr">
         <is>
-          <t>A matéria apresentou o Elas Jogam Summit e sua proposta de transformar a Copa Feminina 2027 em legado por meio de políticas públicas, investimento, formação de base, espaços seguros para meninas, visibilidade e participação de profissionais do futebol feminino.</t>
+          <t>A CBF comunicou aos clubes que as competições masculinas e femininas terão pausa obrigatória entre 24/06 e 25/07/2027, durante toda a Copa do Mundo Feminina, enquanto a entidade ajusta o calendário nacional e a disponibilidade das oito arenas do torneio.</t>
         </is>
       </c>
     </row>
@@ -33981,12 +33981,12 @@
       </c>
       <c r="B89" s="23" t="inlineStr">
         <is>
-          <t>Painel debate legado da Copa 2027 no Summit Mulheres nas Profissões</t>
+          <t>Elas Jogam Summit propõe ações para construir o legado da Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C89" s="23" t="inlineStr">
         <is>
-          <t>Legado / futebol feminino</t>
+          <t>Elas Jogam Summit / legado</t>
         </is>
       </c>
       <c r="D89" s="23" t="inlineStr">
@@ -33996,12 +33996,12 @@
       </c>
       <c r="E89" s="23" t="inlineStr">
         <is>
-          <t>O Liberal</t>
+          <t>Donas FC</t>
         </is>
       </c>
       <c r="F89" s="23" t="inlineStr">
         <is>
-          <t>https://www.oliberal.com/esportes/nao-da-para-falar-em-paixao-nacional-so-valorizando-o-masculino-diz-secretaria-da-copa-1.1153852</t>
+          <t>https://donasfc.com.br/2026/08/05/elas-jogam-summit-discutira-o-legado-da-copa-do-mundo-feminina-2027-em-evento-no-pacaembu/</t>
         </is>
       </c>
       <c r="G89" s="23" t="inlineStr">
@@ -34016,22 +34016,22 @@
       </c>
       <c r="I89" s="23" t="inlineStr">
         <is>
-          <t>Painel reuniu representantes do esporte e Formiga para discutir legado, turismo e valorização do futebol feminino.</t>
+          <t>A matéria apresentou o Elas Jogam Summit e sua proposta de transformar a Copa Feminina 2027 em legado por meio de políticas públicas, investimento, formação de base, espaços seguros para meninas, visibilidade e participação de profissionais do futebol feminino.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="33" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="B90" s="23" t="inlineStr">
         <is>
-          <t>Especialistas defendem descentralização do legado da Copa Feminina 2027</t>
+          <t>Painel debate legado da Copa 2027 no Summit Mulheres nas Profissões</t>
         </is>
       </c>
       <c r="C90" s="23" t="inlineStr">
         <is>
-          <t>Fórum Sustentabilidade em Campo / legado / EVT-0063</t>
+          <t>Legado / futebol feminino</t>
         </is>
       </c>
       <c r="D90" s="23" t="inlineStr">
@@ -34041,17 +34041,17 @@
       </c>
       <c r="E90" s="23" t="inlineStr">
         <is>
-          <t>Máquina do Esporte</t>
+          <t>O Liberal</t>
         </is>
       </c>
       <c r="F90" s="23" t="inlineStr">
         <is>
-          <t>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/desafio-para-copa-do-mundo-feminina-2027-e-descentralizar-legado-dizem-especialistas/</t>
+          <t>https://www.oliberal.com/esportes/nao-da-para-falar-em-paixao-nacional-so-valorizando-o-masculino-diz-secretaria-da-copa-1.1153852</t>
         </is>
       </c>
       <c r="G90" s="23" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Positivo</t>
         </is>
       </c>
       <c r="H90" s="23" t="inlineStr">
@@ -34061,65 +34061,99 @@
       </c>
       <c r="I90" s="23" t="inlineStr">
         <is>
-          <t>No Fórum Sustentabilidade em Campo (EVT-0063), especialistas defenderam que os investimentos e benefícios da Copa Feminina 2027 alcancem mercados periféricos e diferentes regiões do país. O debate também apontou gestão, base, patrocínio e governança como condições para um legado sustentável.</t>
+          <t>Painel reuniu representantes do esporte e Formiga para discutir legado, turismo e valorização do futebol feminino.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="33" t="n">
+        <v>46238</v>
+      </c>
+      <c r="B91" s="23" t="inlineStr">
+        <is>
+          <t>Especialistas defendem descentralização do legado da Copa Feminina 2027</t>
+        </is>
+      </c>
+      <c r="C91" s="23" t="inlineStr">
+        <is>
+          <t>Fórum Sustentabilidade em Campo / legado / EVT-0063</t>
+        </is>
+      </c>
+      <c r="D91" s="23" t="inlineStr">
+        <is>
+          <t>São Paulo/SP</t>
+        </is>
+      </c>
+      <c r="E91" s="23" t="inlineStr">
+        <is>
+          <t>Máquina do Esporte</t>
+        </is>
+      </c>
+      <c r="F91" s="23" t="inlineStr">
+        <is>
+          <t>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/desafio-para-copa-do-mundo-feminina-2027-e-descentralizar-legado-dizem-especialistas/</t>
+        </is>
+      </c>
+      <c r="G91" s="23" t="inlineStr">
+        <is>
+          <t>Neutro</t>
+        </is>
+      </c>
+      <c r="H91" s="23" t="inlineStr">
+        <is>
+          <t>Médio</t>
+        </is>
+      </c>
+      <c r="I91" s="23" t="inlineStr">
+        <is>
+          <t>No Fórum Sustentabilidade em Campo (EVT-0063), especialistas defenderam que os investimentos e benefícios da Copa Feminina 2027 alcancem mercados periféricos e diferentes regiões do país. O debate também apontou gestão, base, patrocínio e governança como condições para um legado sustentável.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="33" t="n">
         <v>46199</v>
       </c>
-      <c r="B91" s="23" t="inlineStr">
+      <c r="B92" s="23" t="inlineStr">
         <is>
           <t>CBF divulga calendário do segundo semestre das Seleções Femininas de Base</t>
         </is>
       </c>
-      <c r="C91" s="23" t="inlineStr">
+      <c r="C92" s="23" t="inlineStr">
         <is>
           <t>Seleções de Base / calendário 2026</t>
         </is>
       </c>
-      <c r="D91" s="23" t="inlineStr">
+      <c r="D92" s="23" t="inlineStr">
         <is>
           <t>Brasil e exterior</t>
         </is>
       </c>
-      <c r="E91" s="23" t="inlineStr">
+      <c r="E92" s="23" t="inlineStr">
         <is>
           <t>CBF</t>
         </is>
       </c>
-      <c r="F91" s="23" t="inlineStr">
+      <c r="F92" s="23" t="inlineStr">
         <is>
           <t>https://www.cbf.com.br/selecao-brasileira/noticias/noticias/selecao-base-feminina/confira-o-calendario-do-segundo-semestre-das-selecoes-femininas-de-base</t>
         </is>
       </c>
-      <c r="G91" s="23" t="inlineStr">
+      <c r="G92" s="23" t="inlineStr">
         <is>
           <t>Neutro</t>
         </is>
       </c>
-      <c r="H91" s="23" t="inlineStr">
+      <c r="H92" s="23" t="inlineStr">
         <is>
           <t>Alto</t>
         </is>
       </c>
-      <c r="I91" s="23" t="inlineStr">
+      <c r="I92" s="23" t="inlineStr">
         <is>
           <t>O calendário oficial reúne Liga Evolução Sub-15, Copas do Mundo Sub-17 e Sub-20, períodos de treinamento, Torneio Brasil e amistosos internacionais entre junho e dezembro de 2026.</t>
         </is>
       </c>
-    </row>
-    <row r="92">
-      <c r="A92" s="6" t="n"/>
-      <c r="B92" s="23" t="n"/>
-      <c r="C92" s="23" t="n"/>
-      <c r="D92" s="23" t="n"/>
-      <c r="E92" s="23" t="n"/>
-      <c r="F92" s="23" t="n"/>
-      <c r="G92" s="23" t="n"/>
-      <c r="H92" s="23" t="n"/>
-      <c r="I92" s="23" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="6" t="n"/>

</xml_diff>

<commit_message>
Sincroniza planilha com dados atuais do Radar
</commit_message>
<xml_diff>
--- a/Radar_Brasil_2027.xlsx
+++ b/Radar_Brasil_2027.xlsx
@@ -1351,7 +1351,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="NoticiasTable" displayName="NoticiasTable" ref="A1:I95" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="NoticiasTable" displayName="NoticiasTable" ref="A1:I94" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="A1:I58"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Data"/>
@@ -30122,7 +30122,7 @@
       </c>
       <c r="B2" s="9" t="inlineStr">
         <is>
-          <t>Quais serão as cidades-sedes e os estádios do Brasil na Copa do Mundo Feminina de 2027? - LANCE!</t>
+          <t>Copa do Mundo Feminina 2027: saiba as datas e locais dos jogos da Seleção Brasileira - Terra</t>
         </is>
       </c>
       <c r="C2" s="9" t="inlineStr">
@@ -30137,12 +30137,12 @@
       </c>
       <c r="E2" s="9" t="inlineStr">
         <is>
-          <t>lance.com.br</t>
+          <t>terra.com.br</t>
         </is>
       </c>
       <c r="F2" s="9" t="inlineStr">
         <is>
-          <t>https://www.lance.com.br/futebol-nacional/quais-serao-as-cidades-sedes-e-os-estadios-do-brasil-na-copa-do-mundo-feminina-de-2027.html</t>
+          <t>https://www.terra.com.br/esportes/futebol/copa-feminina/copa-do-mundo-feminina-2027-saiba-as-datas-e-locais-dos-jogos-da-selecao-brasileira,ebc8ed8cc608d85c97b8cce34f91611b3t35hsvt.html</t>
         </is>
       </c>
       <c r="G2" s="9" t="inlineStr">
@@ -30157,17 +30157,17 @@
       </c>
       <c r="I2" s="9" t="inlineStr">
         <is>
-          <t>Quais serão as cidades-sedes e os estádios do Brasil na Copa do Mundo Feminina de 2027? Brasileirão Tabelas Vídeos Onde Assistir Lance! Jogos Futebol Nacional Quais serão as cidades-sedes e os estádios do Brasil na Copa do Mundo Feminina de 2027? Candidatura do Brasil definiu 10 estádios para sediar os jogos Por Lance! • Rio de Janeiro (RJ) 17/05/2024 08:55 Supervisionado por Lance! , Favorite o Lance! no Google Supervisionado por Lance! , Brasil foi escolhido como sede da Copa do Mundo Feminina 2027 (Fifa) A candidatura do Brasil para sediar a Copa do Mundo Feminina de 2027 definiu 10 estádios para realizar o torneio. Embora a Fifa ainda possa alterar essa programação, o país conta com arenas modernas por conta do Mundial Masculino realizado em 2014. ➡ A boa do Lance! Betting: vamos dobrar seu primeiro depósito, até R$200! Basta abrir sua conta e tá na mão! De acordo com a apuração do "</t>
+          <t>A Fifa realizou nesta quinta-feira, 20, a cerimônia oficial para divulgar a tabela da Copa do Mundo Feminina de 2027, que será disputada no Brasil, definindo os locais das partidas da Seleção. A Copa Feminina será realizada entre os dias 24 de junho e 25 de julho de 2027. Receba as principais notícias direto no WhatsApp! Inscreva-se no canal do Terra Se avançar para as oitavas, o Brasil pode jogar: Sendo 1º lugar no grupo A, o caminho nas quartas e na semifinal seria com estas datas: Sendo 2º lugar no grupo A, o restante do caminho seria com estas datas: A final está marcada para o domingo 25 de julho , no Maracanã, no Rio de Janeiro. A disputa de terceiro lugar acontece um dia antes, no sábado 24 de julho , em São Paulo. O sorteio dos grupos de cada seleção será realizado em dezembro, em data ainda a ser definida. Apenas o Brasil, anfitrião da competição, já sabe que está no grupo A. Du</t>
         </is>
       </c>
     </row>
     <row r="3" ht="114" customHeight="1" s="1">
       <c r="A3" s="31" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>Copa do Mundo Feminina 2027: saiba as datas e locais dos jogos da Seleção Brasileira - Terra</t>
+          <t>Brasil recebe Mundial Feminino 2027 e define regras para trabalho de imigrantes - www.gov.br</t>
         </is>
       </c>
       <c r="C3" s="9" t="inlineStr">
@@ -30182,12 +30182,12 @@
       </c>
       <c r="E3" s="9" t="inlineStr">
         <is>
-          <t>terra.com.br</t>
+          <t>gov.br</t>
         </is>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
-          <t>https://www.terra.com.br/esportes/futebol/copa-feminina/copa-do-mundo-feminina-2027-saiba-as-datas-e-locais-dos-jogos-da-selecao-brasileira,ebc8ed8cc608d85c97b8cce34f91611b3t35hsvt.html</t>
+          <t>https://www.gov.br/mj/pt-br/assuntos/noticias-1/brasil-recebe-mundial-feminino-2027-e-define-regras-para-trabalho-de-estrangeiros</t>
         </is>
       </c>
       <c r="G3" s="9" t="inlineStr">
@@ -30202,7 +30202,7 @@
       </c>
       <c r="I3" s="9" t="inlineStr">
         <is>
-          <t>Copa do Mundo Feminina 2027: saiba as datas e locais dos jogos da Seleção Brasileira Script = https://s1.trrsf.com/update-1789154714/fe/zaz-ui-t360/_js/transition.min.js Script = https://pagead2.googlesyndication.com/pagead/js/adsbygoogle.js?client=ca-pub-7059064278943417 Ir ao conteúdo Página principal ASSINE O TERRA MAIL Central do Assinante E-mail PUBLICIDADE Copa do Mundo Feminina Times Selecione o time para ver as notícias Publicidade Notícias relacionadas Fifa define calendário e repescagem da Copa Feminina 2027 CBF confirma parada do calendário durante a Copa do Mundo Feminina de 2027 Copa do Mundo Feminina de 2027 no Brasil deve levar mais de 2 milhões de torcedores aos estádios, projeta FIFA Copa do Mundo Feminina 2027: saiba as datas e locais dos jogos da Seleção Brasileira Mundial será disputado no Brasil entre os dias 24 de junho e 25 de julho de 2027 20 ago 2026 - 08h48 (atu</t>
+          <t xml:space="preserve">Para o Mundial de 2027, foi estabelecido procedimento específico de visto temporário para pessoas credenciadas ou convidadas pela Federação Internacional de Futebol (Fifa). Para os demais migrantes contratados por pessoa jurídica constituída no Brasil para exercer atividades necessárias aos eventos oficiais, poderão ser concedidos vistos temporários ou autorizações de residência para fins laborais. Nos casos que exigem autorização de residência prévia ou autorização de residência para fins laborais em território nacional, o pedido é analisado pela Coordenação-Geral de Imigração Laboral (CGIL), do Departamento de Migrações (Demig) da Secretaria Nacional de Justiça do Ministério da Justiça e Segurança Pública (MJSP). Visto temporário e autorização de residência são a mesma coisa? Não. Para quem pretende vir ao Brasil a trabalho, os dois documentos podem fazer parte do processo migratório, </t>
         </is>
       </c>
     </row>
@@ -30212,7 +30212,7 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>Brasil recebe Mundial Feminino 2027 e define regras para trabalho de imigrantes - www.gov.br</t>
+          <t>Câmara aprova férias escolares facultativas durante Copa do Mundo Feminina de 2027 - O GLOBO</t>
         </is>
       </c>
       <c r="C4" s="9" t="inlineStr">
@@ -30227,12 +30227,12 @@
       </c>
       <c r="E4" s="9" t="inlineStr">
         <is>
-          <t>gov.br</t>
+          <t>oglobo.globo.com</t>
         </is>
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mj/pt-br/assuntos/noticias-1/brasil-recebe-mundial-feminino-2027-e-define-regras-para-trabalho-de-estrangeiros</t>
+          <t>https://oglobo.globo.com/brasil/noticia/2026/09/01/camara-aprova-ferias-escolares-facultativas-durante-copa-do-mundo-feminina-de-2027.ghtml</t>
         </is>
       </c>
       <c r="G4" s="9" t="inlineStr">
@@ -30247,17 +30247,17 @@
       </c>
       <c r="I4" s="9" t="inlineStr">
         <is>
-          <t>Brasil recebe Mundial Feminino 2027 e define regras para trabalho de imigrantes — Ministério da Justiça e Segurança Pública Ir para o Conteúdo 1 Ir para a Página Inicial 2 Ir para o menu de Navegação 3 Ir para a Busca 4 Ir para o Mapa do site 5 Atenção! Seu navegador não pode executar javascript. Alguns recursos podem não funcionar corretamente. --&gt; Abrir menu principal de navegação Nome do site --&gt; Ministério da Justiça e Segurança Pública Termos mais buscados imposto de renda assinatura mei inss Desenrola Brasil Termos mais buscados imposto de renda assinatura mei Assuntos Notícias Secretaria Nacional de Justiça - Senajus DRCI Combate à Corrupção, à Lavagem de Dinheiro e ao Financiamento ao Terrorismo Cooperação Jurídica Internacional Enfrentamento ao Tráfico de Pessoas Refúgio Migrações Justiça e Proteção para as Mulheres Secretaria Nacional de Acesso à Justiça - Saju Projetos Editais</t>
+          <t>A Câmara dos Deputados aprovou, nesta segunda-feira (31), regras que permitem às escolas decidir se querem ajustar o calendário de férias durante a Copa do Mundo Feminina de 2027. A proposta, que busca preservar a autonomia dos sistemas de ensino, segue agora para análise do Senado. O texto é um substitutivo do deputado Alex Manente (Cidadania-SP) ao Projeto de Lei 3.481/26, da deputada Any Ortiz (PP-RS). Ex-jogador Luizão é acusado de agredir namorada por ciúmes Quem é Hayner, jogador do Vila Nova que é alvo de investigação sobre tráfico de drogas e armas A legislação atual, aprovada em junho, determina que escolas públicas e privadas ajustem o calendário escolar para que as férias coincidam com o período de abertura e encerramento do campeonato. Pela nova proposta aprovada pela Câmara, porém, a alteração passa a ser facultativa, e cada sistema de ensino poderá decidir se fará ou não mu</t>
         </is>
       </c>
     </row>
     <row r="5" ht="128.25" customHeight="1" s="1">
       <c r="A5" s="31" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>Câmara aprova férias escolares facultativas durante Copa do Mundo Feminina de 2027 - O GLOBO</t>
+          <t>A 9 meses da Copa do Mundo, TVs já apostam em programas de futebol feminino</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
@@ -30272,12 +30272,12 @@
       </c>
       <c r="E5" s="9" t="inlineStr">
         <is>
-          <t>oglobo.globo.com</t>
+          <t>noticiasdatv.uol.com.br</t>
         </is>
       </c>
       <c r="F5" s="9" t="inlineStr">
         <is>
-          <t>https://oglobo.globo.com/brasil/noticia/2026/09/01/camara-aprova-ferias-escolares-facultativas-durante-copa-do-mundo-feminina-de-2027.ghtml</t>
+          <t>https://noticiasdatv.uol.com.br/noticia/televisao/a-9-meses-da-copa-do-mundo-tvs-ja-apostam-em-programas-de-futebol-feminino-156477</t>
         </is>
       </c>
       <c r="G5" s="9" t="inlineStr">
@@ -30290,24 +30290,20 @@
           <t>Médio</t>
         </is>
       </c>
-      <c r="I5" s="9" t="inlineStr">
-        <is>
-          <t>Câmara aprova férias escolares facultativas durante Copa do Mundo Feminina de 2027 Carregando... Acesse sua conta ou cadastre-se grátis sair Últimas Notícias Newsletter O GLOBO por dentro 101 Brasileiros -- Política Voltar Política Página Principal"&gt; Página Principal Sonar - A escuta das redes"&gt; Sonar - A escuta das redes Pulso"&gt; Pulso Rali"&gt; Rali Eleições 2026"&gt; Eleições 2026 Brasil Voltar Brasil Página Principal"&gt; Página Principal Educação"&gt; Educação Voltar Educação Educação &gt; Página Principal"&gt; Página Principal Educação &gt; Enem 2025"&gt; Enem 2025 Voltar Enem 2025 Educação &gt; Enem 2025 &gt; Página Principal"&gt; Página Principal Educação &gt; Prêmio Jovem Cientista"&gt; Prêmio Jovem Cientista Clima Extremo"&gt; Clima Extremo Meio Ambiente"&gt; Meio Ambiente Segurança Pública"&gt; Segurança Pública Direitos Humanos"&gt; Direitos Humanos São Paulo"&gt; São Paulo Minas Gerais"&gt; Minas Gerais Rio Voltar Rio Página Princi</t>
-        </is>
-      </c>
+      <c r="I5" s="9" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="32" t="n">
-        <v>46277</v>
+        <v>46252</v>
       </c>
       <c r="B6" s="23" t="inlineStr">
         <is>
-          <t>A 9 meses da Copa do Mundo, TVs já apostam em programas de futebol feminino</t>
+          <t>CNE orienta ajustes no calendário escolar durante a Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C6" s="23" t="inlineStr">
         <is>
-          <t>Copa Feminina 2027</t>
+          <t>Educação / calendário escolar / cidades-sede / operação da Copa 2027</t>
         </is>
       </c>
       <c r="D6" s="23" t="inlineStr">
@@ -30317,12 +30313,12 @@
       </c>
       <c r="E6" s="23" t="inlineStr">
         <is>
-          <t>noticiasdatv.uol.com.br</t>
+          <t>MEC / CNE</t>
         </is>
       </c>
       <c r="F6" s="23" t="inlineStr">
         <is>
-          <t>https://noticiasdatv.uol.com.br/noticia/televisao/a-9-meses-da-copa-do-mundo-tvs-ja-apostam-em-programas-de-futebol-feminino-156477</t>
+          <t>https://www.gov.br/mec/pt-br/assuntos/noticias/2026/agosto/cne-orienta-redes-de-ensino-sobre-organizacao-do-calendario-escolar-durante-a-copa-do-mundo-feminina-de-2027</t>
         </is>
       </c>
       <c r="G6" s="23" t="inlineStr">
@@ -30332,38 +30328,42 @@
       </c>
       <c r="H6" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
-        </is>
-      </c>
-      <c r="I6" s="23" t="inlineStr"/>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="I6" s="23" t="inlineStr">
+        <is>
+          <t>O Conselho Nacional de Educação aprovou o Parecer CNE/CEB nº 7/2026 orientando os sistemas de ensino sobre a organização dos calendários escolares de 2027 em razão da Copa do Mundo Feminina. Cidades-sede, regiões metropolitanas e áreas diretamente impactadas deverão promover os ajustes necessários conforme a realidade local e o calendário oficial da competição.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="32" t="n">
-        <v>46252</v>
+        <v>46276</v>
       </c>
       <c r="B7" s="23" t="inlineStr">
         <is>
-          <t>CNE orienta ajustes no calendário escolar durante a Copa Feminina 2027</t>
+          <t>Maracanã trocará gramado em 2027 antes da Copa do Mundo Feminina</t>
         </is>
       </c>
       <c r="C7" s="23" t="inlineStr">
         <is>
-          <t>Educação / calendário escolar / cidades-sede / operação da Copa 2027</t>
+          <t>Rio de Janeiro / Maracanã / gramado / infraestrutura / Copa Feminina 2027</t>
         </is>
       </c>
       <c r="D7" s="23" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Rio de Janeiro/RJ</t>
         </is>
       </c>
       <c r="E7" s="23" t="inlineStr">
         <is>
-          <t>MEC / CNE</t>
+          <t>UOL</t>
         </is>
       </c>
       <c r="F7" s="23" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/assuntos/noticias/2026/agosto/cne-orienta-redes-de-ensino-sobre-organizacao-do-calendario-escolar-durante-a-copa-do-mundo-feminina-de-2027</t>
+          <t>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/09/11/maracana-aponta-fatores-para-campo-ruim-e-informa-que-trocara-tipo-de-grama.ghtm</t>
         </is>
       </c>
       <c r="G7" s="23" t="inlineStr">
@@ -30378,27 +30378,27 @@
       </c>
       <c r="I7" s="23" t="inlineStr">
         <is>
-          <t>O Conselho Nacional de Educação aprovou o Parecer CNE/CEB nº 7/2026 orientando os sistemas de ensino sobre a organização dos calendários escolares de 2027 em razão da Copa do Mundo Feminina. Cidades-sede, regiões metropolitanas e áreas diretamente impactadas deverão promover os ajustes necessários conforme a realidade local e o calendário oficial da competição.</t>
+          <t>A administração do Maracanã informou que substituirá o gramado atual por Celebration Hybrid em 2027. A mudança ocorre em um ano de calendário intenso no estádio, que receberá partidas da Copa do Mundo Feminina, incluindo a abertura e a final do torneio, e busca melhorar a qualidade do campo após críticas recorrentes.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="32" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="B8" s="23" t="inlineStr">
         <is>
-          <t>Maracanã trocará gramado em 2027 antes da Copa do Mundo Feminina</t>
+          <t>Debate cobra legado duradouro da Copa Feminina 2027 para mulheres no esporte</t>
         </is>
       </c>
       <c r="C8" s="23" t="inlineStr">
         <is>
-          <t>Rio de Janeiro / Maracanã / gramado / infraestrutura / Copa Feminina 2027</t>
+          <t>Legado social / futebol feminino / políticas públicas / Copa Feminina 2027</t>
         </is>
       </c>
       <c r="D8" s="23" t="inlineStr">
         <is>
-          <t>Rio de Janeiro/RJ</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E8" s="23" t="inlineStr">
@@ -30408,7 +30408,7 @@
       </c>
       <c r="F8" s="23" t="inlineStr">
         <is>
-          <t>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/09/11/maracana-aponta-fatores-para-campo-ruim-e-informa-que-trocara-tipo-de-grama.ghtm</t>
+          <t>https://noticias.uol.com.br/colunas/joildo-santos/2026/09/10/a-copa-das-mulheres-vai-deixar-um-legado-ou-apenas-uma-fotografia.ghtm</t>
         </is>
       </c>
       <c r="G8" s="23" t="inlineStr">
@@ -30418,12 +30418,12 @@
       </c>
       <c r="H8" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I8" s="23" t="inlineStr">
         <is>
-          <t>A administração do Maracanã informou que substituirá o gramado atual por Celebration Hybrid em 2027. A mudança ocorre em um ano de calendário intenso no estádio, que receberá partidas da Copa do Mundo Feminina, incluindo a abertura e a final do torneio, e busca melhorar a qualidade do campo após críticas recorrentes.</t>
+          <t>Artigo publicado em 10/09/2026 discute se a Copa do Mundo Feminina de 2027 deixará legado estrutural para mulheres no esporte, defendendo investimentos permanentes em infraestrutura, formação, acesso à modalidade e políticas de proteção e equidade, para que o impacto do torneio ultrapasse a realização dos jogos.</t>
         </is>
       </c>
     </row>
@@ -30433,12 +30433,12 @@
       </c>
       <c r="B9" s="23" t="inlineStr">
         <is>
-          <t>Debate cobra legado duradouro da Copa Feminina 2027 para mulheres no esporte</t>
+          <t>CBF prevê pausa no futebol masculino durante a Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C9" s="23" t="inlineStr">
         <is>
-          <t>Legado social / futebol feminino / políticas públicas / Copa Feminina 2027</t>
+          <t>Calendário CBF / operação dos estádios / Copa Feminina 2027</t>
         </is>
       </c>
       <c r="D9" s="23" t="inlineStr">
@@ -30453,7 +30453,7 @@
       </c>
       <c r="F9" s="23" t="inlineStr">
         <is>
-          <t>https://noticias.uol.com.br/colunas/joildo-santos/2026/09/10/a-copa-das-mulheres-vai-deixar-um-legado-ou-apenas-uma-fotografia.ghtm</t>
+          <t>https://www.uol.com.br/esporte/futebol/colunas/rodrigo-mattos/2026/09/10/o-que-se-sabe-sobre-o-calendario-do-futebol-para-2027.ghtm</t>
         </is>
       </c>
       <c r="G9" s="23" t="inlineStr">
@@ -30463,87 +30463,87 @@
       </c>
       <c r="H9" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I9" s="23" t="inlineStr">
         <is>
-          <t>Artigo publicado em 10/09/2026 discute se a Copa do Mundo Feminina de 2027 deixará legado estrutural para mulheres no esporte, defendendo investimentos permanentes em infraestrutura, formação, acesso à modalidade e políticas de proteção e equidade, para que o impacto do torneio ultrapasse a realização dos jogos.</t>
+          <t>A CBF prepara o calendário de 2027 prevendo paralisação do futebol masculino durante a Copa do Mundo Feminina e ajustes cerca de 15 dias antes do início do torneio para liberar os estádios cedidos à FIFA. A medida afeta diretamente a operação de arenas como Maracanã, Arena Itaquera, Beira-Rio, Mineirão e Arena Salvador durante o Mundial.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="32" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B10" s="23" t="inlineStr">
         <is>
-          <t>CBF prevê pausa no futebol masculino durante a Copa Feminina 2027</t>
+          <t>Estádio Presidente Vargas recebe visita técnica da FIFA e avança nos preparativos para 2027</t>
         </is>
       </c>
       <c r="C10" s="23" t="inlineStr">
         <is>
-          <t>Calendário CBF / operação dos estádios / Copa Feminina 2027</t>
+          <t>Fortaleza / estádio de apoio / inspeção FIFA / operação da Copa 2027</t>
         </is>
       </c>
       <c r="D10" s="23" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Fortaleza/CE</t>
         </is>
       </c>
       <c r="E10" s="23" t="inlineStr">
         <is>
-          <t>UOL</t>
+          <t>Portal IN</t>
         </is>
       </c>
       <c r="F10" s="23" t="inlineStr">
         <is>
-          <t>https://www.uol.com.br/esporte/futebol/colunas/rodrigo-mattos/2026/09/10/o-que-se-sabe-sobre-o-calendario-do-futebol-para-2027.ghtm</t>
+          <t>https://www.portalin.com.br/in-loco/estadio-presidente-vargas-recebe-visita-tecnica-da-fifa-e-avanca-os-preparativos/</t>
         </is>
       </c>
       <c r="G10" s="23" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Positivo</t>
         </is>
       </c>
       <c r="H10" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I10" s="23" t="inlineStr">
         <is>
-          <t>A CBF prepara o calendário de 2027 prevendo paralisação do futebol masculino durante a Copa do Mundo Feminina e ajustes cerca de 15 dias antes do início do torneio para liberar os estádios cedidos à FIFA. A medida afeta diretamente a operação de arenas como Maracanã, Arena Itaquera, Beira-Rio, Mineirão e Arena Salvador durante o Mundial.</t>
+          <t>O Estádio Presidente Vargas, em Fortaleza, recebeu visita técnica da FIFA para avaliação de estrutura, logística e operação ligadas à Copa do Mundo Feminina 2027. O equipamento deve integrar a estrutura de apoio da cidade-sede, ao lado da Arena Castelão, atendendo delegações e operações do torneio.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="32" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="B11" s="23" t="inlineStr">
         <is>
-          <t>Estádio Presidente Vargas recebe visita técnica da FIFA e avança nos preparativos para 2027</t>
+          <t>CBF vê Copa Feminina 2027 como teste para Mundial de Clubes de 2029 no Brasil</t>
         </is>
       </c>
       <c r="C11" s="23" t="inlineStr">
         <is>
-          <t>Fortaleza / estádio de apoio / inspeção FIFA / operação da Copa 2027</t>
+          <t>CBF / estratégia internacional / Copa Feminina 2027 / Mundial de Clubes 2029</t>
         </is>
       </c>
       <c r="D11" s="23" t="inlineStr">
         <is>
-          <t>Fortaleza/CE</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E11" s="23" t="inlineStr">
         <is>
-          <t>Portal IN</t>
+          <t>Lance!</t>
         </is>
       </c>
       <c r="F11" s="23" t="inlineStr">
         <is>
-          <t>https://www.portalin.com.br/in-loco/estadio-presidente-vargas-recebe-visita-tecnica-da-fifa-e-avanca-os-preparativos/</t>
+          <t>https://www.lance.com.br/futebol-feminino/cbf-ve-copa-do-mundo-feminina-como-teste-para-mundial-de-clubes-de-2029-no-brasil.html</t>
         </is>
       </c>
       <c r="G11" s="23" t="inlineStr">
@@ -30558,37 +30558,37 @@
       </c>
       <c r="I11" s="23" t="inlineStr">
         <is>
-          <t>O Estádio Presidente Vargas, em Fortaleza, recebeu visita técnica da FIFA para avaliação de estrutura, logística e operação ligadas à Copa do Mundo Feminina 2027. O equipamento deve integrar a estrutura de apoio da cidade-sede, ao lado da Arena Castelão, atendendo delegações e operações do torneio.</t>
+          <t>A CBF trata a organização da Copa do Mundo Feminina de 2027 no Brasil como referência e teste para projetos internacionais futuros, incluindo a possibilidade de receber um Mundial de Clubes em 2029. A pauta destaca iniciativas em discussão e a construção de uma estratégia de longo prazo ligada à realização do torneio feminino no país.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="32" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B12" s="23" t="inlineStr">
         <is>
-          <t>CBF vê Copa Feminina 2027 como teste para Mundial de Clubes de 2029 no Brasil</t>
+          <t>FIFA faz visita técnica ao Estádio Presidente Vargas nos preparativos para a Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C12" s="23" t="inlineStr">
         <is>
-          <t>CBF / estratégia internacional / Copa Feminina 2027 / Mundial de Clubes 2029</t>
+          <t>Fortaleza / centro de treinamento / infraestrutura / preparação da Copa 2027</t>
         </is>
       </c>
       <c r="D12" s="23" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Fortaleza/CE</t>
         </is>
       </c>
       <c r="E12" s="23" t="inlineStr">
         <is>
-          <t>Lance!</t>
+          <t>Prefeitura de Fortaleza</t>
         </is>
       </c>
       <c r="F12" s="23" t="inlineStr">
         <is>
-          <t>https://www.lance.com.br/futebol-feminino/cbf-ve-copa-do-mundo-feminina-como-teste-para-mundial-de-clubes-de-2029-no-brasil.html</t>
+          <t>https://fortaleza.ce.gov.br/noticias/nos-preparativos-para-a-copa-do-mundo-feminina-da-fifa-brasil-2027-estadio-presidente-vargas-recebe-visita-tecnica-da-entidade</t>
         </is>
       </c>
       <c r="G12" s="23" t="inlineStr">
@@ -30603,67 +30603,67 @@
       </c>
       <c r="I12" s="23" t="inlineStr">
         <is>
-          <t>A CBF trata a organização da Copa do Mundo Feminina de 2027 no Brasil como referência e teste para projetos internacionais futuros, incluindo a possibilidade de receber um Mundial de Clubes em 2029. A pauta destaca iniciativas em discussão e a construção de uma estratégia de longo prazo ligada à realização do torneio feminino no país.</t>
+          <t>O Estádio Presidente Vargas, em Fortaleza, recebeu em 04/09/2026 uma visita técnica da FIFA. A equipe avaliou instalações e a organização de espaços que poderão atender delegações e imprensa durante a Copa do Mundo Feminina FIFA 2027, reforçando a preparação da cidade-sede.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="32" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="B13" s="23" t="inlineStr">
         <is>
-          <t>FIFA faz visita técnica ao Estádio Presidente Vargas nos preparativos para a Copa Feminina 2027</t>
+          <t>CBF prepara calendário de 2027 com pausa e adaptação de estádios para a Copa Feminina</t>
         </is>
       </c>
       <c r="C13" s="23" t="inlineStr">
         <is>
-          <t>Fortaleza / centro de treinamento / infraestrutura / preparação da Copa 2027</t>
+          <t>Calendário CBF / clubes / estádios / operação da Copa 2027</t>
         </is>
       </c>
       <c r="D13" s="23" t="inlineStr">
         <is>
-          <t>Fortaleza/CE</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E13" s="23" t="inlineStr">
         <is>
-          <t>Prefeitura de Fortaleza</t>
+          <t>UOL</t>
         </is>
       </c>
       <c r="F13" s="23" t="inlineStr">
         <is>
-          <t>https://fortaleza.ce.gov.br/noticias/nos-preparativos-para-a-copa-do-mundo-feminina-da-fifa-brasil-2027-estadio-presidente-vargas-recebe-visita-tecnica-da-entidade</t>
+          <t>https://www.uol.com.br/esporte/futebol/colunas/rodrigo-mattos/2026/09/10/o-que-se-sabe-sobre-o-calendario-do-futebol-para-2027.htm</t>
         </is>
       </c>
       <c r="G13" s="23" t="inlineStr">
         <is>
-          <t>Positivo</t>
+          <t>Neutro</t>
         </is>
       </c>
       <c r="H13" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I13" s="23" t="inlineStr">
         <is>
-          <t>O Estádio Presidente Vargas, em Fortaleza, recebeu em 04/09/2026 uma visita técnica da FIFA. A equipe avaliou instalações e a organização de espaços que poderão atender delegações e imprensa durante a Copa do Mundo Feminina FIFA 2027, reforçando a preparação da cidade-sede.</t>
+          <t>A CBF prepara o calendário do futebol brasileiro de 2027 considerando a paralisação do futebol masculino durante a Copa do Mundo Feminina e ajustes cerca de 15 dias antes do torneio para evitar jogos nos estádios cedidos à FIFA. A medida afeta arenas como Maracanã, Neo Química Arena, Beira-Rio e Mineirão.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="32" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B14" s="23" t="inlineStr">
         <is>
-          <t>CBF prepara calendário de 2027 com pausa e adaptação de estádios para a Copa Feminina</t>
+          <t>Governo negocia ingressos populares para a Copa do Mundo Feminina 2027</t>
         </is>
       </c>
       <c r="C14" s="23" t="inlineStr">
         <is>
-          <t>Calendário CBF / clubes / estádios / operação da Copa 2027</t>
+          <t>Ingressos / acesso / organização da Copa 2027</t>
         </is>
       </c>
       <c r="D14" s="23" t="inlineStr">
@@ -30673,17 +30673,17 @@
       </c>
       <c r="E14" s="23" t="inlineStr">
         <is>
-          <t>UOL</t>
+          <t>ge</t>
         </is>
       </c>
       <c r="F14" s="23" t="inlineStr">
         <is>
-          <t>https://www.uol.com.br/esporte/futebol/colunas/rodrigo-mattos/2026/09/10/o-que-se-sabe-sobre-o-calendario-do-futebol-para-2027.htm</t>
+          <t>https://ge.globo.com/futebol/copa-do-mundo/noticia/2026/09/09/copa-feminina-governo-negocia-ingressos-populares-e-cre-em-torneio-blindado-da-crise-na-fifa.ghtml</t>
         </is>
       </c>
       <c r="G14" s="23" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Positivo</t>
         </is>
       </c>
       <c r="H14" s="23" t="inlineStr">
@@ -30693,37 +30693,37 @@
       </c>
       <c r="I14" s="23" t="inlineStr">
         <is>
-          <t>A CBF prepara o calendário do futebol brasileiro de 2027 considerando a paralisação do futebol masculino durante a Copa do Mundo Feminina e ajustes cerca de 15 dias antes do torneio para evitar jogos nos estádios cedidos à FIFA. A medida afeta arenas como Maracanã, Neo Química Arena, Beira-Rio e Mineirão.</t>
+          <t>O Governo Federal negocia com a FIFA uma cota de ingressos a preços populares para a Copa do Mundo Feminina de 2027 no Brasil. A pauta também envolve transporte, segurança, legado, calendário e medidas para ampliar o acesso do público aos estádios durante o torneio.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="32" t="n">
-        <v>46274</v>
+        <v>46267</v>
       </c>
       <c r="B15" s="23" t="inlineStr">
         <is>
-          <t>Governo negocia ingressos populares para a Copa do Mundo Feminina 2027</t>
+          <t>Pernambuco sanciona lei estadual para operação da Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C15" s="23" t="inlineStr">
         <is>
-          <t>Ingressos / acesso / organização da Copa 2027</t>
+          <t>Recife / legislação estadual / mobilidade / segurança / operação da Copa 2027</t>
         </is>
       </c>
       <c r="D15" s="23" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Recife/PE</t>
         </is>
       </c>
       <c r="E15" s="23" t="inlineStr">
         <is>
-          <t>ge</t>
+          <t>Alepe Legis</t>
         </is>
       </c>
       <c r="F15" s="23" t="inlineStr">
         <is>
-          <t>https://ge.globo.com/futebol/copa-do-mundo/noticia/2026/09/09/copa-feminina-governo-negocia-ingressos-populares-e-cre-em-torneio-blindado-da-crise-na-fifa.ghtml</t>
+          <t>https://legis.alepe.pe.gov.br/texto.aspx?id=89825&amp;tipo=</t>
         </is>
       </c>
       <c r="G15" s="23" t="inlineStr">
@@ -30738,37 +30738,37 @@
       </c>
       <c r="I15" s="23" t="inlineStr">
         <is>
-          <t>O Governo Federal negocia com a FIFA uma cota de ingressos a preços populares para a Copa do Mundo Feminina de 2027 no Brasil. A pauta também envolve transporte, segurança, legado, calendário e medidas para ampliar o acesso do público aos estádios durante o torneio.</t>
+          <t>Sancionada em 1º/09 e publicada no Diário Oficial em 2/09, a Lei nº 19.341/2026 estabelece as medidas estaduais para viabilizar a Copa Feminina 2027 em Pernambuco. A norma disciplina cooperação institucional, proteção comercial, controle de acesso, segurança, mobilidade, tramitação prioritária de licenças, hidratação do público e ações de turismo, futebol feminino e legado social.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="32" t="n">
-        <v>46267</v>
+        <v>46273</v>
       </c>
       <c r="B16" s="23" t="inlineStr">
         <is>
-          <t>Pernambuco sanciona lei estadual para operação da Copa Feminina 2027</t>
+          <t>Lorena é indicada ao prêmio de melhor goleira da Bola de Ouro 2026</t>
         </is>
       </c>
       <c r="C16" s="23" t="inlineStr">
         <is>
-          <t>Recife / legislação estadual / mobilidade / segurança / operação da Copa 2027</t>
+          <t>Seleção Brasileira / Lorena / Bola de Ouro 2026 / ciclo da Copa Feminina 2027</t>
         </is>
       </c>
       <c r="D16" s="23" t="inlineStr">
         <is>
-          <t>Recife/PE</t>
+          <t>Internacional</t>
         </is>
       </c>
       <c r="E16" s="23" t="inlineStr">
         <is>
-          <t>Alepe Legis</t>
+          <t>CNN Brasil</t>
         </is>
       </c>
       <c r="F16" s="23" t="inlineStr">
         <is>
-          <t>https://legis.alepe.pe.gov.br/texto.aspx?id=89825&amp;tipo=</t>
+          <t>https://www.cnnbrasil.com.br/esportes/futebol/futebol-internacional/bola-de-ouro-lorena-e-indicada-a-melhor-goleira-do-futebol-feminino/</t>
         </is>
       </c>
       <c r="G16" s="23" t="inlineStr">
@@ -30778,42 +30778,42 @@
       </c>
       <c r="H16" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I16" s="23" t="inlineStr">
         <is>
-          <t>Sancionada em 1º/09 e publicada no Diário Oficial em 2/09, a Lei nº 19.341/2026 estabelece as medidas estaduais para viabilizar a Copa Feminina 2027 em Pernambuco. A norma disciplina cooperação institucional, proteção comercial, controle de acesso, segurança, mobilidade, tramitação prioritária de licenças, hidratação do público e ações de turismo, futebol feminino e legado social.</t>
+          <t>Lorena, goleira titular da Seleção Brasileira principal e atleta do Kansas City, foi indicada em 08/09/2026 ao prêmio de melhor goleira do futebol feminino da Bola de Ouro 2026. O reconhecimento internacional integra o acompanhamento das principais atletas brasileiras no ciclo de preparação para a Copa do Mundo Feminina FIFA 2027 no Brasil.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="32" t="n">
-        <v>46273</v>
+        <v>46254</v>
       </c>
       <c r="B17" s="23" t="inlineStr">
         <is>
-          <t>Lorena é indicada ao prêmio de melhor goleira da Bola de Ouro 2026</t>
+          <t>São Paulo terá 10 jogos da Copa Feminina 2027 e prepara mobilidade, turismo e legado</t>
         </is>
       </c>
       <c r="C17" s="23" t="inlineStr">
         <is>
-          <t>Seleção Brasileira / Lorena / Bola de Ouro 2026 / ciclo da Copa Feminina 2027</t>
+          <t>São Paulo / calendário / Arena Itaquera / mobilidade / turismo / legado / Copa 2027</t>
         </is>
       </c>
       <c r="D17" s="23" t="inlineStr">
         <is>
-          <t>Internacional</t>
+          <t>São Paulo/SP</t>
         </is>
       </c>
       <c r="E17" s="23" t="inlineStr">
         <is>
-          <t>CNN Brasil</t>
+          <t>Prefeitura de São Paulo</t>
         </is>
       </c>
       <c r="F17" s="23" t="inlineStr">
         <is>
-          <t>https://www.cnnbrasil.com.br/esportes/futebol/futebol-internacional/bola-de-ouro-lorena-e-indicada-a-melhor-goleira-do-futebol-feminino/</t>
+          <t>https://www2.prefeitura.sp.gov.br/web/prefeitura-de-sao-paulo/w/cidade-com-mais-jogos-s%C3%A3o-paulo-receber%C3%A1-10-partidas-da-copa-do-mundo-feminina-2027</t>
         </is>
       </c>
       <c r="G17" s="23" t="inlineStr">
@@ -30823,42 +30823,42 @@
       </c>
       <c r="H17" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I17" s="23" t="inlineStr">
         <is>
-          <t>Lorena, goleira titular da Seleção Brasileira principal e atleta do Kansas City, foi indicada em 08/09/2026 ao prêmio de melhor goleira do futebol feminino da Bola de Ouro 2026. O reconhecimento internacional integra o acompanhamento das principais atletas brasileiras no ciclo de preparação para a Copa do Mundo Feminina FIFA 2027 no Brasil.</t>
+          <t>A Prefeitura de São Paulo detalhou em 20/08/2026 o calendário da cidade para a Copa do Mundo Feminina 2027. A capital receberá 10 das 64 partidas, o maior número entre as oito sedes, incluindo seis jogos de fase de grupos, a partida da Seleção Brasileira em 29/06/2027, uma oitava de final, uma quarta de final, uma semifinal e a disputa do terceiro lugar na Arena Itaquera. O município informa que mantém planejamento com a FIFA em mobilidade urbana, segurança, turismo, empreendedorismo e legado esportivo, além de ampliar atividades gratuitas de futebol feminino nos centros esportivos municipais.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="32" t="n">
-        <v>46254</v>
+        <v>46268</v>
       </c>
       <c r="B18" s="23" t="inlineStr">
         <is>
-          <t>São Paulo terá 10 jogos da Copa Feminina 2027 e prepara mobilidade, turismo e legado</t>
+          <t>Porto Alegre articula participação de pioneiras do Gre-Nal na programação da Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C18" s="23" t="inlineStr">
         <is>
-          <t>São Paulo / calendário / Arena Itaquera / mobilidade / turismo / legado / Copa 2027</t>
+          <t>Porto Alegre / legado / memória do futebol feminino / programação paralela / Copa 2027</t>
         </is>
       </c>
       <c r="D18" s="23" t="inlineStr">
         <is>
-          <t>São Paulo/SP</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="E18" s="23" t="inlineStr">
         <is>
-          <t>Prefeitura de São Paulo</t>
+          <t>Prefeitura de Porto Alegre / Secopa 2027</t>
         </is>
       </c>
       <c r="F18" s="23" t="inlineStr">
         <is>
-          <t>https://www2.prefeitura.sp.gov.br/web/prefeitura-de-sao-paulo/w/cidade-com-mais-jogos-s%C3%A3o-paulo-receber%C3%A1-10-partidas-da-copa-do-mundo-feminina-2027</t>
+          <t>https://prefeitura.poa.br/secopa2027/noticias/pioneiras-da-dupla-gre-nal-se-reunem-com-secopa-para-alinhar-acoes-para-copa-do</t>
         </is>
       </c>
       <c r="G18" s="23" t="inlineStr">
@@ -30868,42 +30868,42 @@
       </c>
       <c r="H18" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I18" s="23" t="inlineStr">
         <is>
-          <t>A Prefeitura de São Paulo detalhou em 20/08/2026 o calendário da cidade para a Copa do Mundo Feminina 2027. A capital receberá 10 das 64 partidas, o maior número entre as oito sedes, incluindo seis jogos de fase de grupos, a partida da Seleção Brasileira em 29/06/2027, uma oitava de final, uma quarta de final, uma semifinal e a disputa do terceiro lugar na Arena Itaquera. O município informa que mantém planejamento com a FIFA em mobilidade urbana, segurança, turismo, empreendedorismo e legado esportivo, além de ampliar atividades gratuitas de futebol feminino nos centros esportivos municipais.</t>
+          <t>A Secretaria Extraordinária da Copa do Mundo Feminina 2027 de Porto Alegre recebeu, em 03/09/2026, cinco pioneiras do futebol feminino de Grêmio e Internacional para discutir sua integração à programação do Mundial na cidade. Entre as propostas apresentadas estão reconhecimento oficial às atletas, homenagem no Beira-Rio, participação em seminários e eventos paralelos e acesso a partidas. A Secopa informou que avaliará, com as áreas municipais e parceiros do torneio, a viabilidade de incorporar as ações à programação oficial, conectando memória, legado e engajamento local em uma das cidades-sede.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="32" t="n">
-        <v>46268</v>
+        <v>46267</v>
       </c>
       <c r="B19" s="23" t="inlineStr">
         <is>
-          <t>Porto Alegre articula participação de pioneiras do Gre-Nal na programação da Copa Feminina 2027</t>
+          <t>Fortaleza avança em miniterminais no entorno do Castelão para mobilidade da Copa 2027</t>
         </is>
       </c>
       <c r="C19" s="23" t="inlineStr">
         <is>
-          <t>Porto Alegre / legado / memória do futebol feminino / programação paralela / Copa 2027</t>
+          <t>Fortaleza / mobilidade / infraestrutura / Arena Castelão / Copa 2027</t>
         </is>
       </c>
       <c r="D19" s="23" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Fortaleza/CE</t>
         </is>
       </c>
       <c r="E19" s="23" t="inlineStr">
         <is>
-          <t>Prefeitura de Porto Alegre / Secopa 2027</t>
+          <t>Prefeitura de Fortaleza</t>
         </is>
       </c>
       <c r="F19" s="23" t="inlineStr">
         <is>
-          <t>https://prefeitura.poa.br/secopa2027/noticias/pioneiras-da-dupla-gre-nal-se-reunem-com-secopa-para-alinhar-acoes-para-copa-do</t>
+          <t>https://fortaleza.ce.gov.br/noticias/prefeito-evandro-leitao-visita-obras-dos-miniterminais-da-arena-castelao</t>
         </is>
       </c>
       <c r="G19" s="23" t="inlineStr">
@@ -30913,42 +30913,42 @@
       </c>
       <c r="H19" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I19" s="23" t="inlineStr">
         <is>
-          <t>A Secretaria Extraordinária da Copa do Mundo Feminina 2027 de Porto Alegre recebeu, em 03/09/2026, cinco pioneiras do futebol feminino de Grêmio e Internacional para discutir sua integração à programação do Mundial na cidade. Entre as propostas apresentadas estão reconhecimento oficial às atletas, homenagem no Beira-Rio, participação em seminários e eventos paralelos e acesso a partidas. A Secopa informou que avaliará, com as áreas municipais e parceiros do torneio, a viabilidade de incorporar as ações à programação oficial, conectando memória, legado e engajamento local em uma das cidades-sede.</t>
+          <t>A Prefeitura de Fortaleza informou em 02/09/2026 que dois miniterminais de transporte coletivo estão em construção no entorno da Arena Castelão, com investimento aproximado de R$ 2,5 milhões, 30% de execução e conclusão prevista para dezembro de 2026. Os equipamentos terão capacidade para atender até mil pessoas simultaneamente e contarão com painéis de previsão de ônibus, bilhetagem eletrônica, acessibilidade, videomonitoramento e integração com linhas especiais em dias de jogos. O prefeito Evandro Leitão vinculou diretamente a obra à preparação para grandes eventos e para a Copa do Mundo Feminina de 2027, reforçando sua relevância para a mobilidade e a experiência de torcedores na cidade-sede.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="32" t="n">
-        <v>46267</v>
+        <v>46268</v>
       </c>
       <c r="B20" s="23" t="inlineStr">
         <is>
-          <t>Fortaleza avança em miniterminais no entorno do Castelão para mobilidade da Copa 2027</t>
+          <t>Turn On The Light inicia agenda de conexões sociais rumo à Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C20" s="23" t="inlineStr">
         <is>
-          <t>Fortaleza / mobilidade / infraestrutura / Arena Castelão / Copa 2027</t>
+          <t>Ativação / futebol feminino / maternidade / impacto social / Copa 2027</t>
         </is>
       </c>
       <c r="D20" s="23" t="inlineStr">
         <is>
-          <t>Fortaleza/CE</t>
+          <t>São Paulo/SP</t>
         </is>
       </c>
       <c r="E20" s="23" t="inlineStr">
         <is>
-          <t>Prefeitura de Fortaleza</t>
+          <t>BRA1 / Agência VIVA</t>
         </is>
       </c>
       <c r="F20" s="23" t="inlineStr">
         <is>
-          <t>https://fortaleza.ce.gov.br/noticias/prefeito-evandro-leitao-visita-obras-dos-miniterminais-da-arena-castelao</t>
+          <t>https://www.bra1.com.br/geral/id-688491/turn_on_the_light_inaugura_agenda_de_conexoes_entre_futebol_feminino__maternidade_e_causas_sociais_rumo_a_copa_do_mundo_de_2027</t>
         </is>
       </c>
       <c r="G20" s="23" t="inlineStr">
@@ -30958,42 +30958,42 @@
       </c>
       <c r="H20" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I20" s="23" t="inlineStr">
         <is>
-          <t>A Prefeitura de Fortaleza informou em 02/09/2026 que dois miniterminais de transporte coletivo estão em construção no entorno da Arena Castelão, com investimento aproximado de R$ 2,5 milhões, 30% de execução e conclusão prevista para dezembro de 2026. Os equipamentos terão capacidade para atender até mil pessoas simultaneamente e contarão com painéis de previsão de ônibus, bilhetagem eletrônica, acessibilidade, videomonitoramento e integração com linhas especiais em dias de jogos. O prefeito Evandro Leitão vinculou diretamente a obra à preparação para grandes eventos e para a Copa do Mundo Feminina de 2027, reforçando sua relevância para a mobilidade e a experiência de torcedores na cidade-sede.</t>
+          <t>A agência Turn On The Light iniciou uma agenda de encontros e narrativas que conectará futebol feminino, maternidade, carreira e causas sociais até a Copa do Mundo Feminina de 2027. A primeira ação ocorreu na Casa Mãe Paulistana, em São Paulo, com participação da jogadora Tamires, da ex-jogadora Milene Domingues, do comunicador Marco Aurélio e da cantora Gabi Fernandes. A iniciativa pretende usar a preparação para o Mundial como plataforma contínua de engajamento e protagonismo feminino fora dos estádios.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="32" t="n">
-        <v>46268</v>
+        <v>46266</v>
       </c>
       <c r="B21" s="23" t="inlineStr">
         <is>
-          <t>Turn On The Light inicia agenda de conexões sociais rumo à Copa Feminina 2027</t>
+          <t>Bahia prepara Sala Lilás e ações de proteção e legado feminino para a Copa 2027</t>
         </is>
       </c>
       <c r="C21" s="23" t="inlineStr">
         <is>
-          <t>Ativação / futebol feminino / maternidade / impacto social / Copa 2027</t>
+          <t>Salvador / segurança das mulheres / turismo / legado / futebol feminino / Copa 2027</t>
         </is>
       </c>
       <c r="D21" s="23" t="inlineStr">
         <is>
-          <t>São Paulo/SP</t>
+          <t>Salvador/BA</t>
         </is>
       </c>
       <c r="E21" s="23" t="inlineStr">
         <is>
-          <t>BRA1 / Agência VIVA</t>
+          <t>Bahia Notícias</t>
         </is>
       </c>
       <c r="F21" s="23" t="inlineStr">
         <is>
-          <t>https://www.bra1.com.br/geral/id-688491/turn_on_the_light_inaugura_agenda_de_conexoes_entre_futebol_feminino__maternidade_e_causas_sociais_rumo_a_copa_do_mundo_de_2027</t>
+          <t>https://www.bahianoticias.com.br/amp/esportes/noticia/80073-bahia-prepara-sala-lilas-acoes-de-seguranca-e-rdollar-2-mi-para-o-futebol-feminino-na-copa-de-2027-confira-novidades</t>
         </is>
       </c>
       <c r="G21" s="23" t="inlineStr">
@@ -31003,42 +31003,42 @@
       </c>
       <c r="H21" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I21" s="23" t="inlineStr">
         <is>
-          <t>A agência Turn On The Light iniciou uma agenda de encontros e narrativas que conectará futebol feminino, maternidade, carreira e causas sociais até a Copa do Mundo Feminina de 2027. A primeira ação ocorreu na Casa Mãe Paulistana, em São Paulo, com participação da jogadora Tamires, da ex-jogadora Milene Domingues, do comunicador Marco Aurélio e da cantora Gabi Fernandes. A iniciativa pretende usar a preparação para o Mundial como plataforma contínua de engajamento e protagonismo feminino fora dos estádios.</t>
+          <t>A Secretaria de Políticas para as Mulheres da Bahia detalhou medidas de preparação para a Copa do Mundo Feminina 2027 em Salvador, incluindo a implantação de uma Sala Lilás na Arena Fonte Nova para acolhimento de mulheres, certificação da rede turística pelo selo Mulheres Seguras, capacitações e ações de autonomia econômica. O planejamento também inclui edital de R$ 2 milhões com a Sudesb para incentivar torneios femininos no interior e formação voltada à arbitragem feminina, conectando segurança, turismo e legado esportivo do Mundial.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="32" t="n">
-        <v>46266</v>
+        <v>46269</v>
       </c>
       <c r="B22" s="23" t="inlineStr">
         <is>
-          <t>Bahia prepara Sala Lilás e ações de proteção e legado feminino para a Copa 2027</t>
+          <t>Piracicaba reconstrói futebol feminino com foco em ampliar estrutura antes da Copa 2027</t>
         </is>
       </c>
       <c r="C22" s="23" t="inlineStr">
         <is>
-          <t>Salvador / segurança das mulheres / turismo / legado / futebol feminino / Copa 2027</t>
+          <t>Legado / desenvolvimento local / futebol feminino / formação / Copa 2027</t>
         </is>
       </c>
       <c r="D22" s="23" t="inlineStr">
         <is>
-          <t>Salvador/BA</t>
+          <t>Piracicaba/SP</t>
         </is>
       </c>
       <c r="E22" s="23" t="inlineStr">
         <is>
-          <t>Bahia Notícias</t>
+          <t>Jornal de Piracicaba / Sampi</t>
         </is>
       </c>
       <c r="F22" s="23" t="inlineStr">
         <is>
-          <t>https://www.bahianoticias.com.br/amp/esportes/noticia/80073-bahia-prepara-sala-lilas-acoes-de-seguranca-e-rdollar-2-mi-para-o-futebol-feminino-na-copa-de-2027-confira-novidades</t>
+          <t>https://sampi.net.br/campinas/noticias/3002816/cidade/2026/09/piracicaba-busca-reconstruir-futebol-feminino-as-vesperas-da-copa</t>
         </is>
       </c>
       <c r="G22" s="23" t="inlineStr">
@@ -31048,42 +31048,42 @@
       </c>
       <c r="H22" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I22" s="23" t="inlineStr">
         <is>
-          <t>A Secretaria de Políticas para as Mulheres da Bahia detalhou medidas de preparação para a Copa do Mundo Feminina 2027 em Salvador, incluindo a implantação de uma Sala Lilás na Arena Fonte Nova para acolhimento de mulheres, certificação da rede turística pelo selo Mulheres Seguras, capacitações e ações de autonomia econômica. O planejamento também inclui edital de R$ 2 milhões com a Sudesb para incentivar torneios femininos no interior e formação voltada à arbitragem feminina, conectando segurança, turismo e legado esportivo do Mundial.</t>
+          <t>Piracicaba mantém em 2026 um projeto municipal de reconstrução do futebol feminino em parceria com o Caldeirão Futebol Clube, com cerca de 50 atletas a partir de 15 anos, treinamentos gratuitos e investimento de R$ 108 mil. A equipe adulta foi vice-campeã dos Jogos Regionais e garantiu vaga nos Jogos Abertos do Interior, enquanto o planejamento prevê ampliar a estrutura e buscar o retorno às competições estaduais de maior nível em 2027. Gestores locais relacionam a realização da Copa do Mundo Feminina no Brasil à expectativa de maior procura e fortalecimento da modalidade na cidade.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="32" t="n">
-        <v>46269</v>
+        <v>46251</v>
       </c>
       <c r="B23" s="23" t="inlineStr">
         <is>
-          <t>Piracicaba reconstrói futebol feminino com foco em ampliar estrutura antes da Copa 2027</t>
+          <t>Distrito Federal cria grupo de trabalho da Justiça e Cidadania para ações da Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C23" s="23" t="inlineStr">
         <is>
-          <t>Legado / desenvolvimento local / futebol feminino / formação / Copa 2027</t>
+          <t>Brasília / governança / direitos / operação da cidade-sede / Copa 2027</t>
         </is>
       </c>
       <c r="D23" s="23" t="inlineStr">
         <is>
-          <t>Piracicaba/SP</t>
+          <t>Brasília/DF</t>
         </is>
       </c>
       <c r="E23" s="23" t="inlineStr">
         <is>
-          <t>Jornal de Piracicaba / Sampi</t>
+          <t>Diário Oficial do Distrito Federal</t>
         </is>
       </c>
       <c r="F23" s="23" t="inlineStr">
         <is>
-          <t>https://sampi.net.br/campinas/noticias/3002816/cidade/2026/09/piracicaba-busca-reconstruir-futebol-feminino-as-vesperas-da-copa</t>
+          <t>https://www.sinj.df.gov.br/sinj/TextoArquivoDiario.aspx?id_file=afb86271-9977-31e0-ae59-86b99234ddbb</t>
         </is>
       </c>
       <c r="G23" s="23" t="inlineStr">
@@ -31098,42 +31098,42 @@
       </c>
       <c r="I23" s="23" t="inlineStr">
         <is>
-          <t>Piracicaba mantém em 2026 um projeto municipal de reconstrução do futebol feminino em parceria com o Caldeirão Futebol Clube, com cerca de 50 atletas a partir de 15 anos, treinamentos gratuitos e investimento de R$ 108 mil. A equipe adulta foi vice-campeã dos Jogos Regionais e garantiu vaga nos Jogos Abertos do Interior, enquanto o planejamento prevê ampliar a estrutura e buscar o retorno às competições estaduais de maior nível em 2027. Gestores locais relacionam a realização da Copa do Mundo Feminina no Brasil à expectativa de maior procura e fortalecimento da modalidade na cidade.</t>
+          <t>A Secretaria de Estado de Justiça e Cidadania do Distrito Federal instituiu grupo de trabalho para planejar, coordenar, articular, executar, acompanhar e avaliar ações relacionadas à Copa do Mundo Feminina da FIFA Brasil 2027. O grupo deverá elaborar planejamento operacional, articular unidades e instituições, acompanhar cronogramas e resultados e manter integração permanente com a Comissão de Monitoramento e Governança da Copa, reforçando a preparação institucional de Brasília como cidade-sede.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="32" t="n">
-        <v>46251</v>
+        <v>46267</v>
       </c>
       <c r="B24" s="23" t="inlineStr">
         <is>
-          <t>Distrito Federal cria grupo de trabalho da Justiça e Cidadania para ações da Copa Feminina 2027</t>
+          <t>Congresso torna facultativo ajuste das férias escolares durante a Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C24" s="23" t="inlineStr">
         <is>
-          <t>Brasília / governança / direitos / operação da cidade-sede / Copa 2027</t>
+          <t>Legislação / calendário escolar / impacto social / Copa 2027</t>
         </is>
       </c>
       <c r="D24" s="23" t="inlineStr">
         <is>
-          <t>Brasília/DF</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E24" s="23" t="inlineStr">
         <is>
-          <t>Diário Oficial do Distrito Federal</t>
+          <t>Agência Senado / Câmara dos Deputados</t>
         </is>
       </c>
       <c r="F24" s="23" t="inlineStr">
         <is>
-          <t>https://www.sinj.df.gov.br/sinj/TextoArquivoDiario.aspx?id_file=afb86271-9977-31e0-ae59-86b99234ddbb</t>
+          <t>https://www12.senado.leg.br/noticias/senado-agora/2026/09/02/copa-feminina-de-futebol</t>
         </is>
       </c>
       <c r="G24" s="23" t="inlineStr">
         <is>
-          <t>Positivo</t>
+          <t>Neutro</t>
         </is>
       </c>
       <c r="H24" s="23" t="inlineStr">
@@ -31143,87 +31143,87 @@
       </c>
       <c r="I24" s="23" t="inlineStr">
         <is>
-          <t>A Secretaria de Estado de Justiça e Cidadania do Distrito Federal instituiu grupo de trabalho para planejar, coordenar, articular, executar, acompanhar e avaliar ações relacionadas à Copa do Mundo Feminina da FIFA Brasil 2027. O grupo deverá elaborar planejamento operacional, articular unidades e instituições, acompanhar cronogramas e resultados e manter integração permanente com a Comissão de Monitoramento e Governança da Copa, reforçando a preparação institucional de Brasília como cidade-sede.</t>
+          <t>O Senado aprovou em 02/09/2026 o PL 3.481/2026, que torna facultativo o ajuste dos calendários escolares para coincidir com a Copa do Mundo Feminina de 2027. A Câmara havia aprovado o texto em 31/08/2026. A proposta altera a regra da Lei Geral da Copa que previa ajuste obrigatório e segue para sanção presidencial. A mudança afeta a organização social e educacional durante o torneio e pode influenciar a participação de famílias, estudantes e comunidades nas ações ligadas ao Mundial.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="32" t="n">
-        <v>46267</v>
+        <v>46268</v>
       </c>
       <c r="B25" s="23" t="inlineStr">
         <is>
-          <t>Congresso torna facultativo ajuste das férias escolares durante a Copa Feminina 2027</t>
+          <t>Maracanã prepara reforma de R$ 2,5 milhões para adequações da Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C25" s="23" t="inlineStr">
         <is>
-          <t>Legislação / calendário escolar / impacto social / Copa 2027</t>
+          <t>Infraestrutura / estádio-sede / acessibilidade / hospitalidade / Copa 2027</t>
         </is>
       </c>
       <c r="D25" s="23" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Rio de Janeiro/RJ</t>
         </is>
       </c>
       <c r="E25" s="23" t="inlineStr">
         <is>
-          <t>Agência Senado / Câmara dos Deputados</t>
+          <t>ge</t>
         </is>
       </c>
       <c r="F25" s="23" t="inlineStr">
         <is>
-          <t>https://www12.senado.leg.br/noticias/senado-agora/2026/09/02/copa-feminina-de-futebol</t>
+          <t>https://ge.globo.com/futebol/copa-do-mundo-feminina/noticia/2026/09/03/governo-e-consorcio-fla-flu-preparam-reforma-de-r-25-milhoes-em-tribuna-do-maracana-para-a-copa-de-2027.ghtml</t>
         </is>
       </c>
       <c r="G25" s="23" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Positivo</t>
         </is>
       </c>
       <c r="H25" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I25" s="23" t="inlineStr">
         <is>
-          <t>O Senado aprovou em 02/09/2026 o PL 3.481/2026, que torna facultativo o ajuste dos calendários escolares para coincidir com a Copa do Mundo Feminina de 2027. A Câmara havia aprovado o texto em 31/08/2026. A proposta altera a regra da Lei Geral da Copa que previa ajuste obrigatório e segue para sanção presidencial. A mudança afeta a organização social e educacional durante o torneio e pode influenciar a participação de famílias, estudantes e comunidades nas ações ligadas ao Mundial.</t>
+          <t>O Governo do Estado do Rio de Janeiro e o Consórcio Fla-Flu preparam uma reforma estimada em R$ 2,5 milhões na Tribuna de Honra do Maracanã, como parte das adequações para a Copa do Mundo Feminina de 2027. O aditivo contratual prevê melhorias em acessibilidade, hospitalidade, segurança, conforto e funcionalidade, com prazo de execução estimado em 45 dias para a proposta escolhida. O estádio receberá nove partidas do Mundial, incluindo abertura e final.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="32" t="n">
-        <v>46268</v>
+        <v>46265</v>
       </c>
       <c r="B26" s="23" t="inlineStr">
         <is>
-          <t>Maracanã prepara reforma de R$ 2,5 milhões para adequações da Copa Feminina 2027</t>
+          <t>Porto Alegre protocola regras especiais para a Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C26" s="23" t="inlineStr">
         <is>
-          <t>Infraestrutura / estádio-sede / acessibilidade / hospitalidade / Copa 2027</t>
+          <t>Cidade-sede / legislação municipal / mobilidade / ingressos / operação da Copa 2027</t>
         </is>
       </c>
       <c r="D26" s="23" t="inlineStr">
         <is>
-          <t>Rio de Janeiro/RJ</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="E26" s="23" t="inlineStr">
         <is>
-          <t>ge</t>
+          <t>Prefeitura de Porto Alegre</t>
         </is>
       </c>
       <c r="F26" s="23" t="inlineStr">
         <is>
-          <t>https://ge.globo.com/futebol/copa-do-mundo-feminina/noticia/2026/09/03/governo-e-consorcio-fla-flu-preparam-reforma-de-r-25-milhoes-em-tribuna-do-maracana-para-a-copa-de-2027.ghtml</t>
+          <t>https://prefeitura.poa.br/secopa2027/noticias/prefeitura-protocola-projeto-de-lei-com-regras-especiais-para-copa-feminina</t>
         </is>
       </c>
       <c r="G26" s="23" t="inlineStr">
         <is>
-          <t>Positivo</t>
+          <t>Neutro</t>
         </is>
       </c>
       <c r="H26" s="23" t="inlineStr">
@@ -31233,52 +31233,52 @@
       </c>
       <c r="I26" s="23" t="inlineStr">
         <is>
-          <t>O Governo do Estado do Rio de Janeiro e o Consórcio Fla-Flu preparam uma reforma estimada em R$ 2,5 milhões na Tribuna de Honra do Maracanã, como parte das adequações para a Copa do Mundo Feminina de 2027. O aditivo contratual prevê melhorias em acessibilidade, hospitalidade, segurança, conforto e funcionalidade, com prazo de execução estimado em 45 dias para a proposta escolhida. O estádio receberá nove partidas do Mundial, incluindo abertura e final.</t>
+          <t>A Prefeitura de Porto Alegre protocolou o Projeto de Lei nº 028/26 com regras específicas para a realização da Copa do Mundo Feminina FIFA 2027 e seus eventos oficiais. A proposta prevê perímetro temporário de proteção comercial de 1 km no entorno do Beira-Rio, regras exclusivas de ingressos, prioridade de licenciamento, gratuidade no transporte municipal para voluntários e credenciados e coordenação pública da segurança em áreas oficiais. O texto ainda depende de análise e votação pela Câmara Municipal.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="32" t="n">
-        <v>46265</v>
+        <v>46269</v>
       </c>
       <c r="B27" s="23" t="inlineStr">
         <is>
-          <t>Porto Alegre protocola regras especiais para a Copa Feminina 2027</t>
+          <t>Painel em Salvador conecta proteção no esporte e legado da Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C27" s="23" t="inlineStr">
         <is>
-          <t>Cidade-sede / legislação municipal / mobilidade / ingressos / operação da Copa 2027</t>
+          <t>Salvador / safeguarding / legado / formação profissional / Copa 2027</t>
         </is>
       </c>
       <c r="D27" s="23" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Salvador/BA</t>
         </is>
       </c>
       <c r="E27" s="23" t="inlineStr">
         <is>
-          <t>Prefeitura de Porto Alegre</t>
+          <t>Jornal Grande Bahia / GovBA</t>
         </is>
       </c>
       <c r="F27" s="23" t="inlineStr">
         <is>
-          <t>https://prefeitura.poa.br/secopa2027/noticias/prefeitura-protocola-projeto-de-lei-com-regras-especiais-para-copa-feminina</t>
+          <t>https://jornalgrandebahia.com.br/2026/09/futebol-feminino-e-copa-do-mundo-2027-painel-em-salvador-debate-seguranca-e-abre-inscricoes-para-voluntarios/</t>
         </is>
       </c>
       <c r="G27" s="23" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Positivo</t>
         </is>
       </c>
       <c r="H27" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I27" s="23" t="inlineStr">
         <is>
-          <t>A Prefeitura de Porto Alegre protocolou o Projeto de Lei nº 028/26 com regras específicas para a realização da Copa do Mundo Feminina FIFA 2027 e seus eventos oficiais. A proposta prevê perímetro temporário de proteção comercial de 1 km no entorno do Beira-Rio, regras exclusivas de ingressos, prioridade de licenciamento, gratuidade no transporte municipal para voluntários e credenciados e coordenação pública da segurança em áreas oficiais. O texto ainda depende de análise e votação pela Câmara Municipal.</t>
+          <t>Painel Futebol &amp; Cidadania, realizado em 03/09/2026 no Colégio Estadual Professor Rômulo Almeida, em Salvador, reuniu Setre, IPIE, UFBA e comunidade escolar para discutir proteção e prevenção de abusos no esporte, formação profissional e legado ligado à Copa Feminina 2027. O encontro também anunciou mapeamento de projetos de futebol feminino em escolas de tempo integral e apresentou propostas de Centro de Referência do Futebol Feminino e plano estadual de formação para árbitras, treinadoras e gestoras.</t>
         </is>
       </c>
     </row>
@@ -31288,27 +31288,27 @@
       </c>
       <c r="B28" s="23" t="inlineStr">
         <is>
-          <t>Painel em Salvador conecta proteção no esporte e legado da Copa Feminina 2027</t>
+          <t>Formiga destaca potencial da Copa Feminina 2027 para transformar oportunidades de meninas e jogadoras</t>
         </is>
       </c>
       <c r="C28" s="23" t="inlineStr">
         <is>
-          <t>Salvador / safeguarding / legado / formação profissional / Copa 2027</t>
+          <t>Legado / futebol feminino / inspiração / Copa 2027</t>
         </is>
       </c>
       <c r="D28" s="23" t="inlineStr">
         <is>
-          <t>Salvador/BA</t>
+          <t>São Paulo/SP</t>
         </is>
       </c>
       <c r="E28" s="23" t="inlineStr">
         <is>
-          <t>Jornal Grande Bahia / GovBA</t>
+          <t>AFP/BOL</t>
         </is>
       </c>
       <c r="F28" s="23" t="inlineStr">
         <is>
-          <t>https://jornalgrandebahia.com.br/2026/09/futebol-feminino-e-copa-do-mundo-2027-painel-em-salvador-debate-seguranca-e-abre-inscricoes-para-voluntarios/</t>
+          <t>https://www.bol.uol.com.br/noticias/2026/09/04/copa-do-mundo-feminina-no-brasil-pode-mudar-vidas-de-muitas-jogadoras-diz-formiga.htm</t>
         </is>
       </c>
       <c r="G28" s="23" t="inlineStr">
@@ -31323,37 +31323,37 @@
       </c>
       <c r="I28" s="23" t="inlineStr">
         <is>
-          <t>Painel Futebol &amp; Cidadania, realizado em 03/09/2026 no Colégio Estadual Professor Rômulo Almeida, em Salvador, reuniu Setre, IPIE, UFBA e comunidade escolar para discutir proteção e prevenção de abusos no esporte, formação profissional e legado ligado à Copa Feminina 2027. O encontro também anunciou mapeamento de projetos de futebol feminino em escolas de tempo integral e apresentou propostas de Centro de Referência do Futebol Feminino e plano estadual de formação para árbitras, treinadoras e gestoras.</t>
+          <t>Em entrevista à AFP publicada em 04/09/2026, durante o evento Esporte Cria em São Paulo, Formiga afirmou que a Copa do Mundo Feminina de 2027 no Brasil pode mudar a realidade de inúmeras meninas e jogadoras na região. A fala da ex-capitã da Seleção reforça o potencial de legado social e esportivo do torneio e conecta a realização do Mundial à ampliação de oportunidades e visibilidade para o futebol feminino.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="32" t="n">
-        <v>46269</v>
+        <v>46268</v>
       </c>
       <c r="B29" s="23" t="inlineStr">
         <is>
-          <t>Formiga destaca potencial da Copa Feminina 2027 para transformar oportunidades de meninas e jogadoras</t>
+          <t>Futebol feminino bate recordes de transferências internacionais em 2026</t>
         </is>
       </c>
       <c r="C29" s="23" t="inlineStr">
         <is>
-          <t>Legado / futebol feminino / inspiração / Copa 2027</t>
+          <t>Mercado / crescimento / futebol feminino</t>
         </is>
       </c>
       <c r="D29" s="23" t="inlineStr">
         <is>
-          <t>São Paulo/SP</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="E29" s="23" t="inlineStr">
         <is>
-          <t>AFP/BOL</t>
+          <t>FIFA</t>
         </is>
       </c>
       <c r="F29" s="23" t="inlineStr">
         <is>
-          <t>https://www.bol.uol.com.br/noticias/2026/09/04/copa-do-mundo-feminina-no-brasil-pode-mudar-vidas-de-muitas-jogadoras-diz-formiga.htm</t>
+          <t>https://inside.fifa.com/media-releases/world-cup-2026-impact-mid-year-transfer-window</t>
         </is>
       </c>
       <c r="G29" s="23" t="inlineStr">
@@ -31363,12 +31363,12 @@
       </c>
       <c r="H29" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I29" s="23" t="inlineStr">
         <is>
-          <t>Em entrevista à AFP publicada em 04/09/2026, durante o evento Esporte Cria em São Paulo, Formiga afirmou que a Copa do Mundo Feminina de 2027 no Brasil pode mudar a realidade de inúmeras meninas e jogadoras na região. A fala da ex-capitã da Seleção reforça o potencial de legado social e esportivo do torneio e conecta a realização do Mundial à ampliação de oportunidades e visibilidade para o futebol feminino.</t>
+          <t>A FIFA registrou 1.406 transferências internacionais no futebol profissional feminino entre 1º de junho e 2 de setembro de 2026, alta de 19,2% sobre o recorde anterior. Os clubes movimentaram US$ 28,6 milhões em taxas, mais que o dobro da janela equivalente de 2025, confirmando expansão histórica do mercado da modalidade.</t>
         </is>
       </c>
     </row>
@@ -31378,27 +31378,27 @@
       </c>
       <c r="B30" s="23" t="inlineStr">
         <is>
-          <t>Futebol feminino bate recordes de transferências internacionais em 2026</t>
+          <t>Bahia planeja usar a Copa Feminina 2027 para ampliar turismo além de Salvador</t>
         </is>
       </c>
       <c r="C30" s="23" t="inlineStr">
         <is>
-          <t>Mercado / crescimento / futebol feminino</t>
+          <t>Turismo / cidade-sede / legado econômico / infraestrutura aeroportuária</t>
         </is>
       </c>
       <c r="D30" s="23" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Salvador/BA</t>
         </is>
       </c>
       <c r="E30" s="23" t="inlineStr">
         <is>
-          <t>FIFA</t>
+          <t>Let's Go Bahia</t>
         </is>
       </c>
       <c r="F30" s="23" t="inlineStr">
         <is>
-          <t>https://inside.fifa.com/media-releases/world-cup-2026-impact-mid-year-transfer-window</t>
+          <t>https://letsgobahia.com.br/index.php/noticia/radar-por-matheus-pastori/exclusivo-com-mais-de-r-400-milhoes-investidos-bahia-planeja-aproveitar-copa-do-mundo-feminina-para-impulsionar-o-turismo-no-interior</t>
         </is>
       </c>
       <c r="G30" s="23" t="inlineStr">
@@ -31408,12 +31408,12 @@
       </c>
       <c r="H30" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I30" s="23" t="inlineStr">
         <is>
-          <t>A FIFA registrou 1.406 transferências internacionais no futebol profissional feminino entre 1º de junho e 2 de setembro de 2026, alta de 19,2% sobre o recorde anterior. Os clubes movimentaram US$ 28,6 milhões em taxas, mais que o dobro da janela equivalente de 2025, confirmando expansão histórica do mercado da modalidade.</t>
+          <t>Em entrevista publicada em 03/09/2026, o secretário de Turismo da Bahia, Maurício Bacelar, detalhou a estratégia de aproveitar o fluxo gerado pelos sete jogos da Copa Feminina 2027 na Fonte Nova para prolongar a permanência dos visitantes e estimular roteiros no interior. O estado relaciona a preparação a mais de R$ 400 milhões em intervenções aeroportuárias, reforçando o legado turístico e econômico do torneio para além de Salvador.</t>
         </is>
       </c>
     </row>
@@ -31423,27 +31423,27 @@
       </c>
       <c r="B31" s="23" t="inlineStr">
         <is>
-          <t>Bahia planeja usar a Copa Feminina 2027 para ampliar turismo além de Salvador</t>
+          <t>Fortaleza supera 7,3 mil interessados locais no voluntariado da Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C31" s="23" t="inlineStr">
         <is>
-          <t>Turismo / cidade-sede / legado econômico / infraestrutura aeroportuária</t>
+          <t>Voluntariado / engajamento local / cidade-sede</t>
         </is>
       </c>
       <c r="D31" s="23" t="inlineStr">
         <is>
-          <t>Salvador/BA</t>
+          <t>Fortaleza/CE</t>
         </is>
       </c>
       <c r="E31" s="23" t="inlineStr">
         <is>
-          <t>Let's Go Bahia</t>
+          <t>Prefeitura de Fortaleza</t>
         </is>
       </c>
       <c r="F31" s="23" t="inlineStr">
         <is>
-          <t>https://letsgobahia.com.br/index.php/noticia/radar-por-matheus-pastori/exclusivo-com-mais-de-r-400-milhoes-investidos-bahia-planeja-aproveitar-copa-do-mundo-feminina-para-impulsionar-o-turismo-no-interior</t>
+          <t>https://www.fortaleza.ce.gov.br/noticias/fortaleza-mobiliza-voluntarios-para-a-copa-do-mundo-feminina-da-fifa-brasil-2027-e-celebra-abertura-oficial-das-inscricoes</t>
         </is>
       </c>
       <c r="G31" s="23" t="inlineStr">
@@ -31458,7 +31458,7 @@
       </c>
       <c r="I31" s="23" t="inlineStr">
         <is>
-          <t>Em entrevista publicada em 03/09/2026, o secretário de Turismo da Bahia, Maurício Bacelar, detalhou a estratégia de aproveitar o fluxo gerado pelos sete jogos da Copa Feminina 2027 na Fonte Nova para prolongar a permanência dos visitantes e estimular roteiros no interior. O estado relaciona a preparação a mais de R$ 400 milhões em intervenções aeroportuárias, reforçando o legado turístico e econômico do torneio para além de Salvador.</t>
+          <t>A Prefeitura de Fortaleza informou em 03/09/2026 que mais de 7,3 mil pessoas já haviam indicado a capital cearense como cidade-sede de preferência durante a fase de registro de interesse do Programa de Voluntários da Copa do Mundo Feminina 2027. O dado local, divulgado junto à abertura das inscrições oficiais, evidencia forte mobilização e engajamento da população da cidade-sede antes do torneio.</t>
         </is>
       </c>
     </row>
@@ -31468,27 +31468,27 @@
       </c>
       <c r="B32" s="23" t="inlineStr">
         <is>
-          <t>Fortaleza supera 7,3 mil interessados locais no voluntariado da Copa Feminina 2027</t>
+          <t>FIFA abre inscrições oficiais para mais de 6 mil voluntários da Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C32" s="23" t="inlineStr">
         <is>
-          <t>Voluntariado / engajamento local / cidade-sede</t>
+          <t>Voluntariado / engajamento / operação do torneio</t>
         </is>
       </c>
       <c r="D32" s="23" t="inlineStr">
         <is>
-          <t>Fortaleza/CE</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E32" s="23" t="inlineStr">
         <is>
-          <t>Prefeitura de Fortaleza</t>
+          <t>FIFA</t>
         </is>
       </c>
       <c r="F32" s="23" t="inlineStr">
         <is>
-          <t>https://www.fortaleza.ce.gov.br/noticias/fortaleza-mobiliza-voluntarios-para-a-copa-do-mundo-feminina-da-fifa-brasil-2027-e-celebra-abertura-oficial-das-inscricoes</t>
+          <t>https://inside.fifa.com/tournament-organisation/volunteers/media-releases/volunteer-applications-open-womens-world-cup-brazil-2027</t>
         </is>
       </c>
       <c r="G32" s="23" t="inlineStr">
@@ -31498,27 +31498,27 @@
       </c>
       <c r="H32" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I32" s="23" t="inlineStr">
         <is>
-          <t>A Prefeitura de Fortaleza informou em 03/09/2026 que mais de 7,3 mil pessoas já haviam indicado a capital cearense como cidade-sede de preferência durante a fase de registro de interesse do Programa de Voluntários da Copa do Mundo Feminina 2027. O dado local, divulgado junto à abertura das inscrições oficiais, evidencia forte mobilização e engajamento da população da cidade-sede antes do torneio.</t>
+          <t>A FIFA abriu oficialmente em 03/09/2026 as inscrições para o programa de voluntariado da Copa do Mundo Feminina de 2027 no Brasil. Mais de 6 mil voluntários serão recrutados nas oito cidades-sede, após mais de 100 mil manifestações de interesse registradas desde julho. A abertura efetiva das candidaturas é um novo marco operacional e de engajamento, distinto da divulgação anterior das funções disponíveis aos voluntários.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="32" t="n">
-        <v>46268</v>
+        <v>46267</v>
       </c>
       <c r="B33" s="23" t="inlineStr">
         <is>
-          <t>FIFA abre inscrições oficiais para mais de 6 mil voluntários da Copa Feminina 2027</t>
+          <t>Senado aprova prioridade ao futebol feminino e prevê plano de legado da Copa 2027</t>
         </is>
       </c>
       <c r="C33" s="23" t="inlineStr">
         <is>
-          <t>Voluntariado / engajamento / operação do torneio</t>
+          <t>Legislação federal / futebol feminino / legado da Copa 2027</t>
         </is>
       </c>
       <c r="D33" s="23" t="inlineStr">
@@ -31528,12 +31528,12 @@
       </c>
       <c r="E33" s="23" t="inlineStr">
         <is>
-          <t>FIFA</t>
+          <t>Agência Senado</t>
         </is>
       </c>
       <c r="F33" s="23" t="inlineStr">
         <is>
-          <t>https://inside.fifa.com/tournament-organisation/volunteers/media-releases/volunteer-applications-open-womens-world-cup-brazil-2027</t>
+          <t>https://www12.senado.leg.br/noticias/materias/2026/09/02/senado-aprova-prioridade-para-futebol-feminino-na-politica-de-esporte</t>
         </is>
       </c>
       <c r="G33" s="23" t="inlineStr">
@@ -31548,7 +31548,7 @@
       </c>
       <c r="I33" s="23" t="inlineStr">
         <is>
-          <t>A FIFA abriu oficialmente em 03/09/2026 as inscrições para o programa de voluntariado da Copa do Mundo Feminina de 2027 no Brasil. Mais de 6 mil voluntários serão recrutados nas oito cidades-sede, após mais de 100 mil manifestações de interesse registradas desde julho. A abertura efetiva das candidaturas é um novo marco operacional e de engajamento, distinto da divulgação anterior das funções disponíveis aos voluntários.</t>
+          <t>O Senado aprovou projeto que torna o futebol feminino prioridade na política pública esportiva nacional e determina a elaboração de um plano de legado social, esportivo e financeiro da Copa do Mundo Feminina FIFA 2027 no Brasil. O texto também prevê ações para profissionalização, igualdade salarial, participação de mulheres na gestão e arbitragem e combate à discriminação e à violência no esporte.</t>
         </is>
       </c>
     </row>
@@ -31558,12 +31558,12 @@
       </c>
       <c r="B34" s="23" t="inlineStr">
         <is>
-          <t>Senado aprova prioridade ao futebol feminino e prevê plano de legado da Copa 2027</t>
+          <t>SporTV estreia Aquecimento Delas com bancada feminina dedicada ao futebol feminino</t>
         </is>
       </c>
       <c r="C34" s="23" t="inlineStr">
         <is>
-          <t>Legislação federal / futebol feminino / legado da Copa 2027</t>
+          <t>Mídia / futebol feminino / cobertura esportiva</t>
         </is>
       </c>
       <c r="D34" s="23" t="inlineStr">
@@ -31573,12 +31573,12 @@
       </c>
       <c r="E34" s="23" t="inlineStr">
         <is>
-          <t>Agência Senado</t>
+          <t>O Globo</t>
         </is>
       </c>
       <c r="F34" s="23" t="inlineStr">
         <is>
-          <t>https://www12.senado.leg.br/noticias/materias/2026/09/02/senado-aprova-prioridade-para-futebol-feminino-na-politica-de-esporte</t>
+          <t>https://oglobo.globo.com/play/noticia/2026/09/02/nota-10-a-estreia-do-aquecimento-delas-no-sportv.ghtml</t>
         </is>
       </c>
       <c r="G34" s="23" t="inlineStr">
@@ -31588,12 +31588,12 @@
       </c>
       <c r="H34" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I34" s="23" t="inlineStr">
         <is>
-          <t>O Senado aprovou projeto que torna o futebol feminino prioridade na política pública esportiva nacional e determina a elaboração de um plano de legado social, esportivo e financeiro da Copa do Mundo Feminina FIFA 2027 no Brasil. O texto também prevê ações para profissionalização, igualdade salarial, participação de mulheres na gestão e arbitragem e combate à discriminação e à violência no esporte.</t>
+          <t>O SporTV lançou o programa Aquecimento Delas, dedicado ao futebol feminino e apresentado por uma bancada formada por Ana Thais Matos, Renata Mendonça, Mariana Spinelli e Luana Maluf. A iniciativa amplia o espaço permanente de análise e cobertura da modalidade na televisão esportiva em um período de crescente atenção ao futebol feminino antes da Copa do Mundo de 2027 no Brasil.</t>
         </is>
       </c>
     </row>
@@ -31603,12 +31603,12 @@
       </c>
       <c r="B35" s="23" t="inlineStr">
         <is>
-          <t>SporTV estreia Aquecimento Delas com bancada feminina dedicada ao futebol feminino</t>
+          <t>FIFA detalha mais de 30 funções de voluntariado para a Copa do Mundo Feminina 2027</t>
         </is>
       </c>
       <c r="C35" s="23" t="inlineStr">
         <is>
-          <t>Mídia / futebol feminino / cobertura esportiva</t>
+          <t>Voluntariado / operação do torneio / engajamento</t>
         </is>
       </c>
       <c r="D35" s="23" t="inlineStr">
@@ -31618,12 +31618,12 @@
       </c>
       <c r="E35" s="23" t="inlineStr">
         <is>
-          <t>O Globo</t>
+          <t>FIFA</t>
         </is>
       </c>
       <c r="F35" s="23" t="inlineStr">
         <is>
-          <t>https://oglobo.globo.com/play/noticia/2026/09/02/nota-10-a-estreia-do-aquecimento-delas-no-sportv.ghtml</t>
+          <t>https://www.fifa.com/pt/tournaments/womens/womensworldcup/brazil-2027/articles/funcoes-voluntarios-copa-do-mundo-feminina-brasil-2027</t>
         </is>
       </c>
       <c r="G35" s="23" t="inlineStr">
@@ -31633,27 +31633,27 @@
       </c>
       <c r="H35" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I35" s="23" t="inlineStr">
         <is>
-          <t>O SporTV lançou o programa Aquecimento Delas, dedicado ao futebol feminino e apresentado por uma bancada formada por Ana Thais Matos, Renata Mendonça, Mariana Spinelli e Luana Maluf. A iniciativa amplia o espaço permanente de análise e cobertura da modalidade na televisão esportiva em um período de crescente atenção ao futebol feminino antes da Copa do Mundo de 2027 no Brasil.</t>
+          <t>A FIFA detalhou mais de 30 funções previstas para voluntários da Copa do Mundo Feminina de 2027, com atuação em locais oficiais como estádios, hotéis, centros de treinamento e aeroportos. As áreas incluem gestão de acessos, hospedagem, credenciamento, competição, entretenimento, transportes, serviços ao espectador, tecnologia, mídia, hospitalidade, segurança, sustentabilidade, ingressos e operações de estádio.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="32" t="n">
-        <v>46267</v>
+        <v>46265</v>
       </c>
       <c r="B36" s="23" t="inlineStr">
         <is>
-          <t>FIFA detalha mais de 30 funções de voluntariado para a Copa do Mundo Feminina 2027</t>
+          <t>Câmara torna facultativo o ajuste das férias escolares durante a Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C36" s="23" t="inlineStr">
         <is>
-          <t>Voluntariado / operação do torneio / engajamento</t>
+          <t>Legislação federal / educação / calendário escolar / Copa Feminina 2027</t>
         </is>
       </c>
       <c r="D36" s="23" t="inlineStr">
@@ -31663,17 +31663,17 @@
       </c>
       <c r="E36" s="23" t="inlineStr">
         <is>
-          <t>FIFA</t>
+          <t>Agência Câmara</t>
         </is>
       </c>
       <c r="F36" s="23" t="inlineStr">
         <is>
-          <t>https://www.fifa.com/pt/tournaments/womens/womensworldcup/brazil-2027/articles/funcoes-voluntarios-copa-do-mundo-feminina-brasil-2027</t>
+          <t>https://www.camara.leg.br/noticias/1301485-camara-aprova-autonomia-de-escolas-para-ajustar-calendario-na-copa-do-mundo-feminina</t>
         </is>
       </c>
       <c r="G36" s="23" t="inlineStr">
         <is>
-          <t>Positivo</t>
+          <t>Neutro</t>
         </is>
       </c>
       <c r="H36" s="23" t="inlineStr">
@@ -31683,52 +31683,52 @@
       </c>
       <c r="I36" s="23" t="inlineStr">
         <is>
-          <t>A FIFA detalhou mais de 30 funções previstas para voluntários da Copa do Mundo Feminina de 2027, com atuação em locais oficiais como estádios, hotéis, centros de treinamento e aeroportos. As áreas incluem gestão de acessos, hospedagem, credenciamento, competição, entretenimento, transportes, serviços ao espectador, tecnologia, mídia, hospitalidade, segurança, sustentabilidade, ingressos e operações de estádio.</t>
+          <t>A Câmara dos Deputados aprovou o PL 3.481/2026, que torna facultativo aos sistemas de ensino ajustar as férias escolares ao período da Copa do Mundo Feminina 2027. O texto preserva a autonomia das redes, exige o cumprimento da carga horária e dos 200 dias letivos previstos na LDB e foi remetido ao Senado em 1º de setembro de 2026.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="32" t="n">
-        <v>46265</v>
+        <v>46264</v>
       </c>
       <c r="B37" s="23" t="inlineStr">
         <is>
-          <t>Câmara torna facultativo o ajuste das férias escolares durante a Copa Feminina 2027</t>
+          <t>Seleção Feminina Sub-20 chega a Bielsko-Biała para a reta final antes do Mundial</t>
         </is>
       </c>
       <c r="C37" s="23" t="inlineStr">
         <is>
-          <t>Legislação federal / educação / calendário escolar / Copa Feminina 2027</t>
+          <t>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</t>
         </is>
       </c>
       <c r="D37" s="23" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Bielsko-Biała/POL</t>
         </is>
       </c>
       <c r="E37" s="23" t="inlineStr">
         <is>
-          <t>Agência Câmara</t>
+          <t>CBF</t>
         </is>
       </c>
       <c r="F37" s="23" t="inlineStr">
         <is>
-          <t>https://www.camara.leg.br/noticias/1301485-camara-aprova-autonomia-de-escolas-para-ajustar-calendario-na-copa-do-mundo-feminina</t>
+          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-base-feminina/selecao-feminina-sub-20/selecao-feminina-sub-20-chega-a-bielsko-biala-para-reta-final-antes-da-estreia-no-mundial</t>
         </is>
       </c>
       <c r="G37" s="23" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Positivo</t>
         </is>
       </c>
       <c r="H37" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I37" s="23" t="inlineStr">
         <is>
-          <t>A Câmara dos Deputados aprovou o PL 3.481/2026, que torna facultativo aos sistemas de ensino ajustar as férias escolares ao período da Copa do Mundo Feminina 2027. O texto preserva a autonomia das redes, exige o cumprimento da carga horária e dos 200 dias letivos previstos na LDB e foi remetido ao Senado em 1º de setembro de 2026.</t>
+          <t>A Seleção Brasileira Feminina Sub-20 chegou a Bielsko-Biała, na Polônia, para concluir a preparação antes da estreia na Copa do Mundo da categoria. A delegação entra na etapa final de adaptação e treinamentos para o torneio, que começa em 5 de setembro.</t>
         </is>
       </c>
     </row>
@@ -31738,17 +31738,17 @@
       </c>
       <c r="B38" s="23" t="inlineStr">
         <is>
-          <t>Seleção Feminina Sub-20 chega a Bielsko-Biała para a reta final antes do Mundial</t>
+          <t>Thaís Lima destaca integração entre base e Seleção principal antes do Mundial Sub-20</t>
         </is>
       </c>
       <c r="C38" s="23" t="inlineStr">
         <is>
-          <t>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</t>
+          <t>Seleções de Base / Sub-20 Feminina / integração com a Seleção principal</t>
         </is>
       </c>
       <c r="D38" s="23" t="inlineStr">
         <is>
-          <t>Bielsko-Biała/POL</t>
+          <t>Polônia</t>
         </is>
       </c>
       <c r="E38" s="23" t="inlineStr">
@@ -31758,7 +31758,7 @@
       </c>
       <c r="F38" s="23" t="inlineStr">
         <is>
-          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-base-feminina/selecao-feminina-sub-20/selecao-feminina-sub-20-chega-a-bielsko-biala-para-reta-final-antes-da-estreia-no-mundial</t>
+          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/thais-lima-comenta-integracao-entre-as-selecoes-de-base-e-a-principal</t>
         </is>
       </c>
       <c r="G38" s="23" t="inlineStr">
@@ -31773,22 +31773,22 @@
       </c>
       <c r="I38" s="23" t="inlineStr">
         <is>
-          <t>A Seleção Brasileira Feminina Sub-20 chegou a Bielsko-Biała, na Polônia, para concluir a preparação antes da estreia na Copa do Mundo da categoria. A delegação entra na etapa final de adaptação e treinamentos para o torneio, que começa em 5 de setembro.</t>
+          <t>Às vésperas da Copa do Mundo Feminina Sub-20, a atacante Thaís Lima destacou a integração entre as Seleções de base e a equipe principal. A jogadora, que acumula convocações em diferentes categorias, exemplifica a continuidade do processo de formação da CBF durante a preparação do Brasil na Polônia.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="32" t="n">
-        <v>46264</v>
+        <v>46263</v>
       </c>
       <c r="B39" s="23" t="inlineStr">
         <is>
-          <t>Thaís Lima destaca integração entre base e Seleção principal antes do Mundial Sub-20</t>
+          <t>Bianca destaca entrosamento da Seleção Sub-20 antes do Mundial</t>
         </is>
       </c>
       <c r="C39" s="23" t="inlineStr">
         <is>
-          <t>Seleções de Base / Sub-20 Feminina / integração com a Seleção principal</t>
+          <t>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</t>
         </is>
       </c>
       <c r="D39" s="23" t="inlineStr">
@@ -31803,7 +31803,7 @@
       </c>
       <c r="F39" s="23" t="inlineStr">
         <is>
-          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/thais-lima-comenta-integracao-entre-as-selecoes-de-base-e-a-principal</t>
+          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/bianca-relembra-conquista-do-sul-americano-e-valoriza-entrosamento-na-selecao-sub-20</t>
         </is>
       </c>
       <c r="G39" s="23" t="inlineStr">
@@ -31818,37 +31818,37 @@
       </c>
       <c r="I39" s="23" t="inlineStr">
         <is>
-          <t>Às vésperas da Copa do Mundo Feminina Sub-20, a atacante Thaís Lima destacou a integração entre as Seleções de base e a equipe principal. A jogadora, que acumula convocações em diferentes categorias, exemplifica a continuidade do processo de formação da CBF durante a preparação do Brasil na Polônia.</t>
+          <t>A zagueira Bianca relembrou a conquista do Sul-Americano Sub-20 e destacou o entrosamento da Seleção Brasileira durante a preparação na Polônia para a Copa do Mundo Feminina Sub-20 de 2026. A fala reforça a confiança do grupo antes da estreia no Mundial.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="32" t="n">
-        <v>46263</v>
+        <v>46262</v>
       </c>
       <c r="B40" s="23" t="inlineStr">
         <is>
-          <t>Bianca destaca entrosamento da Seleção Sub-20 antes do Mundial</t>
+          <t>Fortaleza avança na Lei da Copa e prepara inspeção da FIFA no Castelão</t>
         </is>
       </c>
       <c r="C40" s="23" t="inlineStr">
         <is>
-          <t>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</t>
+          <t>Preparação de cidade-sede / legislação estadual / mobilidade / Arena Castelão</t>
         </is>
       </c>
       <c r="D40" s="23" t="inlineStr">
         <is>
-          <t>Polônia</t>
+          <t>Fortaleza/CE</t>
         </is>
       </c>
       <c r="E40" s="23" t="inlineStr">
         <is>
-          <t>CBF</t>
+          <t>Diário do Nordeste</t>
         </is>
       </c>
       <c r="F40" s="23" t="inlineStr">
         <is>
-          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/bianca-relembra-conquista-do-sul-americano-e-valoriza-entrosamento-na-selecao-sub-20</t>
+          <t>https://diariodonordeste.verdesmares.com.br/jogada/fortaleza-avanca-na-lei-da-copa-e-prepara-castelao-para-inspecao-da-fifa-a-300-dias-do-mundial-1.3787756</t>
         </is>
       </c>
       <c r="G40" s="23" t="inlineStr">
@@ -31858,12 +31858,12 @@
       </c>
       <c r="H40" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I40" s="23" t="inlineStr">
         <is>
-          <t>A zagueira Bianca relembrou a conquista do Sul-Americano Sub-20 e destacou o entrosamento da Seleção Brasileira durante a preparação na Polônia para a Copa do Mundo Feminina Sub-20 de 2026. A fala reforça a confiança do grupo antes da estreia no Mundial.</t>
+          <t>A 300 dias da Copa do Mundo Feminina 2027, Fortaleza informou que prepara a promulgação da Lei Estadual da Copa, conclui o plano de mobilidade e discute gratuidade no transporte público em dias de jogos. A Arena Castelão, que receberá nove partidas, terá nova inspeção técnica da FIFA em setembro, enquanto Estado, município e federação avançam em infraestrutura, responsabilidade social e legado.</t>
         </is>
       </c>
     </row>
@@ -31873,27 +31873,27 @@
       </c>
       <c r="B41" s="23" t="inlineStr">
         <is>
-          <t>Fortaleza avança na Lei da Copa e prepara inspeção da FIFA no Castelão</t>
+          <t>Dulce transforma experiência no Mundial Sub-17 em preparação para a Seleção Sub-20</t>
         </is>
       </c>
       <c r="C41" s="23" t="inlineStr">
         <is>
-          <t>Preparação de cidade-sede / legislação estadual / mobilidade / Arena Castelão</t>
+          <t>Seleções de Base / Sub-20 Feminina / transição de categoria</t>
         </is>
       </c>
       <c r="D41" s="23" t="inlineStr">
         <is>
-          <t>Fortaleza/CE</t>
+          <t>Cracóvia/POL</t>
         </is>
       </c>
       <c r="E41" s="23" t="inlineStr">
         <is>
-          <t>Diário do Nordeste</t>
+          <t>CBF</t>
         </is>
       </c>
       <c r="F41" s="23" t="inlineStr">
         <is>
-          <t>https://diariodonordeste.verdesmares.com.br/jogada/fortaleza-avanca-na-lei-da-copa-e-prepara-castelao-para-inspecao-da-fifa-a-300-dias-do-mundial-1.3787756</t>
+          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/de-um-mundial-ao-outro-dulce-vive-novo-desafio-com-a-selecao-brasileira</t>
         </is>
       </c>
       <c r="G41" s="23" t="inlineStr">
@@ -31903,12 +31903,12 @@
       </c>
       <c r="H41" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I41" s="23" t="inlineStr">
         <is>
-          <t>A 300 dias da Copa do Mundo Feminina 2027, Fortaleza informou que prepara a promulgação da Lei Estadual da Copa, conclui o plano de mobilidade e discute gratuidade no transporte público em dias de jogos. A Arena Castelão, que receberá nove partidas, terá nova inspeção técnica da FIFA em setembro, enquanto Estado, município e federação avançam em infraestrutura, responsabilidade social e legado.</t>
+          <t>A CBF destacou a trajetória da meio-campista Dulce, que integrou a campanha brasileira de quarto lugar no Mundial Sub-17 de 2025 e agora se prepara na Polônia para disputar sua primeira Copa do Mundo Feminina Sub-20. A atleta do Corinthians chega ao torneio após marcar 12 gols em 15 jogos na temporada e representa a transição da formação para uma categoria mais próxima da Seleção principal.</t>
         </is>
       </c>
     </row>
@@ -31918,27 +31918,27 @@
       </c>
       <c r="B42" s="23" t="inlineStr">
         <is>
-          <t>Dulce transforma experiência no Mundial Sub-17 em preparação para a Seleção Sub-20</t>
+          <t>Empetur abre licitação para infraestrutura temporária da Copa 2027 na Arena Pernambuco</t>
         </is>
       </c>
       <c r="C42" s="23" t="inlineStr">
         <is>
-          <t>Seleções de Base / Sub-20 Feminina / transição de categoria</t>
+          <t>Infraestrutura / Arena Pernambuco / contratação pública</t>
         </is>
       </c>
       <c r="D42" s="23" t="inlineStr">
         <is>
-          <t>Cracóvia/POL</t>
+          <t>Recife/PE</t>
         </is>
       </c>
       <c r="E42" s="23" t="inlineStr">
         <is>
-          <t>CBF</t>
+          <t>Empetur</t>
         </is>
       </c>
       <c r="F42" s="23" t="inlineStr">
         <is>
-          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/de-um-mundial-ao-outro-dulce-vive-novo-desafio-com-a-selecao-brasileira</t>
+          <t>https://www.empetur.pe.gov.br/h-licitacoes/2556-empetur-aviso-de-abertura-processo-n-1687-2026-cel-iii-pe-0008-empetur</t>
         </is>
       </c>
       <c r="G42" s="23" t="inlineStr">
@@ -31953,7 +31953,7 @@
       </c>
       <c r="I42" s="23" t="inlineStr">
         <is>
-          <t>A CBF destacou a trajetória da meio-campista Dulce, que integrou a campanha brasileira de quarto lugar no Mundial Sub-17 de 2025 e agora se prepara na Polônia para disputar sua primeira Copa do Mundo Feminina Sub-20. A atleta do Corinthians chega ao torneio após marcar 12 gols em 15 jogos na temporada e representa a transição da formação para uma categoria mais próxima da Seleção principal.</t>
+          <t>A Empetur abriu disputa para o fornecimento de cadeiras empilháveis destinadas à infraestrutura temporária da Copa do Mundo Feminina FIFA 2027 na Arena Pernambuco. A contratação tem valor máximo estimado de R$ 155.176, com posterior incorporação dos bens ao patrimônio do estádio.</t>
         </is>
       </c>
     </row>
@@ -31963,27 +31963,27 @@
       </c>
       <c r="B43" s="23" t="inlineStr">
         <is>
-          <t>Empetur abre licitação para infraestrutura temporária da Copa 2027 na Arena Pernambuco</t>
+          <t>Lei Complementar destrava benefícios tributários federais para a Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C43" s="23" t="inlineStr">
         <is>
-          <t>Infraestrutura / Arena Pernambuco / contratação pública</t>
+          <t>Tributação / legislação federal / organização</t>
         </is>
       </c>
       <c r="D43" s="23" t="inlineStr">
         <is>
-          <t>Recife/PE</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E43" s="23" t="inlineStr">
         <is>
-          <t>Empetur</t>
+          <t>Presidência da República</t>
         </is>
       </c>
       <c r="F43" s="23" t="inlineStr">
         <is>
-          <t>https://www.empetur.pe.gov.br/h-licitacoes/2556-empetur-aviso-de-abertura-processo-n-1687-2026-cel-iii-pe-0008-empetur</t>
+          <t>https://www.planalto.gov.br/ccivil_03/leis/lcp/lcp235.htm</t>
         </is>
       </c>
       <c r="G43" s="23" t="inlineStr">
@@ -31993,12 +31993,12 @@
       </c>
       <c r="H43" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I43" s="23" t="inlineStr">
         <is>
-          <t>A Empetur abriu disputa para o fornecimento de cadeiras empilháveis destinadas à infraestrutura temporária da Copa do Mundo Feminina FIFA 2027 na Arena Pernambuco. A contratação tem valor máximo estimado de R$ 155.176, com posterior incorporação dos bens ao patrimônio do estádio.</t>
+          <t>Sancionada em 27/08 e publicada em 28/08, a Lei Complementar nº 235/2026 excepciona regras fiscais para viabilizar benefícios tributários federais destinados à realização da Copa do Mundo Feminina FIFA 2027 no Brasil. A medida remove restrições legais à concessão dos incentivos previstos para a organização do torneio.</t>
         </is>
       </c>
     </row>
@@ -32008,27 +32008,27 @@
       </c>
       <c r="B44" s="23" t="inlineStr">
         <is>
-          <t>Lei Complementar destrava benefícios tributários federais para a Copa Feminina 2027</t>
+          <t>Porto Alegre detalha Fan Fest e Caminho das Gurias a 300 dias da Copa 2027</t>
         </is>
       </c>
       <c r="C44" s="23" t="inlineStr">
         <is>
-          <t>Tributação / legislação federal / organização</t>
+          <t>Contagem regressiva / Porto Alegre / Fan Fest / legado</t>
         </is>
       </c>
       <c r="D44" s="23" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="E44" s="23" t="inlineStr">
         <is>
-          <t>Presidência da República</t>
+          <t>Correio do Povo</t>
         </is>
       </c>
       <c r="F44" s="23" t="inlineStr">
         <is>
-          <t>https://www.planalto.gov.br/ccivil_03/leis/lcp/lcp235.htm</t>
+          <t>https://www.correiodopovo.com.br/esportes/300-dias-para-a-copa-feminina-veja-o-que-ja-se-sabe-sobre-o-mundial-1.1743064</t>
         </is>
       </c>
       <c r="G44" s="23" t="inlineStr">
@@ -32038,12 +32038,12 @@
       </c>
       <c r="H44" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I44" s="23" t="inlineStr">
         <is>
-          <t>Sancionada em 27/08 e publicada em 28/08, a Lei Complementar nº 235/2026 excepciona regras fiscais para viabilizar benefícios tributários federais destinados à realização da Copa do Mundo Feminina FIFA 2027 no Brasil. A medida remove restrições legais à concessão dos incentivos previstos para a organização do torneio.</t>
+          <t>A 300 dias da Copa do Mundo Feminina 2027, Porto Alegre informou que prepara Fan Fest, ativações e o Caminho das Gurias, experiência inspirada no Caminho do Gol de 2014. A matéria também consolida os sete jogos no Beira-Rio, o programa de voluntários e a estratégia de levar o legado do torneio a escolas, projetos sociais e comunidades.</t>
         </is>
       </c>
     </row>
@@ -32053,77 +32053,77 @@
       </c>
       <c r="B45" s="23" t="inlineStr">
         <is>
-          <t>Porto Alegre detalha Fan Fest e Caminho das Gurias a 300 dias da Copa 2027</t>
+          <t>Vaquejada e reforma podem tirar fase final da repescagem da Arena Pernambuco</t>
         </is>
       </c>
       <c r="C45" s="23" t="inlineStr">
         <is>
-          <t>Contagem regressiva / Porto Alegre / Fan Fest / legado</t>
+          <t>Repescagem / infraestrutura / cidade-sede</t>
         </is>
       </c>
       <c r="D45" s="23" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Recife/PE</t>
         </is>
       </c>
       <c r="E45" s="23" t="inlineStr">
         <is>
-          <t>Correio do Povo</t>
+          <t>Diário de Pernambuco</t>
         </is>
       </c>
       <c r="F45" s="23" t="inlineStr">
         <is>
-          <t>https://www.correiodopovo.com.br/esportes/300-dias-para-a-copa-feminina-veja-o-que-ja-se-sabe-sobre-o-mundial-1.1743064</t>
+          <t>https://www.diariodepernambuco.com.br/esportes-dp/internacional/2026/08/11722675-vaquejada-pode-tirar-repescagem-da-copa-do-mundo-feminina-da-arena-de-pernambuco.html</t>
         </is>
       </c>
       <c r="G45" s="23" t="inlineStr">
         <is>
-          <t>Positivo</t>
+          <t>Neutro</t>
         </is>
       </c>
       <c r="H45" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I45" s="23" t="inlineStr">
         <is>
-          <t>A 300 dias da Copa do Mundo Feminina 2027, Porto Alegre informou que prepara Fan Fest, ativações e o Caminho das Gurias, experiência inspirada no Caminho do Gol de 2014. A matéria também consolida os sete jogos no Beira-Rio, o programa de voluntários e a estratégia de levar o legado do torneio a escolas, projetos sociais e comunidades.</t>
+          <t>A FIFA solicitou a Arena Pernambuco para a fase final do Torneio Classificatório da Copa Feminina 2027, prevista entre 23 de fevereiro e 6 de março de 2027. Uma vaquejada marcada para novembro de 2026, a substituição do gramado e o cronograma de reformas podem inviabilizar o estádio; as tratativas continuam e outras sedes são avaliadas.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="32" t="n">
-        <v>46262</v>
+        <v>46261</v>
       </c>
       <c r="B46" s="23" t="inlineStr">
         <is>
-          <t>Vaquejada e reforma podem tirar fase final da repescagem da Arena Pernambuco</t>
+          <t>Bahia propõe proteção às mulheres e fórum permanente das cidades-sede para a Copa 2027</t>
         </is>
       </c>
       <c r="C46" s="23" t="inlineStr">
         <is>
-          <t>Repescagem / infraestrutura / cidade-sede</t>
+          <t>Workshop das Cidades-Sede / segurança das mulheres / legado / Salvador</t>
         </is>
       </c>
       <c r="D46" s="23" t="inlineStr">
         <is>
-          <t>Recife/PE</t>
+          <t>Salvador/BA</t>
         </is>
       </c>
       <c r="E46" s="23" t="inlineStr">
         <is>
-          <t>Diário de Pernambuco</t>
+          <t>Bahia Notícias</t>
         </is>
       </c>
       <c r="F46" s="23" t="inlineStr">
         <is>
-          <t>https://www.diariodepernambuco.com.br/esportes-dp/internacional/2026/08/11722675-vaquejada-pode-tirar-repescagem-da-copa-do-mundo-feminina-da-arena-de-pernambuco.html</t>
+          <t>https://www.bahianoticias.com.br/esportes/noticia/80028-protecao-as-mulheres-entra-no-planejamento-da-bahia-para-a-copa-feminina-de-2027</t>
         </is>
       </c>
       <c r="G46" s="23" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Positivo</t>
         </is>
       </c>
       <c r="H46" s="23" t="inlineStr">
@@ -32133,7 +32133,7 @@
       </c>
       <c r="I46" s="23" t="inlineStr">
         <is>
-          <t>A FIFA solicitou a Arena Pernambuco para a fase final do Torneio Classificatório da Copa Feminina 2027, prevista entre 23 de fevereiro e 6 de março de 2027. Uma vaquejada marcada para novembro de 2026, a substituição do gramado e o cronograma de reformas podem inviabilizar o estádio; as tratativas continuam e outras sedes são avaliadas.</t>
+          <t>No Workshop das Cidades-Sede da Copa Feminina 2027, a delegação baiana propôs tornar permanente a ação de vagão exclusivo para mulheres no metrô de Salvador, ampliar as Salas Elas à Frente e criar um fórum contínuo entre as oito sedes para articular mobilidade, segurança e operação do torneio.</t>
         </is>
       </c>
     </row>
@@ -32143,27 +32143,27 @@
       </c>
       <c r="B47" s="23" t="inlineStr">
         <is>
-          <t>Bahia propõe proteção às mulheres e fórum permanente das cidades-sede para a Copa 2027</t>
+          <t>Buscas pela Copa Feminina 2027 impulsionam interesse digital e oportunidades para marcas</t>
         </is>
       </c>
       <c r="C47" s="23" t="inlineStr">
         <is>
-          <t>Workshop das Cidades-Sede / segurança das mulheres / legado / Salvador</t>
+          <t>Marketing / audiência digital / patrocínios / Copa Feminina 2027</t>
         </is>
       </c>
       <c r="D47" s="23" t="inlineStr">
         <is>
-          <t>Salvador/BA</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E47" s="23" t="inlineStr">
         <is>
-          <t>Bahia Notícias</t>
+          <t>Meio &amp; Mensagem</t>
         </is>
       </c>
       <c r="F47" s="23" t="inlineStr">
         <is>
-          <t>https://www.bahianoticias.com.br/esportes/noticia/80028-protecao-as-mulheres-entra-no-planejamento-da-bahia-para-a-copa-feminina-de-2027</t>
+          <t>https://www.meioemensagem.com.br/womentowatch/interesse-pelo-futebol-feminino-dispara-no-digital</t>
         </is>
       </c>
       <c r="G47" s="23" t="inlineStr">
@@ -32173,12 +32173,12 @@
       </c>
       <c r="H47" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I47" s="23" t="inlineStr">
         <is>
-          <t>No Workshop das Cidades-Sede da Copa Feminina 2027, a delegação baiana propôs tornar permanente a ação de vagão exclusivo para mulheres no metrô de Salvador, ampliar as Salas Elas à Frente e criar um fórum contínuo entre as oito sedes para articular mobilidade, segurança e operação do torneio.</t>
+          <t>Estudo divulgado no evento FF.Co mostrou alta de 200% nas buscas brasileiras por futebol feminino no YouTube e de 130% no Google em cinco anos. As dúvidas mais pesquisadas em 2026 incluem sedes, voluntariado, ingressos e transmissão da Copa do Mundo Feminina 2027, reforçando o potencial comercial do torneio para patrocinadores.</t>
         </is>
       </c>
     </row>
@@ -32188,27 +32188,27 @@
       </c>
       <c r="B48" s="23" t="inlineStr">
         <is>
-          <t>Buscas pela Copa Feminina 2027 impulsionam interesse digital e oportunidades para marcas</t>
+          <t>Camilla Orlando avalia ajustes finais da Seleção Sub-20 após primeiro treino na Polônia</t>
         </is>
       </c>
       <c r="C48" s="23" t="inlineStr">
         <is>
-          <t>Marketing / audiência digital / patrocínios / Copa Feminina 2027</t>
+          <t>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</t>
         </is>
       </c>
       <c r="D48" s="23" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Cracóvia/POL</t>
         </is>
       </c>
       <c r="E48" s="23" t="inlineStr">
         <is>
-          <t>Meio &amp; Mensagem</t>
+          <t>CBF</t>
         </is>
       </c>
       <c r="F48" s="23" t="inlineStr">
         <is>
-          <t>https://www.meioemensagem.com.br/womentowatch/interesse-pelo-futebol-feminino-dispara-no-digital</t>
+          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/camilla-orlando-analisa-preparacao-do-brasil-apos-primeiro-treino-para-o-mundial-sub-20-e-o-momento-dos-ajustes-finais</t>
         </is>
       </c>
       <c r="G48" s="23" t="inlineStr">
@@ -32223,7 +32223,7 @@
       </c>
       <c r="I48" s="23" t="inlineStr">
         <is>
-          <t>Estudo divulgado no evento FF.Co mostrou alta de 200% nas buscas brasileiras por futebol feminino no YouTube e de 130% no Google em cinco anos. As dúvidas mais pesquisadas em 2026 incluem sedes, voluntariado, ingressos e transmissão da Copa do Mundo Feminina 2027, reforçando o potencial comercial do torneio para patrocinadores.</t>
+          <t>Após o primeiro treino em campo na Polônia, a técnica Camilla Orlando avaliou a preparação da Seleção Brasileira Feminina Sub-20 para a Copa do Mundo e destacou que a etapa é dedicada aos ajustes finais antes da estreia no torneio.</t>
         </is>
       </c>
     </row>
@@ -32233,27 +32233,27 @@
       </c>
       <c r="B49" s="23" t="inlineStr">
         <is>
-          <t>Camilla Orlando avalia ajustes finais da Seleção Sub-20 após primeiro treino na Polônia</t>
+          <t>Rio propõe benefícios fiscais e metas de legado para a Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C49" s="23" t="inlineStr">
         <is>
-          <t>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</t>
+          <t>Políticas públicas / benefícios fiscais / legado / Rio de Janeiro</t>
         </is>
       </c>
       <c r="D49" s="23" t="inlineStr">
         <is>
-          <t>Cracóvia/POL</t>
+          <t>Rio de Janeiro/RJ</t>
         </is>
       </c>
       <c r="E49" s="23" t="inlineStr">
         <is>
-          <t>CBF</t>
+          <t>Alerj</t>
         </is>
       </c>
       <c r="F49" s="23" t="inlineStr">
         <is>
-          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/camilla-orlando-analisa-preparacao-do-brasil-apos-primeiro-treino-para-o-mundial-sub-20-e-o-momento-dos-ajustes-finais</t>
+          <t>https://www.alerj.rj.gov.br/Visualizar/Noticia/87696</t>
         </is>
       </c>
       <c r="G49" s="23" t="inlineStr">
@@ -32263,12 +32263,12 @@
       </c>
       <c r="H49" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I49" s="23" t="inlineStr">
         <is>
-          <t>Após o primeiro treino em campo na Polônia, a técnica Camilla Orlando avaliou a preparação da Seleção Brasileira Feminina Sub-20 para a Copa do Mundo e destacou que a etapa é dedicada aos ajustes finais antes da estreia no torneio.</t>
+          <t>A Alerj recebeu o Projeto de Lei 8.223/26, que incorpora benefícios de ICMS vinculados à organização da Copa do Mundo Feminina 2027. A proposta estabelece metas de mais de 7.500 empregos diretos no estado, público acumulado superior a 150 mil pessoas nos jogos e compromissos ambientais, com avaliação após o torneio.</t>
         </is>
       </c>
     </row>
@@ -32278,27 +32278,27 @@
       </c>
       <c r="B50" s="23" t="inlineStr">
         <is>
-          <t>Rio propõe benefícios fiscais e metas de legado para a Copa Feminina 2027</t>
+          <t>Vitorinha destaca força de vontade e companheirismo da Seleção Sub-20 para o Mundial</t>
         </is>
       </c>
       <c r="C50" s="23" t="inlineStr">
         <is>
-          <t>Políticas públicas / benefícios fiscais / legado / Rio de Janeiro</t>
+          <t>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</t>
         </is>
       </c>
       <c r="D50" s="23" t="inlineStr">
         <is>
-          <t>Rio de Janeiro/RJ</t>
+          <t>Cracóvia/POL</t>
         </is>
       </c>
       <c r="E50" s="23" t="inlineStr">
         <is>
-          <t>Alerj</t>
+          <t>CBF</t>
         </is>
       </c>
       <c r="F50" s="23" t="inlineStr">
         <is>
-          <t>https://www.alerj.rj.gov.br/Visualizar/Noticia/87696</t>
+          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/vitorinha-celebra-oportunidade-no-mundial-e-destaca-pontos-fortes-do-brasil-para-a-competicao</t>
         </is>
       </c>
       <c r="G50" s="23" t="inlineStr">
@@ -32308,42 +32308,42 @@
       </c>
       <c r="H50" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I50" s="23" t="inlineStr">
         <is>
-          <t>A Alerj recebeu o Projeto de Lei 8.223/26, que incorpora benefícios de ICMS vinculados à organização da Copa do Mundo Feminina 2027. A proposta estabelece metas de mais de 7.500 empregos diretos no estado, público acumulado superior a 150 mil pessoas nos jogos e compromissos ambientais, com avaliação após o torneio.</t>
+          <t>Em preparação na Polônia para a Copa do Mundo Feminina Sub-20, a meio-campista Vitorinha celebrou a oportunidade de disputar o Mundial e apontou força de vontade e companheirismo como pontos fortes da Seleção Brasileira. A atleta também relembrou sua trajetória até a convocação.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="32" t="n">
-        <v>46261</v>
+        <v>46260</v>
       </c>
       <c r="B51" s="23" t="inlineStr">
         <is>
-          <t>Vitorinha destaca força de vontade e companheirismo da Seleção Sub-20 para o Mundial</t>
+          <t>FIFA anuncia Tour da Taça por todas as cidades-sede antes da Copa 2027</t>
         </is>
       </c>
       <c r="C51" s="23" t="inlineStr">
         <is>
-          <t>Seleções de Base / Sub-20 Feminina / preparação para o Mundial</t>
+          <t>Tour da Taça / ativações / EVT-0090</t>
         </is>
       </c>
       <c r="D51" s="23" t="inlineStr">
         <is>
-          <t>Cracóvia/POL</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E51" s="23" t="inlineStr">
         <is>
-          <t>CBF</t>
+          <t>Correio do Povo</t>
         </is>
       </c>
       <c r="F51" s="23" t="inlineStr">
         <is>
-          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/vitorinha-celebra-oportunidade-no-mundial-e-destaca-pontos-fortes-do-brasil-para-a-competicao</t>
+          <t>https://www.correiodopovo.com.br/esportes/taca-da-copa-feminina-fara-tour-pelo-brasil-entre-abril-e-maio-de-2027-1.1742125</t>
         </is>
       </c>
       <c r="G51" s="23" t="inlineStr">
@@ -32353,12 +32353,12 @@
       </c>
       <c r="H51" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I51" s="23" t="inlineStr">
         <is>
-          <t>Em preparação na Polônia para a Copa do Mundo Feminina Sub-20, a meio-campista Vitorinha celebrou a oportunidade de disputar o Mundial e apontou força de vontade e companheirismo como pontos fortes da Seleção Brasileira. A atleta também relembrou sua trajetória até a convocação.</t>
+          <t>Durante o II Workshop de Cidades-Sede e Estádios, a FIFA anunciou o Tour da Taça (EVT-0090) para abril e maio de 2027. O troféu deverá passar pelas oito cidades-sede; datas e locais ainda serão definidos, enquanto Porto Alegre negocia uma permanência de pelo menos cinco dias e exposição no Beira-Rio.</t>
         </is>
       </c>
     </row>
@@ -32368,27 +32368,27 @@
       </c>
       <c r="B52" s="23" t="inlineStr">
         <is>
-          <t>FIFA anuncia Tour da Taça por todas as cidades-sede antes da Copa 2027</t>
+          <t>Porto Alegre mapeia ajustes de infraestrutura no workshop da Copa 2027</t>
         </is>
       </c>
       <c r="C52" s="23" t="inlineStr">
         <is>
-          <t>Tour da Taça / ativações / EVT-0090</t>
+          <t>II Workshop de Cidades-Sede e Estádios / Porto Alegre</t>
         </is>
       </c>
       <c r="D52" s="23" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="E52" s="23" t="inlineStr">
         <is>
-          <t>Correio do Povo</t>
+          <t>Federação Gaúcha de Futebol</t>
         </is>
       </c>
       <c r="F52" s="23" t="inlineStr">
         <is>
-          <t>https://www.correiodopovo.com.br/esportes/taca-da-copa-feminina-fara-tour-pelo-brasil-entre-abril-e-maio-de-2027-1.1742125</t>
+          <t>https://www.fgf.com.br/noticia/fgf-participa-do-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-2027</t>
         </is>
       </c>
       <c r="G52" s="23" t="inlineStr">
@@ -32398,12 +32398,12 @@
       </c>
       <c r="H52" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I52" s="23" t="inlineStr">
         <is>
-          <t>Durante o II Workshop de Cidades-Sede e Estádios, a FIFA anunciou o Tour da Taça (EVT-0090) para abril e maio de 2027. O troféu deverá passar pelas oito cidades-sede; datas e locais ainda serão definidos, enquanto Porto Alegre negocia uma permanência de pelo menos cinco dias e exposição no Beira-Rio.</t>
+          <t>A delegação gaúcha detalhou sua participação no II Workshop de Cidades-Sede e Estádios da Copa 2027. FIFA e CBF realizaram sessões individuais com as sedes para avaliar o planejamento, mapear iniciativas já executadas e indicar ajustes de infraestrutura; Porto Alegre apresentou seu avanço ao lado do Governo do RS, da FGF e do Internacional, responsável pelo Beira-Rio.</t>
         </is>
       </c>
     </row>
@@ -32413,27 +32413,27 @@
       </c>
       <c r="B53" s="23" t="inlineStr">
         <is>
-          <t>Porto Alegre mapeia ajustes de infraestrutura no workshop da Copa 2027</t>
+          <t>Recife integrará programa de voluntários da Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C53" s="23" t="inlineStr">
         <is>
-          <t>II Workshop de Cidades-Sede e Estádios / Porto Alegre</t>
+          <t>Voluntariado / preparação das cidades-sede / Recife</t>
         </is>
       </c>
       <c r="D53" s="23" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Recife/PE</t>
         </is>
       </c>
       <c r="E53" s="23" t="inlineStr">
         <is>
-          <t>Federação Gaúcha de Futebol</t>
+          <t>Folha de Pernambuco</t>
         </is>
       </c>
       <c r="F53" s="23" t="inlineStr">
         <is>
-          <t>https://www.fgf.com.br/noticia/fgf-participa-do-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-2027</t>
+          <t>https://www.folhape.com.br/esportes/copa-feminina-2027-recife-integrara-programa-de-voluntarios/508924/</t>
         </is>
       </c>
       <c r="G53" s="23" t="inlineStr">
@@ -32448,7 +32448,7 @@
       </c>
       <c r="I53" s="23" t="inlineStr">
         <is>
-          <t>A delegação gaúcha detalhou sua participação no II Workshop de Cidades-Sede e Estádios da Copa 2027. FIFA e CBF realizaram sessões individuais com as sedes para avaliar o planejamento, mapear iniciativas já executadas e indicar ajustes de infraestrutura; Porto Alegre apresentou seu avanço ao lado do Governo do RS, da FGF e do Internacional, responsável pelo Beira-Rio.</t>
+          <t>Recife confirmou participação no programa de voluntários da Copa do Mundo Feminina 2027. A seleção oficial para atuar no Mundial está prevista para começar em setembro, ampliando a preparação operacional e o envolvimento da cidade-sede pernambucana.</t>
         </is>
       </c>
     </row>
@@ -32458,27 +32458,27 @@
       </c>
       <c r="B54" s="23" t="inlineStr">
         <is>
-          <t>Recife integrará programa de voluntários da Copa Feminina 2027</t>
+          <t>Seleção Brasileira Sub-20 desembarca na Polônia para o Mundial</t>
         </is>
       </c>
       <c r="C54" s="23" t="inlineStr">
         <is>
-          <t>Voluntariado / preparação das cidades-sede / Recife</t>
+          <t>Seleções de Base / Sub-20 Feminina</t>
         </is>
       </c>
       <c r="D54" s="23" t="inlineStr">
         <is>
-          <t>Recife/PE</t>
+          <t>Bielsko-Biała/POL</t>
         </is>
       </c>
       <c r="E54" s="23" t="inlineStr">
         <is>
-          <t>Folha de Pernambuco</t>
+          <t>CBF</t>
         </is>
       </c>
       <c r="F54" s="23" t="inlineStr">
         <is>
-          <t>https://www.folhape.com.br/esportes/copa-feminina-2027-recife-integrara-programa-de-voluntarios/508924/</t>
+          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/selecao-feminina-sub-20-desembarca-na-polonia-para-disputar-a-copa-do-mundo</t>
         </is>
       </c>
       <c r="G54" s="23" t="inlineStr">
@@ -32493,7 +32493,7 @@
       </c>
       <c r="I54" s="23" t="inlineStr">
         <is>
-          <t>Recife confirmou participação no programa de voluntários da Copa do Mundo Feminina 2027. A seleção oficial para atuar no Mundial está prevista para começar em setembro, ampliando a preparação operacional e o envolvimento da cidade-sede pernambucana.</t>
+          <t>A Seleção Brasileira Feminina Sub-20 chegou à Polônia e iniciou a preparação local para a Copa do Mundo da categoria, que começa em 5 de setembro. O Brasil enfrentará Tanzânia, Canadá e Inglaterra na fase de grupos.</t>
         </is>
       </c>
     </row>
@@ -32503,12 +32503,12 @@
       </c>
       <c r="B55" s="23" t="inlineStr">
         <is>
-          <t>Seleção Brasileira Sub-20 desembarca na Polônia para o Mundial</t>
+          <t>Seleção Feminina Sub-20 inicia adaptação na Polônia após viagem</t>
         </is>
       </c>
       <c r="C55" s="23" t="inlineStr">
         <is>
-          <t>Seleções de Base / Sub-20 Feminina</t>
+          <t>Seleções de Base / Sub-20 Feminina / preparação</t>
         </is>
       </c>
       <c r="D55" s="23" t="inlineStr">
@@ -32523,7 +32523,7 @@
       </c>
       <c r="F55" s="23" t="inlineStr">
         <is>
-          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/selecao-feminina-sub-20-desembarca-na-polonia-para-disputar-a-copa-do-mundo</t>
+          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/com-atividades-no-hotel-selecao-feminina-sub-20-comeca-adaptacao-na-polonia</t>
         </is>
       </c>
       <c r="G55" s="23" t="inlineStr">
@@ -32538,7 +32538,7 @@
       </c>
       <c r="I55" s="23" t="inlineStr">
         <is>
-          <t>A Seleção Brasileira Feminina Sub-20 chegou à Polônia e iniciou a preparação local para a Copa do Mundo da categoria, que começa em 5 de setembro. O Brasil enfrentará Tanzânia, Canadá e Inglaterra na fase de grupos.</t>
+          <t>Em novo capítulo da preparação para a Copa do Mundo Feminina Sub-20, a Seleção Brasileira iniciou em Bielsko-Biała atividades leves de adaptação após a viagem à Polônia, com caminhada, mobilidade e recuperação orientadas pela comissão técnica antes dos treinamentos de campo.</t>
         </is>
       </c>
     </row>
@@ -32548,27 +32548,27 @@
       </c>
       <c r="B56" s="23" t="inlineStr">
         <is>
-          <t>Seleção Feminina Sub-20 inicia adaptação na Polônia após viagem</t>
+          <t>Sportv lança campanha e debate cobertura da Copa 2027 no Festival Feitas de Esporte</t>
         </is>
       </c>
       <c r="C56" s="23" t="inlineStr">
         <is>
-          <t>Seleções de Base / Sub-20 Feminina / preparação</t>
+          <t>Festival Feitas de Esporte / mídia / ativação / Copa Feminina 2027</t>
         </is>
       </c>
       <c r="D56" s="23" t="inlineStr">
         <is>
-          <t>Bielsko-Biała/POL</t>
+          <t>São Paulo/SP</t>
         </is>
       </c>
       <c r="E56" s="23" t="inlineStr">
         <is>
-          <t>CBF</t>
+          <t>Meio &amp; Mensagem</t>
         </is>
       </c>
       <c r="F56" s="23" t="inlineStr">
         <is>
-          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-feminina-sub-20/a/com-atividades-no-hotel-selecao-feminina-sub-20-comeca-adaptacao-na-polonia</t>
+          <t>https://www.meioemensagem.com.br/midia/sportv-faz-evento-para-celebrar-protagonismo-feminino</t>
         </is>
       </c>
       <c r="G56" s="23" t="inlineStr">
@@ -32583,7 +32583,7 @@
       </c>
       <c r="I56" s="23" t="inlineStr">
         <is>
-          <t>Em novo capítulo da preparação para a Copa do Mundo Feminina Sub-20, a Seleção Brasileira iniciou em Bielsko-Biała atividades leves de adaptação após a viagem à Polônia, com caminhada, mobilidade e recuperação orientadas pela comissão técnica antes dos treinamentos de campo.</t>
+          <t>O Sportv anunciou o Festival Feitas de Esporte para 30/08 na Nossa Arena, em São Paulo, com atividades esportivas, lançamento de campanha sobre futebol feminino e debate específico sobre a cobertura do canal para a Copa do Mundo Feminina 2027. O evento relacionado reúne Alline Calandrini, Júlia Vergueiro e convidados e também marca a entrega de novos vestiários.</t>
         </is>
       </c>
     </row>
@@ -32593,87 +32593,87 @@
       </c>
       <c r="B57" s="23" t="inlineStr">
         <is>
-          <t>Sportv lança campanha e debate cobertura da Copa 2027 no Festival Feitas de Esporte</t>
+          <t>UEFA deve retirar ameaça de boicote antes do Mundial Feminino Sub-20</t>
         </is>
       </c>
       <c r="C57" s="23" t="inlineStr">
         <is>
-          <t>Festival Feitas de Esporte / mídia / ativação / Copa Feminina 2027</t>
+          <t>Seleções de Base / Sub-20 Feminina / governança FIFA</t>
         </is>
       </c>
       <c r="D57" s="23" t="inlineStr">
         <is>
-          <t>São Paulo/SP</t>
+          <t>Internacional</t>
         </is>
       </c>
       <c r="E57" s="23" t="inlineStr">
         <is>
-          <t>Meio &amp; Mensagem</t>
+          <t>Folha de S.Paulo / AFP</t>
         </is>
       </c>
       <c r="F57" s="23" t="inlineStr">
         <is>
-          <t>https://www.meioemensagem.com.br/midia/sportv-faz-evento-para-celebrar-protagonismo-feminino</t>
+          <t>https://www1.folha.uol.com.br/esporte/2026/08/uefa-deve-retirar-ameaca-de-boicote-a-torneios-da-fifa.shtml</t>
         </is>
       </c>
       <c r="G57" s="23" t="inlineStr">
         <is>
-          <t>Positivo</t>
+          <t>Neutro</t>
         </is>
       </c>
       <c r="H57" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I57" s="23" t="inlineStr">
         <is>
-          <t>O Sportv anunciou o Festival Feitas de Esporte para 30/08 na Nossa Arena, em São Paulo, com atividades esportivas, lançamento de campanha sobre futebol feminino e debate específico sobre a cobertura do canal para a Copa do Mundo Feminina 2027. O evento relacionado reúne Alline Calandrini, Júlia Vergueiro e convidados e também marca a entrega de novos vestiários.</t>
+          <t>A UEFA deve retirar a ameaça de boicote às competições da FIFA antes da Copa do Mundo Feminina Sub-20 de 2026 na Polônia, torneio que contará com a Seleção Brasileira. O desdobramento reduz a incerteza institucional às vésperas da estreia do Brasil em 5 de setembro.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="32" t="n">
-        <v>46260</v>
+        <v>46259</v>
       </c>
       <c r="B58" s="23" t="inlineStr">
         <is>
-          <t>UEFA deve retirar ameaça de boicote antes do Mundial Feminino Sub-20</t>
+          <t>Acarajé é autorizado dentro da Arena Fonte Nova durante a Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C58" s="23" t="inlineStr">
         <is>
-          <t>Seleções de Base / Sub-20 Feminina / governança FIFA</t>
+          <t>Cultura / turismo / alimentação / Salvador</t>
         </is>
       </c>
       <c r="D58" s="23" t="inlineStr">
         <is>
-          <t>Internacional</t>
+          <t>Salvador/BA</t>
         </is>
       </c>
       <c r="E58" s="23" t="inlineStr">
         <is>
-          <t>Folha de S.Paulo / AFP</t>
+          <t>A TARDE</t>
         </is>
       </c>
       <c r="F58" s="23" t="inlineStr">
         <is>
-          <t>https://www1.folha.uol.com.br/esporte/2026/08/uefa-deve-retirar-ameaca-de-boicote-a-torneios-da-fifa.shtml</t>
+          <t>https://atarde.com.br/bahia/copa-feminina-2027-tera-acaraje-dentro-da-arena-fonte-nova-1399762</t>
         </is>
       </c>
       <c r="G58" s="23" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Positivo</t>
         </is>
       </c>
       <c r="H58" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I58" s="23" t="inlineStr">
         <is>
-          <t>A UEFA deve retirar a ameaça de boicote às competições da FIFA antes da Copa do Mundo Feminina Sub-20 de 2026 na Polônia, torneio que contará com a Seleção Brasileira. O desdobramento reduz a incerteza institucional às vésperas da estreia do Brasil em 5 de setembro.</t>
+          <t>Após articulação do Governo da Bahia, GECOPA, Prefeitura de Salvador e Arena Fonte Nova, as baianas de acarajé foram autorizadas a vender o produto dentro do estádio durante os jogos da Copa Feminina 2027. A decisão integra a estratégia de legado cultural e promoção turística da sede baiana.</t>
         </is>
       </c>
     </row>
@@ -32683,42 +32683,42 @@
       </c>
       <c r="B59" s="23" t="inlineStr">
         <is>
-          <t>Acarajé é autorizado dentro da Arena Fonte Nova durante a Copa Feminina 2027</t>
+          <t>Boicote europeu e meta de premiação pressionam o sorteio da Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C59" s="23" t="inlineStr">
         <is>
-          <t>Cultura / turismo / alimentação / Salvador</t>
+          <t>Sorteio / governança / premiação / EVT-0010</t>
         </is>
       </c>
       <c r="D59" s="23" t="inlineStr">
         <is>
-          <t>Salvador/BA</t>
+          <t>Rio de Janeiro/RJ</t>
         </is>
       </c>
       <c r="E59" s="23" t="inlineStr">
         <is>
-          <t>A TARDE</t>
+          <t>Máquina do Esporte</t>
         </is>
       </c>
       <c r="F59" s="23" t="inlineStr">
         <is>
-          <t>https://atarde.com.br/bahia/copa-feminina-2027-tera-acaraje-dentro-da-arena-fonte-nova-1399762</t>
+          <t>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/boicote-da-uefa-e-premios-em-dinheiro-marcam-sorteio-da-copa-do-mundo-feminina-2027-no-rio/</t>
         </is>
       </c>
       <c r="G59" s="23" t="inlineStr">
         <is>
-          <t>Positivo</t>
+          <t>Neutro</t>
         </is>
       </c>
       <c r="H59" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I59" s="23" t="inlineStr">
         <is>
-          <t>Após articulação do Governo da Bahia, GECOPA, Prefeitura de Salvador e Arena Fonte Nova, as baianas de acarajé foram autorizadas a vender o produto dentro do estádio durante os jogos da Copa Feminina 2027. A decisão integra a estratégia de legado cultural e promoção turística da sede baiana.</t>
+          <t>Em novo desdobramento do sorteio dos grupos (EVT-0010), a FIFA enfrenta ameaça de boicote de países da Uefa e projeta US$ 1 bilhão em receita para a Copa Feminina 2027. Gianni Infantino também prometeu equiparar a premiação do torneio no Brasil à da Copa Masculina de 2026, embora o valor ainda não tenha sido anunciado.</t>
         </is>
       </c>
     </row>
@@ -32728,27 +32728,27 @@
       </c>
       <c r="B60" s="23" t="inlineStr">
         <is>
-          <t>Boicote europeu e meta de premiação pressionam o sorteio da Copa Feminina 2027</t>
+          <t>Conmebol ajusta calendário continental de 2027 para a pausa da Copa Feminina</t>
         </is>
       </c>
       <c r="C60" s="23" t="inlineStr">
         <is>
-          <t>Sorteio / governança / premiação / EVT-0010</t>
+          <t>Calendário continental / clubes / organização</t>
         </is>
       </c>
       <c r="D60" s="23" t="inlineStr">
         <is>
-          <t>Rio de Janeiro/RJ</t>
+          <t>América do Sul / Brasil</t>
         </is>
       </c>
       <c r="E60" s="23" t="inlineStr">
         <is>
-          <t>Máquina do Esporte</t>
+          <t>ge</t>
         </is>
       </c>
       <c r="F60" s="23" t="inlineStr">
         <is>
-          <t>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/boicote-da-uefa-e-premios-em-dinheiro-marcam-sorteio-da-copa-do-mundo-feminina-2027-no-rio/</t>
+          <t>https://ge.globo.com/rs/futebol/noticia/2026/08/25/conmebol-divulga-calendario-de-2027-com-paralisacao-para-copa-do-mundo-feminina.ghtml</t>
         </is>
       </c>
       <c r="G60" s="23" t="inlineStr">
@@ -32763,7 +32763,7 @@
       </c>
       <c r="I60" s="23" t="inlineStr">
         <is>
-          <t>Em novo desdobramento do sorteio dos grupos (EVT-0010), a FIFA enfrenta ameaça de boicote de países da Uefa e projeta US$ 1 bilhão em receita para a Copa Feminina 2027. Gianni Infantino também prometeu equiparar a premiação do torneio no Brasil à da Copa Masculina de 2026, embora o valor ainda não tenha sido anunciado.</t>
+          <t>A Conmebol divulgou o calendário de Libertadores, Sul-Americana e Recopa de 2027 já considerando a paralisação durante a Copa do Mundo Feminina no Brasil. A decisão amplia para as competições continentais o ajuste de calendário que afeta os clubes brasileiros e reduz conflitos durante o Mundial.</t>
         </is>
       </c>
     </row>
@@ -32773,32 +32773,32 @@
       </c>
       <c r="B61" s="23" t="inlineStr">
         <is>
-          <t>Conmebol ajusta calendário continental de 2027 para a pausa da Copa Feminina</t>
+          <t>FIFA projeta Copa Feminina 2027 como primeira edição lucrativa da história</t>
         </is>
       </c>
       <c r="C61" s="23" t="inlineStr">
         <is>
-          <t>Calendário continental / clubes / organização</t>
+          <t>Negócios / audiência / patrocínios</t>
         </is>
       </c>
       <c r="D61" s="23" t="inlineStr">
         <is>
-          <t>América do Sul / Brasil</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E61" s="23" t="inlineStr">
         <is>
-          <t>ge</t>
+          <t>MKT Esportivo</t>
         </is>
       </c>
       <c r="F61" s="23" t="inlineStr">
         <is>
-          <t>https://ge.globo.com/rs/futebol/noticia/2026/08/25/conmebol-divulga-calendario-de-2027-com-paralisacao-para-copa-do-mundo-feminina.ghtml</t>
+          <t>https://www.mktesportivo.com/2026/08/copa-do-mundo-2027-chega-ao-brasil-com-meta-de-lucro-e-maior-interesse-comercial/</t>
         </is>
       </c>
       <c r="G61" s="23" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Positivo</t>
         </is>
       </c>
       <c r="H61" s="23" t="inlineStr">
@@ -32808,7 +32808,7 @@
       </c>
       <c r="I61" s="23" t="inlineStr">
         <is>
-          <t>A Conmebol divulgou o calendário de Libertadores, Sul-Americana e Recopa de 2027 já considerando a paralisação durante a Copa do Mundo Feminina no Brasil. A decisão amplia para as competições continentais o ajuste de calendário que afeta os clubes brasileiros e reduz conflitos durante o Mundial.</t>
+          <t>Em entrevista, Gal Barradas, executiva da FIFA para receitas, marketing e inteligência de negócios da Copa Feminina 2027, afirmou que a entidade projeta a primeira edição lucrativa da história do torneio. O mercado brasileiro, o fuso favorável à audiência internacional e o interesse de marcas sustentam a expectativa comercial.</t>
         </is>
       </c>
     </row>
@@ -32818,87 +32818,87 @@
       </c>
       <c r="B62" s="23" t="inlineStr">
         <is>
-          <t>FIFA projeta Copa Feminina 2027 como primeira edição lucrativa da história</t>
+          <t>Porto Alegre busca amistoso da Seleção antes da Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C62" s="23" t="inlineStr">
         <is>
-          <t>Negócios / audiência / patrocínios</t>
+          <t>Seleção Brasileira / preparação / Porto Alegre</t>
         </is>
       </c>
       <c r="D62" s="23" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="E62" s="23" t="inlineStr">
         <is>
-          <t>MKT Esportivo</t>
+          <t>GZH</t>
         </is>
       </c>
       <c r="F62" s="23" t="inlineStr">
         <is>
-          <t>https://www.mktesportivo.com/2026/08/copa-do-mundo-2027-chega-ao-brasil-com-meta-de-lucro-e-maior-interesse-comercial/</t>
+          <t>https://gauchazh.clicrbs.com.br/esportes/futebol-feminino/noticia/2026/08/uma-das-sedes-da-copa-do-mundo-feminina-de-2027-porto-alegre-ainda-sonha-com-primeiro-jogo-da-selecao-brasileira-cmt7r6ipv00br015gysntaz4r.html</t>
         </is>
       </c>
       <c r="G62" s="23" t="inlineStr">
         <is>
-          <t>Positivo</t>
+          <t>Neutro</t>
         </is>
       </c>
       <c r="H62" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I62" s="23" t="inlineStr">
         <is>
-          <t>Em entrevista, Gal Barradas, executiva da FIFA para receitas, marketing e inteligência de negócios da Copa Feminina 2027, afirmou que a entidade projeta a primeira edição lucrativa da história do torneio. O mercado brasileiro, o fuso favorável à audiência internacional e o interesse de marcas sustentam a expectativa comercial.</t>
+          <t>Sem jogos do Brasil previstos no Beira-Rio durante a Copa Feminina 2027, Porto Alegre tenta receber pela primeira vez a Seleção Feminina em um amistoso preparatório. A CBF confirmou que a capital nunca sediou partida da equipe, e ainda há cinco janelas internacionais antes do Mundial.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="33" t="n">
-        <v>46259</v>
+        <v>46258</v>
       </c>
       <c r="B63" s="23" t="inlineStr">
         <is>
-          <t>Porto Alegre busca amistoso da Seleção antes da Copa Feminina 2027</t>
+          <t>CBF ajusta calendário para preservar mandos dos clubes durante a Copa 2027</t>
         </is>
       </c>
       <c r="C63" s="23" t="inlineStr">
         <is>
-          <t>Seleção Brasileira / preparação / Porto Alegre</t>
+          <t>Calendário / estádios / EVT-0077</t>
         </is>
       </c>
       <c r="D63" s="23" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E63" s="23" t="inlineStr">
         <is>
-          <t>GZH</t>
+          <t>UOL</t>
         </is>
       </c>
       <c r="F63" s="23" t="inlineStr">
         <is>
-          <t>https://gauchazh.clicrbs.com.br/esportes/futebol-feminino/noticia/2026/08/uma-das-sedes-da-copa-do-mundo-feminina-de-2027-porto-alegre-ainda-sonha-com-primeiro-jogo-da-selecao-brasileira-cmt7r6ipv00br015gysntaz4r.html</t>
+          <t>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/cbf-garante-solucao-para-clubes-nao-perderem-mandos-na-copa-feminina.ghtm</t>
         </is>
       </c>
       <c r="G63" s="23" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Positivo</t>
         </is>
       </c>
       <c r="H63" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I63" s="23" t="inlineStr">
         <is>
-          <t>Sem jogos do Brasil previstos no Beira-Rio durante a Copa Feminina 2027, Porto Alegre tenta receber pela primeira vez a Seleção Feminina em um amistoso preparatório. A CBF confirmou que a capital nunca sediou partida da equipe, e ainda há cinco janelas internacionais antes do Mundial.</t>
+          <t>Em desdobramento do período de uso exclusivo dos estádios — incluindo o início da entrega do Maracanã em 10/06/2027, registrado no EVT-0077 — a CBF trabalha para acomodar no calendário os 14 dias anteriores à Copa Feminina 2027 e evitar que clubes percam mandos, receitas ou precisem atuar longe de casa.</t>
         </is>
       </c>
     </row>
@@ -32908,27 +32908,27 @@
       </c>
       <c r="B64" s="23" t="inlineStr">
         <is>
-          <t>CBF ajusta calendário para preservar mandos dos clubes durante a Copa 2027</t>
+          <t>CBF reúne cidades-sede para alinhar operação da Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C64" s="23" t="inlineStr">
         <is>
-          <t>Calendário / estádios / EVT-0077</t>
+          <t>II Workshop de Cidades-Sede / planejamento / EVT-0023</t>
         </is>
       </c>
       <c r="D64" s="23" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Rio de Janeiro/RJ</t>
         </is>
       </c>
       <c r="E64" s="23" t="inlineStr">
         <is>
-          <t>UOL</t>
+          <t>CBF</t>
         </is>
       </c>
       <c r="F64" s="23" t="inlineStr">
         <is>
-          <t>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/cbf-garante-solucao-para-clubes-nao-perderem-mandos-na-copa-feminina.ghtm</t>
+          <t>https://www.cbf.com.br/a-cbf/noticias/por-dentro-cbf-noticias/a/rio-sedia-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-da-fifa-2027</t>
         </is>
       </c>
       <c r="G64" s="23" t="inlineStr">
@@ -32938,12 +32938,12 @@
       </c>
       <c r="H64" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I64" s="23" t="inlineStr">
         <is>
-          <t>Em desdobramento do período de uso exclusivo dos estádios — incluindo o início da entrega do Maracanã em 10/06/2027, registrado no EVT-0077 — a CBF trabalha para acomodar no calendário os 14 dias anteriores à Copa Feminina 2027 e evitar que clubes percam mandos, receitas ou precisem atuar longe de casa.</t>
+          <t>A CBF confirmou a realização do II Workshop de Cidades-Sede e Estádios (EVT-0023), de 24 a 26 de agosto no Rio, reunindo FIFA, CBF, governos e representantes das oito sedes para alinhar temas operacionais, infraestrutura e preparação do Mundial.</t>
         </is>
       </c>
     </row>
@@ -32953,27 +32953,27 @@
       </c>
       <c r="B65" s="23" t="inlineStr">
         <is>
-          <t>CBF reúne cidades-sede para alinhar operação da Copa Feminina 2027</t>
+          <t>Elas Jogam Summit defende legado social, turístico e econômico para a Copa 2027</t>
         </is>
       </c>
       <c r="C65" s="23" t="inlineStr">
         <is>
-          <t>II Workshop de Cidades-Sede / planejamento / EVT-0023</t>
+          <t>Elas Jogam Summit / legado / EVT-0021</t>
         </is>
       </c>
       <c r="D65" s="23" t="inlineStr">
         <is>
-          <t>Rio de Janeiro/RJ</t>
+          <t>São Paulo/SP</t>
         </is>
       </c>
       <c r="E65" s="23" t="inlineStr">
         <is>
-          <t>CBF</t>
+          <t>TV Brasil</t>
         </is>
       </c>
       <c r="F65" s="23" t="inlineStr">
         <is>
-          <t>https://www.cbf.com.br/a-cbf/noticias/por-dentro-cbf-noticias/a/rio-sedia-ii-workshop-de-cidades-sede-e-estadios-da-copa-do-mundo-feminina-da-fifa-2027</t>
+          <t>https://tvbrasil.ebc.com.br/reporter-brasil-tarde/2026/08/museu-do-futebol-sedia-evento-sobre-legado-da-copa-feminina-de-futebol</t>
         </is>
       </c>
       <c r="G65" s="23" t="inlineStr">
@@ -32988,7 +32988,7 @@
       </c>
       <c r="I65" s="23" t="inlineStr">
         <is>
-          <t>A CBF confirmou a realização do II Workshop de Cidades-Sede e Estádios (EVT-0023), de 24 a 26 de agosto no Rio, reunindo FIFA, CBF, governos e representantes das oito sedes para alinhar temas operacionais, infraestrutura e preparação do Mundial.</t>
+          <t>A cobertura pós-evento do Elas Jogam Summit (EVT-0021) destacou a defesa de um legado social, turístico e econômico duradouro para a Copa Feminina 2027, com estruturação da base e fortalecimento do futebol feminino profissional.</t>
         </is>
       </c>
     </row>
@@ -32998,27 +32998,27 @@
       </c>
       <c r="B66" s="23" t="inlineStr">
         <is>
-          <t>Elas Jogam Summit defende legado social, turístico e econômico para a Copa 2027</t>
+          <t>Fortaleza projeta aumento do turismo e da demanda por serviços com a Copa 2027</t>
         </is>
       </c>
       <c r="C66" s="23" t="inlineStr">
         <is>
-          <t>Elas Jogam Summit / legado / EVT-0021</t>
+          <t>Turismo / hotelaria / economia local</t>
         </is>
       </c>
       <c r="D66" s="23" t="inlineStr">
         <is>
-          <t>São Paulo/SP</t>
+          <t>Fortaleza/CE</t>
         </is>
       </c>
       <c r="E66" s="23" t="inlineStr">
         <is>
-          <t>TV Brasil</t>
+          <t>TurisNews</t>
         </is>
       </c>
       <c r="F66" s="23" t="inlineStr">
         <is>
-          <t>https://tvbrasil.ebc.com.br/reporter-brasil-tarde/2026/08/museu-do-futebol-sedia-evento-sobre-legado-da-copa-feminina-de-futebol</t>
+          <t>https://turisnews.com.br/fortaleza-projeta-alta-no-turismo-com-a-copa-feminina-2027/</t>
         </is>
       </c>
       <c r="G66" s="23" t="inlineStr">
@@ -33033,7 +33033,7 @@
       </c>
       <c r="I66" s="23" t="inlineStr">
         <is>
-          <t>A cobertura pós-evento do Elas Jogam Summit (EVT-0021) destacou a defesa de um legado social, turístico e econômico duradouro para a Copa Feminina 2027, com estruturação da base e fortalecimento do futebol feminino profissional.</t>
+          <t>Com nove jogos previstos no Castelão, Fortaleza projeta aumento da demanda por hotelaria, gastronomia, transporte, comércio e serviços durante a Copa Feminina 2027. A cidade recebeu 2,24 milhões de turistas no primeiro semestre de 2026, e o Visite Ceará já mapeou a rede hoteleira segundo os critérios da FIFA.</t>
         </is>
       </c>
     </row>
@@ -33043,12 +33043,12 @@
       </c>
       <c r="B67" s="23" t="inlineStr">
         <is>
-          <t>Fortaleza projeta aumento do turismo e da demanda por serviços com a Copa 2027</t>
+          <t>Sebrae e Sesporte articulam programa de sustentabilidade para o Castelão na Copa 2027</t>
         </is>
       </c>
       <c r="C67" s="23" t="inlineStr">
         <is>
-          <t>Turismo / hotelaria / economia local</t>
+          <t>Sustentabilidade / Fortaleza</t>
         </is>
       </c>
       <c r="D67" s="23" t="inlineStr">
@@ -33058,12 +33058,12 @@
       </c>
       <c r="E67" s="23" t="inlineStr">
         <is>
-          <t>TurisNews</t>
+          <t>Agência Sebrae de Notícias</t>
         </is>
       </c>
       <c r="F67" s="23" t="inlineStr">
         <is>
-          <t>https://turisnews.com.br/fortaleza-projeta-alta-no-turismo-com-a-copa-feminina-2027/</t>
+          <t>https://ce.agenciasebrae.com.br/cultura-empreendedora/sebrae-ce-e-sesporte-discutem-acoes-na-area-da-sustentabilidade/</t>
         </is>
       </c>
       <c r="G67" s="23" t="inlineStr">
@@ -33078,7 +33078,7 @@
       </c>
       <c r="I67" s="23" t="inlineStr">
         <is>
-          <t>Com nove jogos previstos no Castelão, Fortaleza projeta aumento da demanda por hotelaria, gastronomia, transporte, comércio e serviços durante a Copa Feminina 2027. A cidade recebeu 2,24 milhões de turistas no primeiro semestre de 2026, e o Visite Ceará já mapeou a rede hoteleira segundo os critérios da FIFA.</t>
+          <t>Sebrae/CE e Secretaria do Esporte do Ceará iniciaram diálogo para implementar o programa de sustentabilidade e responsabilidade social exigido pela FIFA na Arena Castelão, sede da Copa Feminina 2027, com participação da comunidade e dos pequenos negócios do entorno.</t>
         </is>
       </c>
     </row>
@@ -33088,27 +33088,27 @@
       </c>
       <c r="B68" s="23" t="inlineStr">
         <is>
-          <t>Sebrae e Sesporte articulam programa de sustentabilidade para o Castelão na Copa 2027</t>
+          <t>Sorteio da Copa Feminina 2027 será em 11 de dezembro no MAM Rio</t>
         </is>
       </c>
       <c r="C68" s="23" t="inlineStr">
         <is>
-          <t>Sustentabilidade / Fortaleza</t>
+          <t>Sorteio / calendário / EVT-0010</t>
         </is>
       </c>
       <c r="D68" s="23" t="inlineStr">
         <is>
-          <t>Fortaleza/CE</t>
+          <t>Rio de Janeiro/RJ</t>
         </is>
       </c>
       <c r="E68" s="23" t="inlineStr">
         <is>
-          <t>Agência Sebrae de Notícias</t>
+          <t>UOL</t>
         </is>
       </c>
       <c r="F68" s="23" t="inlineStr">
         <is>
-          <t>https://ce.agenciasebrae.com.br/cultura-empreendedora/sebrae-ce-e-sesporte-discutem-acoes-na-area-da-sustentabilidade/</t>
+          <t>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/sorteio-da-copa-do-mundo-feminina-2027-sera-em-11-de-dezembro-no-mam-rio.ghtm</t>
         </is>
       </c>
       <c r="G68" s="23" t="inlineStr">
@@ -33118,42 +33118,42 @@
       </c>
       <c r="H68" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I68" s="23" t="inlineStr">
         <is>
-          <t>Sebrae/CE e Secretaria do Esporte do Ceará iniciaram diálogo para implementar o programa de sustentabilidade e responsabilidade social exigido pela FIFA na Arena Castelão, sede da Copa Feminina 2027, com participação da comunidade e dos pequenos negócios do entorno.</t>
+          <t>A FIFA confirmou que o sorteio final dos grupos da Copa Feminina 2027 será realizado em 11/12/2026 no Museu de Arte Moderna do Rio. O anúncio atualiza o EVT-0010 e antecipa um evento para mais de mil convidados, que definirá os grupos e o caminho das 32 seleções.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="33" t="n">
-        <v>46258</v>
+        <v>46257</v>
       </c>
       <c r="B69" s="23" t="inlineStr">
         <is>
-          <t>Sorteio da Copa Feminina 2027 será em 11 de dezembro no MAM Rio</t>
+          <t>Coca-Cola confirma patrocínio e prepara presença de peso na Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C69" s="23" t="inlineStr">
         <is>
-          <t>Sorteio / calendário / EVT-0010</t>
+          <t>Patrocínio / negócios</t>
         </is>
       </c>
       <c r="D69" s="23" t="inlineStr">
         <is>
-          <t>Rio de Janeiro/RJ</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E69" s="23" t="inlineStr">
         <is>
-          <t>UOL</t>
+          <t>Exame</t>
         </is>
       </c>
       <c r="F69" s="23" t="inlineStr">
         <is>
-          <t>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/24/sorteio-da-copa-do-mundo-feminina-2027-sera-em-11-de-dezembro-no-mam-rio.ghtm</t>
+          <t>https://exame.com/negocios/vamos-patrocinar-a-copa-do-mundo-feminina-2027-diz-presidente-da-coca-cola-brasil/</t>
         </is>
       </c>
       <c r="G69" s="23" t="inlineStr">
@@ -33168,7 +33168,7 @@
       </c>
       <c r="I69" s="23" t="inlineStr">
         <is>
-          <t>A FIFA confirmou que o sorteio final dos grupos da Copa Feminina 2027 será realizado em 11/12/2026 no Museu de Arte Moderna do Rio. O anúncio atualiza o EVT-0010 e antecipa um evento para mais de mil convidados, que definirá os grupos e o caminho das 32 seleções.</t>
+          <t>A presidente da Coca-Cola Brasil confirmou que a companhia patrocinará a Copa do Mundo Feminina 2027 no Brasil e pretende ter presença comparável à adotada no Mundial masculino. A empresa prepara ativações para o torneio e ampliou sua atuação no futebol nacional por meio de novos acordos com a CBF.</t>
         </is>
       </c>
     </row>
@@ -33178,27 +33178,27 @@
       </c>
       <c r="B70" s="23" t="inlineStr">
         <is>
-          <t>Coca-Cola confirma patrocínio e prepara presença de peso na Copa Feminina 2027</t>
+          <t>Rio envia à Alerj projeto de isenção de ICMS para a Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C70" s="23" t="inlineStr">
         <is>
-          <t>Patrocínio / negócios</t>
+          <t>Tributação / organização / políticas públicas</t>
         </is>
       </c>
       <c r="D70" s="23" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Rio de Janeiro/RJ</t>
         </is>
       </c>
       <c r="E70" s="23" t="inlineStr">
         <is>
-          <t>Exame</t>
+          <t>Governo do Estado do Rio de Janeiro</t>
         </is>
       </c>
       <c r="F70" s="23" t="inlineStr">
         <is>
-          <t>https://exame.com/negocios/vamos-patrocinar-a-copa-do-mundo-feminina-2027-diz-presidente-da-coca-cola-brasil/</t>
+          <t>https://www.rj.gov.br/radioroquettepinto/node/20221</t>
         </is>
       </c>
       <c r="G70" s="23" t="inlineStr">
@@ -33213,37 +33213,37 @@
       </c>
       <c r="I70" s="23" t="inlineStr">
         <is>
-          <t>A presidente da Coca-Cola Brasil confirmou que a companhia patrocinará a Copa do Mundo Feminina 2027 no Brasil e pretende ter presença comparável à adotada no Mundial masculino. A empresa prepara ativações para o torneio e ampliou sua atuação no futebol nacional por meio de novos acordos com a CBF.</t>
+          <t>O Governo do Rio encaminhou à Alerj projeto para incorporar à legislação estadual a isenção e a suspensão de ICMS previstas pelo Confaz em operações e prestações ligadas à organização da Copa Feminina 2027. A proposta, protocolada em 21/08, busca viabilizar a desoneração tributária das atividades do torneio no estado.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="33" t="n">
-        <v>46257</v>
+        <v>46256</v>
       </c>
       <c r="B71" s="23" t="inlineStr">
         <is>
-          <t>Rio envia à Alerj projeto de isenção de ICMS para a Copa Feminina 2027</t>
+          <t>Copa Salvador Interbairros amplia participação feminina e premia campeãs com R$ 40 mil</t>
         </is>
       </c>
       <c r="C71" s="23" t="inlineStr">
         <is>
-          <t>Tributação / organização / políticas públicas</t>
+          <t>Copa Salvador Interbairros / legado / EVT-0064</t>
         </is>
       </c>
       <c r="D71" s="23" t="inlineStr">
         <is>
-          <t>Rio de Janeiro/RJ</t>
+          <t>Salvador/BA</t>
         </is>
       </c>
       <c r="E71" s="23" t="inlineStr">
         <is>
-          <t>Governo do Estado do Rio de Janeiro</t>
+          <t>Correio</t>
         </is>
       </c>
       <c r="F71" s="23" t="inlineStr">
         <is>
-          <t>https://www.rj.gov.br/radioroquettepinto/node/20221</t>
+          <t>https://www.correio24horas.com.br/salvador/copa-salvador-interbairros-2026-tera-r-40-mil-para-campeoes-e-comeca-dia-30-veja-novidades-0826</t>
         </is>
       </c>
       <c r="G71" s="23" t="inlineStr">
@@ -33253,42 +33253,42 @@
       </c>
       <c r="H71" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I71" s="23" t="inlineStr">
         <is>
-          <t>O Governo do Rio encaminhou à Alerj projeto para incorporar à legislação estadual a isenção e a suspensão de ICMS previstas pelo Confaz em operações e prestações ligadas à organização da Copa Feminina 2027. A proposta, protocolada em 21/08, busca viabilizar a desoneração tributária das atividades do torneio no estado.</t>
+          <t>A Copa Salvador Interbairros (EVT-0064) reunirá cerca de 1,2 mil atletas, incluindo dez equipes femininas, e distribuirá R$ 40 mil aos campeões das categorias Livre masculina e feminina. A Prefeitura apresenta a competição como legado comunitário para a Copa 2027.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="33" t="n">
-        <v>46256</v>
+        <v>46255</v>
       </c>
       <c r="B72" s="23" t="inlineStr">
         <is>
-          <t>Copa Salvador Interbairros amplia participação feminina e premia campeãs com R$ 40 mil</t>
+          <t>Elas Jogam Summit reúne atletas e especialistas para discutir o legado da Copa 2027</t>
         </is>
       </c>
       <c r="C72" s="23" t="inlineStr">
         <is>
-          <t>Copa Salvador Interbairros / legado / EVT-0064</t>
+          <t>Elas Jogam Summit / legado</t>
         </is>
       </c>
       <c r="D72" s="23" t="inlineStr">
         <is>
-          <t>Salvador/BA</t>
+          <t>São Paulo/SP</t>
         </is>
       </c>
       <c r="E72" s="23" t="inlineStr">
         <is>
-          <t>Correio</t>
+          <t>Folha de S.Paulo</t>
         </is>
       </c>
       <c r="F72" s="23" t="inlineStr">
         <is>
-          <t>https://www.correio24horas.com.br/salvador/copa-salvador-interbairros-2026-tera-r-40-mil-para-campeoes-e-comeca-dia-30-veja-novidades-0826</t>
+          <t>https://www1.folha.uol.com.br/colunas/monicabergamo/2026/08/tamires-fala-sobre-copa-do-mundo-feminina-de-2027-no-museu-do-futebol.shtml</t>
         </is>
       </c>
       <c r="G72" s="23" t="inlineStr">
@@ -33303,37 +33303,37 @@
       </c>
       <c r="I72" s="23" t="inlineStr">
         <is>
-          <t>A Copa Salvador Interbairros (EVT-0064) reunirá cerca de 1,2 mil atletas, incluindo dez equipes femininas, e distribuirá R$ 40 mil aos campeões das categorias Livre masculina e feminina. A Prefeitura apresenta a competição como legado comunitário para a Copa 2027.</t>
+          <t>A cobertura antecipou o Elas Jogam Summit no Museu do Futebol, destacando debates sobre formação, comunicação, mercado, investimento, memória e transformação social como parte do legado da Copa Feminina 2027, além de uma oficina para meninas da periferia de São Paulo.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="33" t="n">
-        <v>46255</v>
+        <v>46254</v>
       </c>
       <c r="B73" s="23" t="inlineStr">
         <is>
-          <t>Elas Jogam Summit reúne atletas e especialistas para discutir o legado da Copa 2027</t>
+          <t>Arthur Elias diz que Seleção está 70% definida e vê vantagem na abertura no Maracanã</t>
         </is>
       </c>
       <c r="C73" s="23" t="inlineStr">
         <is>
-          <t>Elas Jogam Summit / legado</t>
+          <t>Seleção Brasileira / preparação</t>
         </is>
       </c>
       <c r="D73" s="23" t="inlineStr">
         <is>
-          <t>São Paulo/SP</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E73" s="23" t="inlineStr">
         <is>
-          <t>Folha de S.Paulo</t>
+          <t>ge</t>
         </is>
       </c>
       <c r="F73" s="23" t="inlineStr">
         <is>
-          <t>https://www1.folha.uol.com.br/colunas/monicabergamo/2026/08/tamires-fala-sobre-copa-do-mundo-feminina-de-2027-no-museu-do-futebol.shtml</t>
+          <t>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/20/arthur-elias-diz-que-selecao-esta-70percent-fechada-para-a-copa-e-que-marta-tem-ano-desafiador.ghtml</t>
         </is>
       </c>
       <c r="G73" s="23" t="inlineStr">
@@ -33348,7 +33348,7 @@
       </c>
       <c r="I73" s="23" t="inlineStr">
         <is>
-          <t>A cobertura antecipou o Elas Jogam Summit no Museu do Futebol, destacando debates sobre formação, comunicação, mercado, investimento, memória e transformação social como parte do legado da Copa Feminina 2027, além de uma oficina para meninas da periferia de São Paulo.</t>
+          <t>Após a divulgação da tabela da Copa Feminina 2027, o técnico Arthur Elias afirmou que cerca de 70% do grupo da Seleção está definido, manteve Marta nos planos e avaliou que abrir o torneio no Maracanã representa vantagem para o Brasil.</t>
         </is>
       </c>
     </row>
@@ -33358,12 +33358,12 @@
       </c>
       <c r="B74" s="23" t="inlineStr">
         <is>
-          <t>Arthur Elias diz que Seleção está 70% definida e vê vantagem na abertura no Maracanã</t>
+          <t>FIFA abre cadastro de interesse para ingressos da Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C74" s="23" t="inlineStr">
         <is>
-          <t>Seleção Brasileira / preparação</t>
+          <t>Ingressos / relacionamento</t>
         </is>
       </c>
       <c r="D74" s="23" t="inlineStr">
@@ -33373,17 +33373,17 @@
       </c>
       <c r="E74" s="23" t="inlineStr">
         <is>
-          <t>ge</t>
+          <t>UOL</t>
         </is>
       </c>
       <c r="F74" s="23" t="inlineStr">
         <is>
-          <t>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/20/arthur-elias-diz-que-selecao-esta-70percent-fechada-para-a-copa-e-que-marta-tem-ano-desafiador.ghtml</t>
+          <t>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/20/copa-2027-venda-de-ingressos-ainda-nao-comecou-como-registrar-interesse.ghtm</t>
         </is>
       </c>
       <c r="G74" s="23" t="inlineStr">
         <is>
-          <t>Positivo</t>
+          <t>Neutro</t>
         </is>
       </c>
       <c r="H74" s="23" t="inlineStr">
@@ -33393,7 +33393,7 @@
       </c>
       <c r="I74" s="23" t="inlineStr">
         <is>
-          <t>Após a divulgação da tabela da Copa Feminina 2027, o técnico Arthur Elias afirmou que cerca de 70% do grupo da Seleção está definido, manteve Marta nos planos e avaliou que abrir o torneio no Maracanã representa vantagem para o Brasil.</t>
+          <t>A venda de ingressos ainda não começou e não há data oficial de abertura; torcedores já podem registrar interesse no portal da FIFA para receber atualizações.</t>
         </is>
       </c>
     </row>
@@ -33403,12 +33403,12 @@
       </c>
       <c r="B75" s="23" t="inlineStr">
         <is>
-          <t>FIFA abre cadastro de interesse para ingressos da Copa Feminina 2027</t>
+          <t>FIFA divulga tabela-base da Copa 2027 e confirma Maracanã na abertura e final</t>
         </is>
       </c>
       <c r="C75" s="23" t="inlineStr">
         <is>
-          <t>Ingressos / relacionamento</t>
+          <t>Calendário / sedes</t>
         </is>
       </c>
       <c r="D75" s="23" t="inlineStr">
@@ -33418,27 +33418,27 @@
       </c>
       <c r="E75" s="23" t="inlineStr">
         <is>
-          <t>UOL</t>
+          <t>FIFA</t>
         </is>
       </c>
       <c r="F75" s="23" t="inlineStr">
         <is>
-          <t>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/20/copa-2027-venda-de-ingressos-ainda-nao-comecou-como-registrar-interesse.ghtm</t>
+          <t>https://www.fifa.com/pt/articles/tabela-jogos-copa-feminina-divulgacao-maracana-final-abertura</t>
         </is>
       </c>
       <c r="G75" s="23" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Positivo</t>
         </is>
       </c>
       <c r="H75" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I75" s="23" t="inlineStr">
         <is>
-          <t>A venda de ingressos ainda não começou e não há data oficial de abertura; torcedores já podem registrar interesse no portal da FIFA para receber atualizações.</t>
+          <t>Tabela-base confirma 64 jogos entre 24/06 e 25/07/2027, abertura e final no Maracanã e partidas do Brasil no Rio, em São Paulo e em Brasília.</t>
         </is>
       </c>
     </row>
@@ -33448,12 +33448,12 @@
       </c>
       <c r="B76" s="23" t="inlineStr">
         <is>
-          <t>FIFA divulga tabela-base da Copa 2027 e confirma Maracanã na abertura e final</t>
+          <t>Governo prevê aporte mínimo de R$ 1,5 bilhão para organizar a Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C76" s="23" t="inlineStr">
         <is>
-          <t>Calendário / sedes</t>
+          <t>Investimentos públicos / segurança / infraestrutura</t>
         </is>
       </c>
       <c r="D76" s="23" t="inlineStr">
@@ -33463,17 +33463,17 @@
       </c>
       <c r="E76" s="23" t="inlineStr">
         <is>
-          <t>FIFA</t>
+          <t>Folha de S.Paulo</t>
         </is>
       </c>
       <c r="F76" s="23" t="inlineStr">
         <is>
-          <t>https://www.fifa.com/pt/articles/tabela-jogos-copa-feminina-divulgacao-maracana-final-abertura</t>
+          <t>https://www1.folha.uol.com.br/esporte/2026/08/brasil-joga-na-fase-de-grupos-da-copa-feminina-em-sao-paulo-rio-e-brasilia.shtml</t>
         </is>
       </c>
       <c r="G76" s="23" t="inlineStr">
         <is>
-          <t>Positivo</t>
+          <t>Neutro</t>
         </is>
       </c>
       <c r="H76" s="23" t="inlineStr">
@@ -33483,7 +33483,7 @@
       </c>
       <c r="I76" s="23" t="inlineStr">
         <is>
-          <t>Tabela-base confirma 64 jogos entre 24/06 e 25/07/2027, abertura e final no Maracanã e partidas do Brasil no Rio, em São Paulo e em Brasília.</t>
+          <t>Ao detalhar o calendário e o caminho da Seleção na Copa Feminina 2027, a Folha informou que o governo federal estima aporte mínimo de R$ 1,5 bilhão. Os recursos devem atender segurança pública, telecomunicações, promoção do torneio e construção do legado nas oito cidades-sede.</t>
         </is>
       </c>
     </row>
@@ -33493,12 +33493,12 @@
       </c>
       <c r="B77" s="23" t="inlineStr">
         <is>
-          <t>Governo prevê aporte mínimo de R$ 1,5 bilhão para organizar a Copa Feminina 2027</t>
+          <t>Sorteio define caminhos da fase preliminar da repescagem mundial</t>
         </is>
       </c>
       <c r="C77" s="23" t="inlineStr">
         <is>
-          <t>Investimentos públicos / segurança / infraestrutura</t>
+          <t>Repescagem / sorteio</t>
         </is>
       </c>
       <c r="D77" s="23" t="inlineStr">
@@ -33508,12 +33508,12 @@
       </c>
       <c r="E77" s="23" t="inlineStr">
         <is>
-          <t>Folha de S.Paulo</t>
+          <t>FIFA</t>
         </is>
       </c>
       <c r="F77" s="23" t="inlineStr">
         <is>
-          <t>https://www1.folha.uol.com.br/esporte/2026/08/brasil-joga-na-fase-de-grupos-da-copa-feminina-em-sao-paulo-rio-e-brasilia.shtml</t>
+          <t>https://www.fifa.com/pt/tournaments/womens/womensworldcup/brazil-2027/articles/resultados-sorteio-fase-preliminar-torneio-classificatorio-fifa-brasil-2027</t>
         </is>
       </c>
       <c r="G77" s="23" t="inlineStr">
@@ -33528,27 +33528,27 @@
       </c>
       <c r="I77" s="23" t="inlineStr">
         <is>
-          <t>Ao detalhar o calendário e o caminho da Seleção na Copa Feminina 2027, a Folha informou que o governo federal estima aporte mínimo de R$ 1,5 bilhão. Os recursos devem atender segurança pública, telecomunicações, promoção do torneio e construção do legado nas oito cidades-sede.</t>
+          <t>FIFA definiu a ordem dos confrontos entre Uzbequistão, África do Sul, Papua-Nova Guiné, Taipé Chinês, Gana e Equador; a fase será disputada de 24/11 a 05/12/2026.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="33" t="n">
-        <v>46254</v>
+        <v>46253</v>
       </c>
       <c r="B78" s="23" t="inlineStr">
         <is>
-          <t>Sorteio define caminhos da fase preliminar da repescagem mundial</t>
+          <t>Brasil confirma convocadas para a Copa do Mundo Feminina Sub-20</t>
         </is>
       </c>
       <c r="C78" s="23" t="inlineStr">
         <is>
-          <t>Repescagem / sorteio</t>
+          <t>Seleções de Base / Sub-20 Feminina</t>
         </is>
       </c>
       <c r="D78" s="23" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Brasil / Polônia</t>
         </is>
       </c>
       <c r="E78" s="23" t="inlineStr">
@@ -33558,22 +33558,22 @@
       </c>
       <c r="F78" s="23" t="inlineStr">
         <is>
-          <t>https://www.fifa.com/pt/tournaments/womens/womensworldcup/brazil-2027/articles/resultados-sorteio-fase-preliminar-torneio-classificatorio-fifa-brasil-2027</t>
+          <t>https://www.fifa.com/pt/articles/brasil-convocadas-copa-do-mundo-feminina-sub-20-2026</t>
         </is>
       </c>
       <c r="G78" s="23" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Positivo</t>
         </is>
       </c>
       <c r="H78" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I78" s="23" t="inlineStr">
         <is>
-          <t>FIFA definiu a ordem dos confrontos entre Uzbequistão, África do Sul, Papua-Nova Guiné, Taipé Chinês, Gana e Equador; a fase será disputada de 24/11 a 05/12/2026.</t>
+          <t>A lista brasileira para o Mundial Feminino Sub-20 de 2026 foi confirmada. A equipe de Camilla Orlando se apresenta antes do embarque e estreia contra a Tanzânia em 5 de setembro, seguida por Canadá e Inglaterra.</t>
         </is>
       </c>
     </row>
@@ -33583,42 +33583,42 @@
       </c>
       <c r="B79" s="23" t="inlineStr">
         <is>
-          <t>Brasil confirma convocadas para a Copa do Mundo Feminina Sub-20</t>
+          <t>CNE limita férias escolares da Copa Feminina 2027 às cidades-sede e vizinhas</t>
         </is>
       </c>
       <c r="C79" s="23" t="inlineStr">
         <is>
-          <t>Seleções de Base / Sub-20 Feminina</t>
+          <t>Políticas públicas / educação</t>
         </is>
       </c>
       <c r="D79" s="23" t="inlineStr">
         <is>
-          <t>Brasil / Polônia</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E79" s="23" t="inlineStr">
         <is>
-          <t>FIFA</t>
+          <t>UOL</t>
         </is>
       </c>
       <c r="F79" s="23" t="inlineStr">
         <is>
-          <t>https://www.fifa.com/pt/articles/brasil-convocadas-copa-do-mundo-feminina-sub-20-2026</t>
+          <t>https://educacao.uol.com.br/noticias/2026/08/19/conselho-ferias-copa-do-mundo-futebol-feminina.ghtm</t>
         </is>
       </c>
       <c r="G79" s="23" t="inlineStr">
         <is>
-          <t>Positivo</t>
+          <t>Neutro</t>
         </is>
       </c>
       <c r="H79" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I79" s="23" t="inlineStr">
         <is>
-          <t>A lista brasileira para o Mundial Feminino Sub-20 de 2026 foi confirmada. A equipe de Camilla Orlando se apresenta antes do embarque e estreia contra a Tanzânia em 5 de setembro, seguida por Canadá e Inglaterra.</t>
+          <t>O Conselho Nacional de Educação decidiu que a obrigação de férias durante a Copa Feminina 2027 deve alcançar somente as oito cidades-sede e municípios vizinhos; o parecer ainda depende de homologação do Ministério da Educação e afeta o planejamento do ano letivo.</t>
         </is>
       </c>
     </row>
@@ -33628,12 +33628,12 @@
       </c>
       <c r="B80" s="23" t="inlineStr">
         <is>
-          <t>CNE limita férias escolares da Copa Feminina 2027 às cidades-sede e vizinhas</t>
+          <t>Supermercados entram no planejamento comercial para a Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C80" s="23" t="inlineStr">
         <is>
-          <t>Políticas públicas / educação</t>
+          <t>Varejo / consumo / oportunidades comerciais</t>
         </is>
       </c>
       <c r="D80" s="23" t="inlineStr">
@@ -33643,57 +33643,57 @@
       </c>
       <c r="E80" s="23" t="inlineStr">
         <is>
-          <t>UOL</t>
+          <t>Revista Super Negócios / ASSERJ</t>
         </is>
       </c>
       <c r="F80" s="23" t="inlineStr">
         <is>
-          <t>https://educacao.uol.com.br/noticias/2026/08/19/conselho-ferias-copa-do-mundo-futebol-feminina.ghtm</t>
+          <t>https://asserj.com.br/en/w/copa-do-mundo-feminina-entra-no-radar-dos-supermercados</t>
         </is>
       </c>
       <c r="G80" s="23" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Positivo</t>
         </is>
       </c>
       <c r="H80" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I80" s="23" t="inlineStr">
         <is>
-          <t>O Conselho Nacional de Educação decidiu que a obrigação de férias durante a Copa Feminina 2027 deve alcançar somente as oito cidades-sede e municípios vizinhos; o parecer ainda depende de homologação do Ministério da Educação e afeta o planejamento do ano letivo.</t>
+          <t>A Associação de Supermercados do Estado do Rio de Janeiro aponta a Copa Feminina 2027 como oportunidade para o varejo alimentar, com foco no consumo doméstico e familiar, cestas mais diversificadas e ativações comerciais. A análise cita 750 mil interessados em ingressos e a projeção de R$ 8,8 bilhões movimentados pelo torneio.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="33" t="n">
-        <v>46253</v>
+        <v>46252</v>
       </c>
       <c r="B81" s="23" t="inlineStr">
         <is>
-          <t>Supermercados entram no planejamento comercial para a Copa Feminina 2027</t>
+          <t>Painel em Brasília defende estrutura duradoura como legado da Copa 2027</t>
         </is>
       </c>
       <c r="C81" s="23" t="inlineStr">
         <is>
-          <t>Varejo / consumo / oportunidades comerciais</t>
+          <t>Elas em Ação / legado / EVT-0081</t>
         </is>
       </c>
       <c r="D81" s="23" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Brasília/DF</t>
         </is>
       </c>
       <c r="E81" s="23" t="inlineStr">
         <is>
-          <t>Revista Super Negócios / ASSERJ</t>
+          <t>FSports</t>
         </is>
       </c>
       <c r="F81" s="23" t="inlineStr">
         <is>
-          <t>https://asserj.com.br/en/w/copa-do-mundo-feminina-entra-no-radar-dos-supermercados</t>
+          <t>https://pt.linkedin.com/posts/fsports-ag_o-legado-come%C3%A7a-antes-do-primeiro-apito-activity-7495445214967484417-5m11</t>
         </is>
       </c>
       <c r="G81" s="23" t="inlineStr">
@@ -33708,37 +33708,37 @@
       </c>
       <c r="I81" s="23" t="inlineStr">
         <is>
-          <t>A Associação de Supermercados do Estado do Rio de Janeiro aponta a Copa Feminina 2027 como oportunidade para o varejo alimentar, com foco no consumo doméstico e familiar, cestas mais diversificadas e ativações comerciais. A análise cita 750 mil interessados em ingressos e a projeção de R$ 8,8 bilhões movimentados pelo torneio.</t>
+          <t>No painel “Esporte como Arena de Poder” do Elas em Ação (EVT-0081), Juliana Picoli Agatte e Ruskaya Zanini defenderam que a Copa Feminina 2027 deixe estrutura para clubes e atletas, amplie a participação de meninas, mantenha marcas investindo e coloque mais mulheres em posições de decisão.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="33" t="n">
-        <v>46252</v>
+        <v>46251</v>
       </c>
       <c r="B82" s="23" t="inlineStr">
         <is>
-          <t>Painel em Brasília defende estrutura duradoura como legado da Copa 2027</t>
+          <t>Brasil convoca Seleção Feminina Sub-15 para a Liga Evolução</t>
         </is>
       </c>
       <c r="C82" s="23" t="inlineStr">
         <is>
-          <t>Elas em Ação / legado / EVT-0081</t>
+          <t>Seleções de Base / Sub-15 Feminina</t>
         </is>
       </c>
       <c r="D82" s="23" t="inlineStr">
         <is>
-          <t>Brasília/DF</t>
+          <t>Assunção/PRY</t>
         </is>
       </c>
       <c r="E82" s="23" t="inlineStr">
         <is>
-          <t>FSports</t>
+          <t>CBF</t>
         </is>
       </c>
       <c r="F82" s="23" t="inlineStr">
         <is>
-          <t>https://pt.linkedin.com/posts/fsports-ag_o-legado-come%C3%A7a-antes-do-primeiro-apito-activity-7495445214967484417-5m11</t>
+          <t>https://www.cbf.com.br/selecao-brasileira/noticias/convocacoes-selecao-feminina-sub-15/a/beatriz-vaz-convoca-20-atletas-para-liga-evolucao-sub-15-da-conmebol</t>
         </is>
       </c>
       <c r="G82" s="23" t="inlineStr">
@@ -33753,7 +33753,7 @@
       </c>
       <c r="I82" s="23" t="inlineStr">
         <is>
-          <t>No painel “Esporte como Arena de Poder” do Elas em Ação (EVT-0081), Juliana Picoli Agatte e Ruskaya Zanini defenderam que a Copa Feminina 2027 deixe estrutura para clubes e atletas, amplie a participação de meninas, mantenha marcas investindo e coloque mais mulheres em posições de decisão.</t>
+          <t>Bia Vaz convocou 20 atletas para defender a Seleção Brasileira Feminina Sub-15 na Liga Evolução da CONMEBOL, de 8 a 20 de setembro no Paraguai, em busca do bicampeonato.</t>
         </is>
       </c>
     </row>
@@ -33763,27 +33763,27 @@
       </c>
       <c r="B83" s="23" t="inlineStr">
         <is>
-          <t>Brasil convoca Seleção Feminina Sub-15 para a Liga Evolução</t>
+          <t>FIFA e FPF alinham preparativos da Copa do Mundo Feminina</t>
         </is>
       </c>
       <c r="C83" s="23" t="inlineStr">
         <is>
-          <t>Seleções de Base / Sub-15 Feminina</t>
+          <t>Operação / cidade-sede</t>
         </is>
       </c>
       <c r="D83" s="23" t="inlineStr">
         <is>
-          <t>Assunção/PRY</t>
+          <t>Recife/PE</t>
         </is>
       </c>
       <c r="E83" s="23" t="inlineStr">
         <is>
-          <t>CBF</t>
+          <t>Tribuna Online</t>
         </is>
       </c>
       <c r="F83" s="23" t="inlineStr">
         <is>
-          <t>https://www.cbf.com.br/selecao-brasileira/noticias/convocacoes-selecao-feminina-sub-15/a/beatriz-vaz-convoca-20-atletas-para-liga-evolucao-sub-15-da-conmebol</t>
+          <t>https://tribunaonline.com.br/pernambuco/esporte/fpf-recebe-comitiva-da-fifa-para-alinhar-preparativos-da-copa-do-mundo-feminina-328649</t>
         </is>
       </c>
       <c r="G83" s="23" t="inlineStr">
@@ -33793,12 +33793,12 @@
       </c>
       <c r="H83" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I83" s="23" t="inlineStr">
         <is>
-          <t>Bia Vaz convocou 20 atletas para defender a Seleção Brasileira Feminina Sub-15 na Liga Evolução da CONMEBOL, de 8 a 20 de setembro no Paraguai, em busca do bicampeonato.</t>
+          <t>Reunião institucional reforçou integração da sede pernambucana com as áreas responsáveis pela organização do Mundial.</t>
         </is>
       </c>
     </row>
@@ -33808,72 +33808,72 @@
       </c>
       <c r="B84" s="23" t="inlineStr">
         <is>
-          <t>FIFA e FPF alinham preparativos da Copa do Mundo Feminina</t>
+          <t>Tamires cobra mobilização das cidades-sede para lotar a Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C84" s="23" t="inlineStr">
         <is>
-          <t>Operação / cidade-sede</t>
+          <t>Elas Jogam Summit / público / legado / EVT-0021</t>
         </is>
       </c>
       <c r="D84" s="23" t="inlineStr">
         <is>
-          <t>Recife/PE</t>
+          <t>São Paulo/SP</t>
         </is>
       </c>
       <c r="E84" s="23" t="inlineStr">
         <is>
-          <t>Tribuna Online</t>
+          <t>UOL</t>
         </is>
       </c>
       <c r="F84" s="23" t="inlineStr">
         <is>
-          <t>https://tribunaonline.com.br/pernambuco/esporte/fpf-recebe-comitiva-da-fifa-para-alinhar-preparativos-da-copa-do-mundo-feminina-328649</t>
+          <t>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/17/copa-2027-tamires-pede-engajamento-das-cidades-sede-para-lotar-estadios.ghtm</t>
         </is>
       </c>
       <c r="G84" s="23" t="inlineStr">
         <is>
-          <t>Positivo</t>
+          <t>Neutro</t>
         </is>
       </c>
       <c r="H84" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I84" s="23" t="inlineStr">
         <is>
-          <t>Reunião institucional reforçou integração da sede pernambucana com as áreas responsáveis pela organização do Mundial.</t>
+          <t>Em entrevista durante evento em São Paulo ligado ao debate de legado do Elas Jogam Summit (EVT-0021), Tamires defendeu estratégias locais nas oito cidades-sede para encher os 64 jogos da Copa Feminina 2027. A FIFA pretende superar dois milhões de espectadores e acompanha ações de promoção, Fan Fests e centros de treinamento.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="33" t="n">
-        <v>46251</v>
+        <v>46248</v>
       </c>
       <c r="B85" s="23" t="inlineStr">
         <is>
-          <t>Tamires cobra mobilização das cidades-sede para lotar a Copa Feminina 2027</t>
+          <t>FIFA confirma evento de 20/08 para revelar calendário e sorteio da repescagem</t>
         </is>
       </c>
       <c r="C85" s="23" t="inlineStr">
         <is>
-          <t>Elas Jogam Summit / público / legado / EVT-0021</t>
+          <t>Calendário / sorteio</t>
         </is>
       </c>
       <c r="D85" s="23" t="inlineStr">
         <is>
-          <t>São Paulo/SP</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E85" s="23" t="inlineStr">
         <is>
-          <t>UOL</t>
+          <t>ge</t>
         </is>
       </c>
       <c r="F85" s="23" t="inlineStr">
         <is>
-          <t>https://www.uol.com.br/esporte/futebol/ultimas-noticias/2026/08/17/copa-2027-tamires-pede-engajamento-das-cidades-sede-para-lotar-estadios.ghtm</t>
+          <t>https://ge.globo.com/futebol/copa-do-mundo-feminina/noticia/2026/08/14/copa-do-mundo-2027-calendario-sera-revelado-dia-20-de-agosto.ghtml</t>
         </is>
       </c>
       <c r="G85" s="23" t="inlineStr">
@@ -33883,12 +33883,12 @@
       </c>
       <c r="H85" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I85" s="23" t="inlineStr">
         <is>
-          <t>Em entrevista durante evento em São Paulo ligado ao debate de legado do Elas Jogam Summit (EVT-0021), Tamires defendeu estratégias locais nas oito cidades-sede para encher os 64 jogos da Copa Feminina 2027. A FIFA pretende superar dois milhões de espectadores e acompanha ações de promoção, Fan Fests e centros de treinamento.</t>
+          <t>Em 20/08 serão anunciados distribuição de jogos por sede, locais dos jogos do Brasil e confrontos da fase preliminar da repescagem.</t>
         </is>
       </c>
     </row>
@@ -33898,32 +33898,32 @@
       </c>
       <c r="B86" s="23" t="inlineStr">
         <is>
-          <t>FIFA confirma evento de 20/08 para revelar calendário e sorteio da repescagem</t>
+          <t>FIFA reúne marcas no SP2B para discutir ativações da Copa 2027</t>
         </is>
       </c>
       <c r="C86" s="23" t="inlineStr">
         <is>
-          <t>Calendário / sorteio</t>
+          <t>Patrocínio / ativações</t>
         </is>
       </c>
       <c r="D86" s="23" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>São Paulo/SP</t>
         </is>
       </c>
       <c r="E86" s="23" t="inlineStr">
         <is>
-          <t>ge</t>
+          <t>UOL</t>
         </is>
       </c>
       <c r="F86" s="23" t="inlineStr">
         <is>
-          <t>https://ge.globo.com/futebol/copa-do-mundo-feminina/noticia/2026/08/14/copa-do-mundo-2027-calendario-sera-revelado-dia-20-de-agosto.ghtml</t>
+          <t>https://economia.uol.com.br/noticias/redacao/2026/08/14/copa-do-mundo-feminina-alcanca-750-mil-interessados-em-ingressos.ghtm</t>
         </is>
       </c>
       <c r="G86" s="23" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Positivo</t>
         </is>
       </c>
       <c r="H86" s="23" t="inlineStr">
@@ -33933,7 +33933,7 @@
       </c>
       <c r="I86" s="23" t="inlineStr">
         <is>
-          <t>Em 20/08 serão anunciados distribuição de jogos por sede, locais dos jogos do Brasil e confrontos da fase preliminar da repescagem.</t>
+          <t>Encontro no SP2B discutiu oportunidades comerciais e estratégias de ativação com patrocinadores e executivos.</t>
         </is>
       </c>
     </row>
@@ -33943,27 +33943,27 @@
       </c>
       <c r="B87" s="23" t="inlineStr">
         <is>
-          <t>FIFA reúne marcas no SP2B para discutir ativações da Copa 2027</t>
+          <t>Sesc RJ amplia turmas gratuitas de futebol feminino com foco no legado da Copa 2027</t>
         </is>
       </c>
       <c r="C87" s="23" t="inlineStr">
         <is>
-          <t>Patrocínio / ativações</t>
+          <t>Legado / formação de base / inclusão esportiva</t>
         </is>
       </c>
       <c r="D87" s="23" t="inlineStr">
         <is>
-          <t>São Paulo/SP</t>
+          <t>Diversas cidades/RJ</t>
         </is>
       </c>
       <c r="E87" s="23" t="inlineStr">
         <is>
-          <t>UOL</t>
+          <t>Sesc RJ</t>
         </is>
       </c>
       <c r="F87" s="23" t="inlineStr">
         <is>
-          <t>https://economia.uol.com.br/noticias/redacao/2026/08/14/copa-do-mundo-feminina-alcanca-750-mil-interessados-em-ingressos.ghtm</t>
+          <t>https://www.sescrio.org.br/noticias/esporte/em-clima-de-copa-2027-sesc-rj-amplia-turmas-gratuitas-de-futebol-feminino/</t>
         </is>
       </c>
       <c r="G87" s="23" t="inlineStr">
@@ -33973,42 +33973,42 @@
       </c>
       <c r="H87" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I87" s="23" t="inlineStr">
         <is>
-          <t>Encontro no SP2B discutiu oportunidades comerciais e estratégias de ativação com patrocinadores e executivos.</t>
+          <t>Em iniciativa vinculada ao legado da Copa do Mundo Feminina 2027, o Sesc RJ ampliou as turmas gratuitas de futebol feminino para meninas de 7 a 17 anos. O projeto alcança unidades na capital e em Petrópolis, Nova Iguaçu, São João de Meriti, Niterói e São Gonçalo, com foco em acesso ao esporte, permanência na prática e formação de novas atletas.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="33" t="n">
-        <v>46248</v>
+        <v>46247</v>
       </c>
       <c r="B88" s="23" t="inlineStr">
         <is>
-          <t>Sesc RJ amplia turmas gratuitas de futebol feminino com foco no legado da Copa 2027</t>
+          <t>Base feminina soma 206 atletas convocadas e três desafios internacionais</t>
         </is>
       </c>
       <c r="C88" s="23" t="inlineStr">
         <is>
-          <t>Legado / formação de base / inclusão esportiva</t>
+          <t>Seleções de Base / Sub-15, Sub-17 e Sub-20 Femininas</t>
         </is>
       </c>
       <c r="D88" s="23" t="inlineStr">
         <is>
-          <t>Diversas cidades/RJ</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E88" s="23" t="inlineStr">
         <is>
-          <t>Sesc RJ</t>
+          <t>CBF</t>
         </is>
       </c>
       <c r="F88" s="23" t="inlineStr">
         <is>
-          <t>https://www.sescrio.org.br/noticias/esporte/em-clima-de-copa-2027-sesc-rj-amplia-turmas-gratuitas-de-futebol-feminino/</t>
+          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-base-feminina/a/campeas-continentais-e-mais-de-200-atletas-convocadas-conquistas-e-numeros-do-atual-ciclo-da-base-feminina</t>
         </is>
       </c>
       <c r="G88" s="23" t="inlineStr">
@@ -34023,22 +34023,22 @@
       </c>
       <c r="I88" s="23" t="inlineStr">
         <is>
-          <t>Em iniciativa vinculada ao legado da Copa do Mundo Feminina 2027, o Sesc RJ ampliou as turmas gratuitas de futebol feminino para meninas de 7 a 17 anos. O projeto alcança unidades na capital e em Petrópolis, Nova Iguaçu, São João de Meriti, Niterói e São Gonçalo, com foco em acesso ao esporte, permanência na prática e formação de novas atletas.</t>
+          <t>A CBF apresentou o balanço do ciclo das Seleções Femininas de Base: 206 atletas convocadas, 47 jogos, 32 vitórias e 68% de aproveitamento. Sub-15, Sub-17 e Sub-20 terão competições internacionais no segundo semestre de 2026.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="33" t="n">
-        <v>46247</v>
+        <v>46246</v>
       </c>
       <c r="B89" s="23" t="inlineStr">
         <is>
-          <t>Base feminina soma 206 atletas convocadas e três desafios internacionais</t>
+          <t>Atricon apoia revisão das férias escolares obrigatórias durante a Copa 2027</t>
         </is>
       </c>
       <c r="C89" s="23" t="inlineStr">
         <is>
-          <t>Seleções de Base / Sub-15, Sub-17 e Sub-20 Femininas</t>
+          <t>Políticas públicas / educação</t>
         </is>
       </c>
       <c r="D89" s="23" t="inlineStr">
@@ -34048,17 +34048,17 @@
       </c>
       <c r="E89" s="23" t="inlineStr">
         <is>
-          <t>CBF</t>
+          <t>Folha de S.Paulo</t>
         </is>
       </c>
       <c r="F89" s="23" t="inlineStr">
         <is>
-          <t>https://www.cbf.com.br/selecao-brasileira/noticias/selecao-base-feminina/a/campeas-continentais-e-mais-de-200-atletas-convocadas-conquistas-e-numeros-do-atual-ciclo-da-base-feminina</t>
+          <t>https://www1.folha.uol.com.br/colunas/painel/2026/08/associacao-de-tribunais-de-contas-se-opoe-a-ferias-escolares-obrigatorias-na-copa-do-mundo-feminina.shtml</t>
         </is>
       </c>
       <c r="G89" s="23" t="inlineStr">
         <is>
-          <t>Positivo</t>
+          <t>Neutro</t>
         </is>
       </c>
       <c r="H89" s="23" t="inlineStr">
@@ -34068,22 +34068,22 @@
       </c>
       <c r="I89" s="23" t="inlineStr">
         <is>
-          <t>A CBF apresentou o balanço do ciclo das Seleções Femininas de Base: 206 atletas convocadas, 47 jogos, 32 vitórias e 68% de aproveitamento. Sub-15, Sub-17 e Sub-20 terão competições internacionais no segundo semestre de 2026.</t>
+          <t>A Atricon enviou ofícios à Câmara e ao Senado apoiando projeto que revoga a obrigatoriedade de férias escolares durante a Copa Feminina 2027, argumentando que a regra pode prejudicar calendários pedagógicos, transporte e alimentação escolar em regiões sem jogos.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="33" t="n">
-        <v>46246</v>
+        <v>46239</v>
       </c>
       <c r="B90" s="23" t="inlineStr">
         <is>
-          <t>Atricon apoia revisão das férias escolares obrigatórias durante a Copa 2027</t>
+          <t>CBF determina pausa nacional durante toda a Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C90" s="23" t="inlineStr">
         <is>
-          <t>Políticas públicas / educação</t>
+          <t>Calendário / competições nacionais</t>
         </is>
       </c>
       <c r="D90" s="23" t="inlineStr">
@@ -34093,12 +34093,12 @@
       </c>
       <c r="E90" s="23" t="inlineStr">
         <is>
-          <t>Folha de S.Paulo</t>
+          <t>ge</t>
         </is>
       </c>
       <c r="F90" s="23" t="inlineStr">
         <is>
-          <t>https://www1.folha.uol.com.br/colunas/painel/2026/08/associacao-de-tribunais-de-contas-se-opoe-a-ferias-escolares-obrigatorias-na-copa-do-mundo-feminina.shtml</t>
+          <t>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/05/cbf-comunica-aos-clubes-parada-obrigatoria-durante-periodo-da-copa-do-mundo-feminina-de-2027.ghtml</t>
         </is>
       </c>
       <c r="G90" s="23" t="inlineStr">
@@ -34108,12 +34108,12 @@
       </c>
       <c r="H90" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I90" s="23" t="inlineStr">
         <is>
-          <t>A Atricon enviou ofícios à Câmara e ao Senado apoiando projeto que revoga a obrigatoriedade de férias escolares durante a Copa Feminina 2027, argumentando que a regra pode prejudicar calendários pedagógicos, transporte e alimentação escolar em regiões sem jogos.</t>
+          <t>A CBF comunicou aos clubes que as competições masculinas e femininas terão pausa obrigatória entre 24/06 e 25/07/2027, durante toda a Copa do Mundo Feminina, enquanto a entidade ajusta o calendário nacional e a disponibilidade das oito arenas do torneio.</t>
         </is>
       </c>
     </row>
@@ -34123,42 +34123,42 @@
       </c>
       <c r="B91" s="23" t="inlineStr">
         <is>
-          <t>CBF determina pausa nacional durante toda a Copa Feminina 2027</t>
+          <t>Elas Jogam Summit propõe ações para construir o legado da Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C91" s="23" t="inlineStr">
         <is>
-          <t>Calendário / competições nacionais</t>
+          <t>Elas Jogam Summit / legado</t>
         </is>
       </c>
       <c r="D91" s="23" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>São Paulo/SP</t>
         </is>
       </c>
       <c r="E91" s="23" t="inlineStr">
         <is>
-          <t>ge</t>
+          <t>Donas FC</t>
         </is>
       </c>
       <c r="F91" s="23" t="inlineStr">
         <is>
-          <t>https://ge.globo.com/futebol/futebol-internacional/noticia/2026/08/05/cbf-comunica-aos-clubes-parada-obrigatoria-durante-periodo-da-copa-do-mundo-feminina-de-2027.ghtml</t>
+          <t>https://donasfc.com.br/2026/08/05/elas-jogam-summit-discutira-o-legado-da-copa-do-mundo-feminina-2027-em-evento-no-pacaembu/</t>
         </is>
       </c>
       <c r="G91" s="23" t="inlineStr">
         <is>
-          <t>Neutro</t>
+          <t>Positivo</t>
         </is>
       </c>
       <c r="H91" s="23" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="I91" s="23" t="inlineStr">
         <is>
-          <t>A CBF comunicou aos clubes que as competições masculinas e femininas terão pausa obrigatória entre 24/06 e 25/07/2027, durante toda a Copa do Mundo Feminina, enquanto a entidade ajusta o calendário nacional e a disponibilidade das oito arenas do torneio.</t>
+          <t>A matéria apresentou o Elas Jogam Summit e sua proposta de transformar a Copa Feminina 2027 em legado por meio de políticas públicas, investimento, formação de base, espaços seguros para meninas, visibilidade e participação de profissionais do futebol feminino.</t>
         </is>
       </c>
     </row>
@@ -34168,12 +34168,12 @@
       </c>
       <c r="B92" s="23" t="inlineStr">
         <is>
-          <t>Elas Jogam Summit propõe ações para construir o legado da Copa Feminina 2027</t>
+          <t>Painel debate legado da Copa 2027 no Summit Mulheres nas Profissões</t>
         </is>
       </c>
       <c r="C92" s="23" t="inlineStr">
         <is>
-          <t>Elas Jogam Summit / legado</t>
+          <t>Legado / futebol feminino</t>
         </is>
       </c>
       <c r="D92" s="23" t="inlineStr">
@@ -34183,12 +34183,12 @@
       </c>
       <c r="E92" s="23" t="inlineStr">
         <is>
-          <t>Donas FC</t>
+          <t>O Liberal</t>
         </is>
       </c>
       <c r="F92" s="23" t="inlineStr">
         <is>
-          <t>https://donasfc.com.br/2026/08/05/elas-jogam-summit-discutira-o-legado-da-copa-do-mundo-feminina-2027-em-evento-no-pacaembu/</t>
+          <t>https://www.oliberal.com/esportes/nao-da-para-falar-em-paixao-nacional-so-valorizando-o-masculino-diz-secretaria-da-copa-1.1153852</t>
         </is>
       </c>
       <c r="G92" s="23" t="inlineStr">
@@ -34203,22 +34203,22 @@
       </c>
       <c r="I92" s="23" t="inlineStr">
         <is>
-          <t>A matéria apresentou o Elas Jogam Summit e sua proposta de transformar a Copa Feminina 2027 em legado por meio de políticas públicas, investimento, formação de base, espaços seguros para meninas, visibilidade e participação de profissionais do futebol feminino.</t>
+          <t>Painel reuniu representantes do esporte e Formiga para discutir legado, turismo e valorização do futebol feminino.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="33" t="n">
-        <v>46239</v>
+        <v>46238</v>
       </c>
       <c r="B93" s="23" t="inlineStr">
         <is>
-          <t>Painel debate legado da Copa 2027 no Summit Mulheres nas Profissões</t>
+          <t>Especialistas defendem descentralização do legado da Copa Feminina 2027</t>
         </is>
       </c>
       <c r="C93" s="23" t="inlineStr">
         <is>
-          <t>Legado / futebol feminino</t>
+          <t>Fórum Sustentabilidade em Campo / legado / EVT-0063</t>
         </is>
       </c>
       <c r="D93" s="23" t="inlineStr">
@@ -34228,17 +34228,17 @@
       </c>
       <c r="E93" s="23" t="inlineStr">
         <is>
-          <t>O Liberal</t>
+          <t>Máquina do Esporte</t>
         </is>
       </c>
       <c r="F93" s="23" t="inlineStr">
         <is>
-          <t>https://www.oliberal.com/esportes/nao-da-para-falar-em-paixao-nacional-so-valorizando-o-masculino-diz-secretaria-da-copa-1.1153852</t>
+          <t>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/desafio-para-copa-do-mundo-feminina-2027-e-descentralizar-legado-dizem-especialistas/</t>
         </is>
       </c>
       <c r="G93" s="23" t="inlineStr">
         <is>
-          <t>Positivo</t>
+          <t>Neutro</t>
         </is>
       </c>
       <c r="H93" s="23" t="inlineStr">
@@ -34248,37 +34248,37 @@
       </c>
       <c r="I93" s="23" t="inlineStr">
         <is>
-          <t>Painel reuniu representantes do esporte e Formiga para discutir legado, turismo e valorização do futebol feminino.</t>
+          <t>No Fórum Sustentabilidade em Campo (EVT-0063), especialistas defenderam que os investimentos e benefícios da Copa Feminina 2027 alcancem mercados periféricos e diferentes regiões do país. O debate também apontou gestão, base, patrocínio e governança como condições para um legado sustentável.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="33" t="n">
-        <v>46238</v>
+        <v>46199</v>
       </c>
       <c r="B94" s="23" t="inlineStr">
         <is>
-          <t>Especialistas defendem descentralização do legado da Copa Feminina 2027</t>
+          <t>CBF divulga calendário do segundo semestre das Seleções Femininas de Base</t>
         </is>
       </c>
       <c r="C94" s="23" t="inlineStr">
         <is>
-          <t>Fórum Sustentabilidade em Campo / legado / EVT-0063</t>
+          <t>Seleções de Base / calendário 2026</t>
         </is>
       </c>
       <c r="D94" s="23" t="inlineStr">
         <is>
-          <t>São Paulo/SP</t>
+          <t>Brasil e exterior</t>
         </is>
       </c>
       <c r="E94" s="23" t="inlineStr">
         <is>
-          <t>Máquina do Esporte</t>
+          <t>CBF</t>
         </is>
       </c>
       <c r="F94" s="23" t="inlineStr">
         <is>
-          <t>https://maquinadoesporte.com.br/copa-mundo-feminina-2027/desafio-para-copa-do-mundo-feminina-2027-e-descentralizar-legado-dizem-especialistas/</t>
+          <t>https://www.cbf.com.br/selecao-brasileira/noticias/noticias/selecao-base-feminina/confira-o-calendario-do-segundo-semestre-das-selecoes-femininas-de-base</t>
         </is>
       </c>
       <c r="G94" s="23" t="inlineStr">
@@ -34288,59 +34288,25 @@
       </c>
       <c r="H94" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="I94" s="23" t="inlineStr">
         <is>
-          <t>No Fórum Sustentabilidade em Campo (EVT-0063), especialistas defenderam que os investimentos e benefícios da Copa Feminina 2027 alcancem mercados periféricos e diferentes regiões do país. O debate também apontou gestão, base, patrocínio e governança como condições para um legado sustentável.</t>
+          <t>O calendário oficial reúne Liga Evolução Sub-15, Copas do Mundo Sub-17 e Sub-20, períodos de treinamento, Torneio Brasil e amistosos internacionais entre junho e dezembro de 2026.</t>
         </is>
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="33" t="n">
-        <v>46199</v>
-      </c>
-      <c r="B95" s="23" t="inlineStr">
-        <is>
-          <t>CBF divulga calendário do segundo semestre das Seleções Femininas de Base</t>
-        </is>
-      </c>
-      <c r="C95" s="23" t="inlineStr">
-        <is>
-          <t>Seleções de Base / calendário 2026</t>
-        </is>
-      </c>
-      <c r="D95" s="23" t="inlineStr">
-        <is>
-          <t>Brasil e exterior</t>
-        </is>
-      </c>
-      <c r="E95" s="23" t="inlineStr">
-        <is>
-          <t>CBF</t>
-        </is>
-      </c>
-      <c r="F95" s="23" t="inlineStr">
-        <is>
-          <t>https://www.cbf.com.br/selecao-brasileira/noticias/noticias/selecao-base-feminina/confira-o-calendario-do-segundo-semestre-das-selecoes-femininas-de-base</t>
-        </is>
-      </c>
-      <c r="G95" s="23" t="inlineStr">
-        <is>
-          <t>Neutro</t>
-        </is>
-      </c>
-      <c r="H95" s="23" t="inlineStr">
-        <is>
-          <t>Alto</t>
-        </is>
-      </c>
-      <c r="I95" s="23" t="inlineStr">
-        <is>
-          <t>O calendário oficial reúne Liga Evolução Sub-15, Copas do Mundo Sub-17 e Sub-20, períodos de treinamento, Torneio Brasil e amistosos internacionais entre junho e dezembro de 2026.</t>
-        </is>
-      </c>
+      <c r="A95" s="33" t="n"/>
+      <c r="B95" s="23" t="n"/>
+      <c r="C95" s="23" t="n"/>
+      <c r="D95" s="23" t="n"/>
+      <c r="E95" s="23" t="n"/>
+      <c r="F95" s="23" t="n"/>
+      <c r="G95" s="23" t="n"/>
+      <c r="H95" s="23" t="n"/>
+      <c r="I95" s="23" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="6" t="n"/>

</xml_diff>